<commit_message>
feat(dev): add a bot player from the ElinTogether menu
Lobby tab, Debug builds: starts a second game on this machine that joins
the local session by itself and plays at random (walk, travel, pick, drop,
eat, chat, attack, equip; quests and shipping as an option), and a button
to stop the games started that way.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2589,6 +2589,108 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>emp_ui_bot_add</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Add a bot player</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Add a bot player</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>emp_ui_bot_stop</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Stop the bots ({0})</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Stop the bots ({0})</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>emp_ui_bot_all_actions</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Bots also take quests and sell</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Bots also take quests and sell</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>emp_ui_bot_need_local</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Bots need a local server: disconnect, then add a bot to start one</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Bots need a local server: disconnect, then add a bot to start one</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>emp_ui_bot_no_launcher</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>No second copy of the game found (see _tools/make_lab.py)</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>No second copy of the game found (see _tools/make_lab.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>emp_ui_bot_started</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Bot player starting, it joins in about a minute</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Bot player starting, it joins in about a minute</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: random quests, fame and karma per player (untested in game)
Option on the host, on by default. A random quest belongs to the player
who takes it: only that player holds it, turns it in and gets the reward,
fame and karma; 5 quests each. Story quests stay shared. The host keeps
every player's quests and standing in the save and hands them back when
the player settles on its map; a client puts them back after every load
of the world (joining, travelling alone, coming back). While the host
runs a quest step for a player on its map, that player stands in as the
local one. Off: one quest log and one fame for the group, as before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D132"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2691,6 +2691,23 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_personal_quests</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Random quests and fame per player</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Random quests and fame per player</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(dev): the menu bot digs, cuts, builds and uses chests (untested in game)
With the 'bots do everything' box: the host hands a kit (tools, things to
place, food) to the player joining after a bot is started.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -2631,12 +2631,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Bots also take quests and sell</t>
+          <t>Bots do everything (quests, selling, digging, chests)</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Bots also take quests and sell</t>
+          <t>Bots do everything (quests, selling, digging, chests)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: a joining player chooses its character (untested in game)
Host option, on by default. A player who already has characters in the
world gets a list (name, race, job, level) plus 'a new character'; the
host keeps every character a player made. Off: the character played last,
as before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D133"/>
+  <dimension ref="A1:D136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2708,6 +2708,57 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_choose_chara</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Players choose their character when joining</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Players choose their character when joining</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_pick</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Who do you want to play?</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Who do you want to play?</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_new</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>A new character</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>A new character</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: trade window between players
Host option, on by default. The interaction menu on another player's
character offers a trade instead of opening its bag: invitation, a window
where each side puts items and gold, both confirm, and the game simulating
the map checks everything again and moves the real items at once. Changing
an offer clears the confirmations; walking away, closing the window or
leaving cancels. Nothing is set aside or created, so nothing can be
duplicated.
trade_suite 19/19.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D136"/>
+  <dimension ref="A1:D160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2759,6 +2759,414 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_player_trade</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Trade window between players</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Trade window between players</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>emp_act_trade</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Trade</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>emp_ui_trade</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Trade</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>emp_trade_invite</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>{0} wants to trade with you</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>{0} wants to trade with you</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>emp_trade_you_offer</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>You offer</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>You offer</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>emp_trade_they_offer</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>{0} offers</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>{0} offers</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>emp_trade_nothing</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>(nothing yet)</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>(nothing yet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>emp_trade_add</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Add an item</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Add an item</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>emp_trade_gold</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Gold: {0}</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Gold: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>emp_trade_clear</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Take everything back</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Take everything back</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>emp_trade_confirm</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>emp_trade_cancel</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Cancel</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Cancel</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>emp_trade_you_ready</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>You confirmed</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>You confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>emp_trade_you_wait</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>You have not confirmed</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>You have not confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>emp_trade_they_ready</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>the other player confirmed</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>the other player confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>emp_trade_they_wait</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>the other player has not confirmed</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>the other player has not confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>emp_trade_pick</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Which item?</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Which item?</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>emp_trade_howmany</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>How many?</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>How many?</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>emp_trade_howmuch</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>How much gold?</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>How much gold?</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>emp_trade_done</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Trade done</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Trade done</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>emp_trade_cancelled</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Trade cancelled</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Trade cancelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>emp_trade_invalid</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Trade cancelled: something offered is not there anymore</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Trade cancelled: something offered is not there anymore</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>emp_trade_far</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Trade cancelled: too far from each other</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Trade cancelled: too far from each other</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>emp_trade_busy</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>That player is already trading</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>That player is already trading</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Server settings screen in sections, one line of explanation per option
Players and travel / To each player its own / Time and combat / Joining
checks, each option with what it does under it. The random quest option
says it also covers karma. Texts in English, Japanese and Chinese.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D160"/>
+  <dimension ref="A1:D174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Random quests and fame per player</t>
+          <t>ランダムクエスト・名声・カルマはプレイヤーごと</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Random quests and fame per player</t>
+          <t>Random quests, fame and karma per player</t>
         </is>
       </c>
     </row>
@@ -3164,6 +3164,244 @@
       <c r="D160" t="inlineStr">
         <is>
           <t>That player is already trading</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_note_live</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>ホストのルールです。変更はすぐに全員に適用されます。</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>These rules are the host's. A change applies at once, for everyone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_sec_players</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>プレイヤーと移動</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Players and travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_sec_own</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>プレイヤーごとのもの</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>To each player its own</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_sec_time</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>時間と戦闘</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Time and combat</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_sec_checks</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>参加時の検証（上級者向け）</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Joining checks (advanced)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_choose_chara</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>参加時に、この世界の自分のキャラクターから選ぶか、新しく作る。</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>A joining player picks one of its characters in this world, or makes a new one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_independent_travel</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>誰でも好きな場所へ、一人でも一緒でも行ける。オフ：全員がホストについて行く。</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Everyone goes where they want, alone or together. Off: everyone follows the host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_personal_quests</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>各自ランダムクエスト5件、報酬・名声・カルマも各自。メインクエストは共有。</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>5 random quests each, with their reward, fame and karma. Story quests stay shared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_player_shipping</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>出荷箱の売上はアイテムを入れたプレイヤーへ。オフ：すべてホストへ。</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Shipping box money goes to the player who put the item in. Off: all to the host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_player_trade</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>他のプレイヤーをクリックしてアイテムと金貨を交換。双方が確認する。</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Click another player to trade items and gold. Both confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_combat_time</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>モンスターは戦っている相手が動いた時に動く。誰も待たない。ターン制より優先。</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>A monster acts when the player it fights acts: nobody waits. Takes over turn-based.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_turn_combat</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>戦闘中、プレイヤーは順番に行動する。</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>In a fight, players act in turn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_shared_speed</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>全プレイヤーが平均速度を共有。オフ：各自の速度。</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>One speed for all players, the average. Off: each keeps its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_validation</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>参加するプレイヤーのゲームがホストと一致すべきもの。「なし」：誰でも。「すべて」：データとMODが同じ。</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>What a joining player's game must share with yours. None: anyone. All: same data and mods.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: the Turn-Based Combat option says it has no effect while Combat on each player's time is on
Test: the text read in game through the bridge.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9510" yWindow="2685" windowWidth="31695" windowHeight="18195" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="General" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -3362,12 +3362,12 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>戦闘中、プレイヤーは順番に行動する。</t>
+          <t>戦闘中、プレイヤーは順番に行動する。「戦闘は各プレイヤーの時間で進行」がオンの間は無効。</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>In a fight, players act in turn.</t>
+          <t>In a fight, players act in turn. No effect while "Combat on each player's time" is on.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP, never run: each player on its own clock
On a client, Core.gameDelta is replaced by the host's game time as the
network brings it, so every step of a guest waits for it while the sprite
glides on the local clock: uneven steps. With the new host option
PlayerClock (only with PlayerCombatTime) a client keeps its local clock,
and the host no longer goes turbo for a guest's walk.

Compiles. NOT tested in game: move_suite.py (V1-V3) is written for it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9510" yWindow="2685" windowWidth="31695" windowHeight="18195" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="General" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D174"/>
+  <dimension ref="A1:D176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3405,6 +3405,40 @@
         </is>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_player_clock</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>各プレイヤーは自分の時計で動く</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Each player on its own clock</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_player_clock</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>ゲストもホストと同じように滑らかに動く（通信の速さに左右されない）。上のオプションが必要。</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>A guest walks and acts as smoothly as the host, not at the pace of the network. Needs the option above.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: every player steps at the pace of a solo game, whatever the others' speed (host option PlayerStepPace)
move_suite V4 and V5; the suite now sets the options it depends on.
Red on the build without it: with a host three times faster, the guest stepped every 209 ms instead of 120,
the host every 34 ms.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9510" yWindow="2685" windowWidth="31695" windowHeight="18195" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="General" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D176"/>
+  <dimension ref="A1:D178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3439,6 +3439,40 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_step_pace</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>各プレイヤーはソロと同じ歩調で動く</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Every player walks at the pace of a solo game</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_step_pace</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>歩く速さが他のプレイヤーの速度に左右されなくなります。戦闘では速度は今まで通り有効。「戦闘は各プレイヤーの時間で」が必要。</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>The length of a step no longer depends on the other players' speed. Speed still counts in a fight. Needs combat on each player's time.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: join with the character of one of your own solo saves (host option ImportCharacter, off by default)
Third choice on the connection screen, then the list of the last saves written. The save is read beside the
running game, never loaded, never written. The character comes with its stats, looks, equipment, bag and
gold, its fame and karma; not its companions, base, quests or bank. One copy of a save's character per player.
import_suite 21/21 through the real connection menu (red before: the option did not exist): same sheet as the
save at the guest and at the host, no duplicate uid although every uid of the save is taken at the host, the
save byte for byte unchanged, second import refused, option off hides the choice.
Not tested: a big late-game save, a save made with other mods, a character carrying a filled monster ball.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D178"/>
+  <dimension ref="A1:D186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3473,6 +3473,142 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_import_chara</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>自分のセーブのキャラクターで参加できる</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Players can bring a character from their own saves</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_import_chara</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>キャラクター本人、装備、持ち物、所持金、名声、カルマ。仲間、拠点、クエスト、銀行は含まれません。セーブは読むだけで変更しません。</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>The character, its equipment, bag and gold, its fame and karma. Not its companions, base, quests or bank. The save is only read, never changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_import</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>自分のセーブのキャラクター…</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>A character from one of my saves…</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_import_pick</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>どのセーブのキャラクターで参加しますか？（セーブは変更されません）</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Which save to bring the character of? (the save is not changed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_import_back</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>戻る</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Back</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_import_none</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>読み込めるセーブがありません。</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>No save this game can read was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_import_fail</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>このキャラクターは読み込めませんでした。</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>That character could not be brought.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_import_twice</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>このセーブのキャラクターはすでにこの世界にいます。</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>The character of that save is already in this world.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: one date for the whole world (host option SharedWorldTime), first step towards a session without a host
Only the host made the date advance; a player alone on a map it simulates had a date of its own, replaced by
the host's when it came back (minus 300 minutes after five hours away). Now the most advanced date is the
world's: a map holder reports the date its game reached (WorldTimeReportDelta), the host catches up with
everything a passing hour or day does and tells everyone; a map holder catches up the same way when the
world went further without it. Rule UseSharedWorldTime, key 10.
time_suite W1-W5: red 7/12 with the option off, green 12/12.
Not tested: two holders at once, a holder with visitors, three players.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D186"/>
+  <dimension ref="A1:D188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3609,6 +3608,40 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_world_time</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>世界の時間は全員で一つ</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>One date for the whole world</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_world_time</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>一人で別のマップにいるプレイヤーの時間も世界の時間になります。一番進んだ日付が世界の日付。オフ：ホストの日付だけ。</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Time passed by a player alone on another map counts for everyone: the most advanced date is the world's. Off: only the host's date counts.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: a save depot, the server that is only the save (client setting DepotPath)
A folder every player of the group can reach keeps the world. Whoever comes first takes it and hosts it with
the mod as it is, the others join, every save goes back to the folder (written beside, then swapped), and
when the host leaves the next player can take over. host.txt says who hosts, refreshed every minute.
Buttons on the Lobby tab (take the world / put this save), folder set on the Client Settings tab.
depot_suite D1-D6: 11/11 (the local copy is deleted before the second player takes the world: it comes from
the depot). ponytail: the lock is a file date, two players taking the world in the same minute both get it.
Not done: handing the world over while others are still playing (they go back to the title today).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D190"/>
+  <dimension ref="A1:D198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3676,6 +3676,142 @@
         </is>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_take</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>デポから世界を取り出してホストする</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Take the world from the depot and host it</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_put</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>このセーブをデポに置く</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Put this save in the depot</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_held</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>{0} がデポの世界をホスト中</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>{0} is hosting the world of the depot</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_empty</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>デポに世界がありません。ホストがセーブを読み込んで「このセーブをデポに置く」を押してください。</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>The depot holds no world yet. Load a save and use "Put this save in the depot".</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_fail</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>デポのフォルダを読み書きできませんでした。</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>The depot folder could not be read or written.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_put_done</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>この世界はデポに置かれました。誰でも取り出してホストできます。</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>This world is now in the depot: any player of the group can take it and host it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_folder</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>デポのフォルダ: {0}</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Depot folder: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_folder_ask</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>セーブデポのフォルダ（グループ全員が使える共有フォルダ。空欄でオフ）</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Folder of the save depot (a folder the whole group can reach; empty for none)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: a server like a Minecraft server: a game nobody plays, started with -empserver <save>, joined by address
It loads the save and opens the session by itself, saves every five minutes while someone plays, and the
players join it whenever they want through "Join by address" on the Lobby tab (host:55556). Everything
else was there: direct connection, players simulating their own maps, one date for the world (a server
nobody plays follows the players' time).
server_suite V1-V5: 7/7 (the server starts alone; a player joins by address, spends time on the server's map
and alone on another, leaves and finds its character again). Server and player ran on the same Steam account.
Not tested: across two PCs and the Internet (port 55556 to open, or a private network), a second player.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D198"/>
+  <dimension ref="A1:D200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3812,6 +3812,40 @@
         </is>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>emp_ui_join_address</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>アドレスで参加</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Join by address</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>emp_ui_join_address_ask</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>サーバーのアドレス（ホスト:ポート、ポートは 55556）</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Address of the server (host:port, the port is 55556)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Elin Together Server, the server application (one 23 KB exe, nothing to install)
Without Elin (the owner's idea, a server that is only the save): it keeps the world as one archive and holds
a real lock; the first player takes the world and hosts it, the others join, every save comes back, three
earlier worlds are kept. The game talks to it by address (DepotPath = host:55557, optional password);
what it sends is unpacked inside the save folder only.
With Elin on that PC: it starts the game as a server without window nor display (-batchmode -nographics
-empserver), shows its state, players, world date and last save (ElinMP/server.txt), and stops it after a
save (ElinMP/server.stop).
depot_suite with DEPOT_SERVER=1: 11/11 through the application. server_suite with the windowless server: 7/7.
Compiled by the C# compiler shipped with Windows (dev/server/build.ps1).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D200"/>
+  <dimension ref="A1:D202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3786,12 +3787,12 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>デポのフォルダ: {0}</t>
+          <t>デポ（フォルダまたはサーバーのアドレス）: {0}</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Depot folder: {0}</t>
+          <t>Depot (folder or server address): {0}</t>
         </is>
       </c>
     </row>
@@ -3803,12 +3804,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>セーブデポのフォルダ（グループ全員が使える共有フォルダ。空欄でオフ）</t>
+          <t>セーブデポ：Elin Together Server のアドレス（ホスト:55557）または共有フォルダ。空欄でオフ</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Folder of the save depot (a folder the whole group can reach; empty for none)</t>
+          <t>Save depot: the address of Elin Together Server (host:55557), or a folder the whole group can reach. Empty for none</t>
         </is>
       </c>
     </row>
@@ -3843,6 +3844,40 @@
       <c r="D200" t="inlineStr">
         <is>
           <t>Address of the server (host:port, the port is 55556)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_password</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>デポのパスワード: {0}</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Depot password: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_password_ask</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>デポのパスワード（サーバーで設定した場合）</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Password of the depot (when one was set in Elin Together Server)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: "Join by address" works with both kinds of server; the timeout message has a text
The user's first try between two PCs: Elin Together Server ran without Elin (TCP 55557) and
"Join by address" only spoke to a game server (UDP 55556), so it ended on a raw "emp_ui_timeout".

- "Join by address" first asks the address whether it is Elin Together Server; if so it becomes
  the depot and its world is taken and hosted (or the player is told who hosts it). Otherwise it
  joins as before.
- emp_ui_timeout had no text in any language; the address prompt names both ports.
- depot_suite with DEPOT_SERVER=1: the second player sets no depot and goes through JoinAddress,
  on port 55558 (a real server of the user may run on 55557). Red 3/4 before, green 11/11 after.

Not tested: the timeout text itself (Release builds only show it).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D202"/>
+  <dimension ref="A1:D203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3838,12 +3838,12 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>サーバーのアドレス（ホスト:ポート、ポートは 55556）</t>
+          <t>サーバーのアドレス（ホスト:ポート。Elin ありは 55556、Elin なしは 55557）</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Address of the server (host:port, the port is 55556)</t>
+          <t>Address of the server (host:port; the port is 55556 with Elin, 55557 without)</t>
         </is>
       </c>
     </row>
@@ -3878,6 +3878,23 @@
       <c r="D202" t="inlineStr">
         <is>
           <t>Password of the depot (when one was set in Elin Together Server)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>emp_ui_timeout</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>サーバーが応答しません。アドレス、ポート、サーバーのモードを確認してください。</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>The server does not answer. Check the address, the port and the mode of the server.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: a wrong server password is said as such, not "password is hosting the world"
The server answers "NO password"; the game read the reason as the name of the player who hosts.
HeldBy only trusts an accepted answer; taking or putting the world shows "The server refused the
password. Set it in Client Settings" (new text, three languages). emp_ui_depot_fail no longer
speaks of a folder only.

depot_suite with DEPOT_SERVER=1: red 11/13 ("password is hosting the world of the depot"),
green 13/13.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D203"/>
+  <dimension ref="A1:D204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3753,12 +3753,12 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>デポのフォルダを読み書きできませんでした。</t>
+          <t>デポに接続できない、または読み書きできませんでした。</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>The depot folder could not be read or written.</t>
+          <t>The depot could not be reached, read or written.</t>
         </is>
       </c>
     </row>
@@ -3895,6 +3895,23 @@
       <c r="D203" t="inlineStr">
         <is>
           <t>The server does not answer. Check the address, the port and the mode of the server.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_password_wrong</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>サーバーがパスワードを拒否しました。「Client Settings」の「デポのパスワード」で設定してください。</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>The server refused the password. Set it in Client Settings, "Depot password".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
wip: dungeon quests for two, when the host took the quest (yes/no box, visitor guards)
Written by an agent, builds, never run in game (together_suite T1-T5), not reviewed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D207"/>
+  <dimension ref="A1:D210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3966,6 +3966,57 @@
         </is>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>emp_quest_follow_ask</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>{0}がクエストに出発します。同行しますか？報酬は{0}のものです。</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>{0} is leaving on a quest. Go along? The reward goes to {0}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>emp_quest_follow_declined</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>{0}は同行を断りました。</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>{0} declined to come along.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>emp_quest_follow_no_answer</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>{0}から返事がありません。</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>{0} did not answer.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: dungeon quests for two when the host took the quest: yes/no box, visitor guards, town recalled on the way out, harvest search (together_suite T1-T6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D207"/>
+  <dimension ref="A1:D210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3966,6 +3966,57 @@
         </is>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>emp_quest_follow_ask</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>{0}がクエストに出発します。同行しますか？報酬は{0}のものです。</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>{0} is leaving on a quest. Go along? The reward goes to {0}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>emp_quest_follow_declined</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>{0}は同行を断りました。</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>{0} declined to come along.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>emp_quest_follow_no_answer</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>{0}から返事がありません。</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>{0} did not answer.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
wip: dungeon quests for two when the guest took the quest (E5, E6) - written by an agent, not compiled alone, freezes the host's load, not validated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D210"/>
+  <dimension ref="A1:D211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4017,6 +4017,23 @@
         </is>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>emp_quest_follow_asked</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>{0}に同行するか尋ねています…</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Asking {0} to come along...</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: dungeon quests for two when the guest took the quest: yes/no box on the host, zone simulated by the host, reward to the taker, the host may go home alone (together_suite T7-T11, 107/107 with T1-T6)
Subdue quests only for now: harvest, music and defense stay the guest's alone (deliveries are counted by the taker's game).
Nothing of a guest's quest is written to the host's save (T11).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D210"/>
+  <dimension ref="A1:D211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4017,6 +4017,23 @@
         </is>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>emp_quest_follow_asked</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>{0}に同行するか尋ねています…</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Asking {0} to come along...</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: a guest no longer pays for nothing at the base: research and hearth skills are refused with a message until they become requests to the host (council 4, step 1; base_suite 53/53). Also the texts of this batch
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D211"/>
+  <dimension ref="A1:D220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4034,6 +4034,159 @@
         </is>
       </c>
     </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>emp_base_host_only</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>今のところ、これはホストだけができます。</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Only the host can do this for now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>emp_trade_equipped</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>取引中止：提示したアイテムが装備されています</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Trade cancelled: an offered item is now equipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>emp_trade_nodrop</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>取引中止：提示したアイテムは手放せません</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Trade cancelled: an offered item cannot be dropped or given away</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>emp_trade_npcprop</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>取引中止：提示したアイテムはNPCの所有物です</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Trade cancelled: an offered item belongs to an NPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>emp_trade_gifted</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>取引中止：提示したアイテムは贈り物のため取引できません</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Trade cancelled: an offered item is a gift and cannot be traded</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>emp_trade_bound</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>取引中止：提示したアイテムはキャラクターに結び付いています</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Trade cancelled: an offered item is bound to a character</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>emp_trade_full</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>取引中止：受け取るアイテムに対してバッグの空きが足りません</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Trade cancelled: a bag does not have enough free slots for what it would receive</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>emp_travel_recalled_by</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>{@Peer} がこの場所に来ます。画面が再読み込みされ、合流します…</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>{@Peer} is coming to this place: the screen will reload to rejoin them…</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>emp_ui_thing_gone</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>遅かったようです。他のプレイヤーが先に取りました</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Too late: someone else already took it</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: a guest's research and hearth skills are requests to the host: the host checks, pays once and everyone sees the result; the host's own research reaches the guests too (council 4, step 2; base_suite B1 20/20, B4 green)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D220"/>
+  <dimension ref="A1:D222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4187,6 +4187,40 @@
         </is>
       </c>
     </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>emp_base_refused</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>ホストに断られました。拠点または所持金では、もう支払えません。</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>The host refused: the base or your purse can no longer pay for this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>emp_base_pending</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>前回の依頼はまだホストの返事を待っています。</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Your last request is still waiting for the host's answer.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: another version of Elin is no longer a wall: only the mod's version must match; players are told, and a host checkbox asks for the same game version again (version_suite 8/8, local connection; the Steam lobby path uses the same check, not played)
Asked by the user after Elin went from EA 23.351 to 23.352 during the session.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D222"/>
+  <dimension ref="A1:D225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4221,6 +4221,57 @@
         </is>
       </c>
     </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>emp_game_version_differs</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>{0} のElinのバージョンが異なります（{1} ／ こちら {2}）。接続は許可されます。問題が起きたら同じバージョンに揃えてください。</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>{0} runs another version of Elin ({1}, here {2}). The connection is allowed; if something goes wrong, use the same version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_same_game_version</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>同じElinバージョンを必須にする</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Require the same Elin version</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_same_game_version</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>オン：Elinのバージョンが違うプレイヤーを拒否。オフ：警告のうえ参加を許可。Modのバージョンは常に同じである必要があります。</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>On: players on another version of Elin are refused. Off: they are let in with a warning. The same version of the mod is always required.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: a guest uses the build mode of the base like the host: floors, walls and new furniture from the menu, mining, digging, cutting. Its game sends the task it would have had its agent do; the game that keeps the map does it with the sender as the player (gold once, materials once from its bag then the stock, what is mined in its bag); host checkbox GuestBuild, on by default. Areas, terrain tool, blueprints and the roof mode are still refused before anything is paid (council 5 steps 4 to 6; build2_suite 28/28, red seen first; build_suite 19/19). Not played: stock items, bridges, dragging, digging, ramps, the checkbox off
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D225"/>
+  <dimension ref="A1:D227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -4272,6 +4271,40 @@
         </is>
       </c>
     </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_guest_build</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>他のプレイヤーも建築モードを使える</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Other players can use build mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_guest_build</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>オン：他のプレイヤーも拠点の建築モード（床・壁・家具・採掘・伐採）を使えます。ホストのゲームが代わりに建て、費用と素材は本人が払います。オフ：ホストだけが建てられます。</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>On: the other players can use the build mode of the base (floors, walls, furniture, mining, cutting). The game of the host builds for them; they pay the gold and the materials. Off: only the host builds.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: a player can no longer kill another player: a blow of a player or of what fights for one that would kill another player's character leaves it at 0 hit points, in every game (one shift+click killed for real: grave, gold, death screen); host checkbox PlayerKill to allow it; first step of council 7 (duel_suite P1, 10/10, both ways, red seen first). The blow came by two roads: the host's own, and the damage the victim's game reports after replaying the attack. Not covered: bleeding, poison, fire, the death sentence; spells and missiles not played. (EmpConfig and the text files of this commit also hold the texts of the GitHub depot, next commit)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D227"/>
+  <dimension ref="A1:D236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3786,12 +3786,12 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>デポ（フォルダまたはサーバーのアドレス）: {0}</t>
+          <t>デポ（フォルダ、サーバーのアドレス、または GitHub）: {0}</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Depot (folder or server address): {0}</t>
+          <t>Depot (folder, server address or GitHub): {0}</t>
         </is>
       </c>
     </row>
@@ -3803,12 +3803,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>セーブデポ：Elin Together Server のアドレス（ホスト:55557）または共有フォルダ。空欄でオフ</t>
+          <t>セーブデポ：Elin Together Server のアドレス（ホスト:55557）、共有フォルダ、または非公開の GitHub リポジトリ（github:所有者/リポジトリ）。空欄でオフ</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Save depot: the address of Elin Together Server (host:55557), or a folder the whole group can reach. Empty for none</t>
+          <t>Save depot: the address of Elin Together Server (host:55557), a folder the whole group can reach, or a private GitHub repository (github:owner/repository). Empty for none</t>
         </is>
       </c>
     </row>
@@ -3854,12 +3854,12 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>デポのパスワード: {0}</t>
+          <t>デポのパスワード／GitHub のキー: {0}</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Depot password: {0}</t>
+          <t>Depot password or GitHub key: {0}</t>
         </is>
       </c>
     </row>
@@ -3871,12 +3871,12 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>デポのパスワード（サーバーで設定した場合）</t>
+          <t>デポのパスワード（サーバーで設定した場合）、または GitHub のアクセスキー。キーは二度と表示されません。空欄のままなら現在のキーを保持します</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Password of the depot (when one was set in Elin Together Server)</t>
+          <t>Password of the depot (when one was set in Elin Together Server), or the GitHub access key. A key is never shown again: leave empty to keep it</t>
         </is>
       </c>
     </row>
@@ -4302,6 +4302,167 @@
       <c r="D227" t="inlineStr">
         <is>
           <t>On: the other players can use the build mode of the base (floors, walls, furniture, mining, cutting). The game of the host builds for them; they pay the gold and the materials. Off: only the host builds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_help</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>非公開の GitHub リポジトリをデポにできます（サーバーも共有フォルダも不要、フレンドは GitHub アカウント不要）：
+1. github.com で、この世界専用の空の非公開（Private）リポジトリを作成します。
+2. そのリポジトリ用のアクセスキーを1つ作成します：Settings → Developer settings → Fine-grained tokens、このリポジトリのみ、Contents: Read and write。
+3. キーを「デポのパスワード／GitHub のキー」に貼り付け、「デポ」に github:所有者/リポジトリ と入力します。
+4. 同じ2行をフレンドに送り、フレンドもここに入力します。このキーで開けるのはこのリポジトリだけです。</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>A private GitHub repository can be the depot (no server, no shared folder, your friends need no GitHub account):
+1. On github.com, create an empty private repository, only for this world.
+2. Create one access key for it: Settings, Developer settings, Fine-grained tokens; only this repository; Contents: Read and write.
+3. Paste the key in "Depot password or GitHub key" and write github:owner/repository in "Depot".
+4. Send the same two lines to your friends: they type them here too. The key only opens this one repository.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_key</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>GitHub がアクセスキーを拒否しました。キーの有効期限、このリポジトリが対象になっているか、「Contents: Read and write」の権限があるかを確認し、「Client Settings」で貼り付け直してください。</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>GitHub refused the access key. Check that it has not expired, that it covers this repository with "Contents: Read and write", then paste it again in Client Settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_missing</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>GitHub でデポのリポジトリが見つかりません。「Client Settings」の名前（github:所有者/リポジトリ）と、アクセスキーがそのリポジトリを対象にしているかを確認してください。</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>GitHub does not find the repository of the depot. Check its name (github:owner/repository) in Client Settings, and that your access key covers it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_public</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>この GitHub リポジトリは公開されています。世界とその履歴がすべて誰にでも見えてしまいます。非公開にしてから（Settings → Danger Zone → Change visibility）、もう一度お試しください。</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>This GitHub repository is public: your world and all its history would be visible to everyone. Make it private (Settings, Danger Zone, Change visibility), then try again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_big</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>この世界は 20 MB を超えており、GitHub のデポには大きすぎます。Elin Together Server か共有フォルダを使ってください。セーブはこのPCに保存されています。</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>This world is over 20 MB: too big for a GitHub depot. Use Elin Together Server or a shared folder instead. The save is kept on this PC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_changed</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>接続が切れている間に、他のプレイヤーがデポの世界をホストしてセーブしました。あなたのセーブはこのPCに残り、デポには届きません。タイトルに戻って、もう一度世界を取り出してください。</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>The world in the depot changed while this game was cut off: someone else hosted it and saved. Your saves stay on this PC and no longer reach the depot. Go back to the title screen and take the world again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_down</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>GitHub から応答がありません。接続を確認して、しばらくしてからもう一度お試しください。</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>GitHub does not answer. Check your connection and try again in a moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_player_kill</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>プレイヤー同士で殺せる</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Players can kill each other</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_player_kill</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>オン：プレイヤー（とその仲間）の攻撃で他のプレイヤーのキャラクターが死にます。オフ：致命的な一撃でも相手のHPは0で止まり、死にません。</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>On: a strike of a player (or of its companions) can kill another player's character. Off: a strike that would kill it leaves it at 0 hit points, alive.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: a guest manages the residents of the host's base: maid, resident or livestock, reserve, recall, sending away (requests to the host, who does it once and tells everyone); leaving the base and deeds refused to a guest; host checkbox HostManagesBase (session rule 14, off). Council 7.
Fixed on the way: the residents window of a guest listed every tab into the one shared list when the host's answer came, the row went hidden and the next click was the game's own (maid removed in the guest's game only). The test helper send_raw read a field as a property and sent nothing: the three "the host refuses anyway" checks were false greens, a control now proves the send.

base_suite: 176/177 red seen first (maid removed by the guest), then B1 to B11 green with the control; B12 green on the run before (the last run stopped in B12 on the bench's out of memory, the PC was full).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D236"/>
+  <dimension ref="A1:D238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4466,6 +4466,40 @@
         </is>
       </c>
     </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_host_manages_base</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>拠点の管理はホストだけ</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Only the host manages the base</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_host_manages_base</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>オン：他のプレイヤーによる拠点の操作（研究、炉の技能、政策、名前、物の設定、住民、建築モード）は拒否されます。オフ：全員がホストと同じように拠点を管理できます。拠点の放棄は常にホストだけです。</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>On: what the other players ask of the base (research, hearth skills, policies, names, settings of an object, residents, build mode) is refused. Off: every player manages the base as the host does. Leaving the base for good always stays the host's.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: duels between players (council 7, steps 2 to 4): "Challenge to a duel" in the menu on another player's character, a yes/no box for the other, a countdown, the fight where they stand; the blow that would kill ends it, nobody dies, both are healed, nothing is lost; leaving or disconnecting ends it without a winner. Host checkbox Duels (session rule 15, on), deltas 837 and 838.
Review: the duellist left at 0 loses whoever struck (its opponent's companion too). Not done: arena, bet, a give-up button; a third player's blow on a duellist is stopped like the opponent's.

duel_suite: red seen first on the build without it (11/18), then 90/91, the red being the test (the guest was not next to the host's cat): D3 alone 13/13 after. Not played: two PCs, spells and arrows, three players.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D238"/>
+  <dimension ref="A1:D250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -4500,6 +4501,210 @@
         </is>
       </c>
     </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_duels</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>プレイヤー同士の決闘</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Duels between players</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_duels</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>オン：相手キャラクターのメニューから決闘を申し込めます。誰も死なず、終了時に両者が回復し、何も失いません。オフ：決闘なし。</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>On: a player can challenge another from the menu on its character. Nobody dies, both are healed, nothing is lost. Off: no duels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>emp_act_duel</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>決闘を申し込む</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Challenge to a duel</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>emp_duel_invite</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>{0} が決闘を申し込んできました。誰も死なず何も失いませんが、決闘中に使ったポーション・矢・チャージは戻りません。受けますか？</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>{0} challenges you to a duel. Nobody dies and nothing is lost, but potions, arrows and charges used during the duel stay spent. Accept?</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>emp_duel_asked</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>{0} に決闘を申し込みました…</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>You challenge {0} to a duel…</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>emp_duel_countdown</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>決闘：{0} 対 {1}。3秒後に開始！</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Duel: {0} against {1}. It starts in 3 seconds!</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>emp_duel_fight</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>始め！</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Fight!</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>emp_duel_won</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>{0} が {1} との決闘に勝ちました。</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>{0} won the duel against {1}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>emp_duel_declined</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>決闘は断られました。</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>The duel was declined.</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>emp_duel_noanswer</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>返事がなく、決闘は行われません。</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>No answer: no duel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>emp_duel_busy</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>そのプレイヤーは決闘中か取引中です。</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>That player is already in a duel or a trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>emp_duel_over</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>決闘は勝者なしで終わりました。</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>The duel is over, without a winner.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: ten frictions with one right answer, from the audit (dev/PLAN_sans_friction.md, A2 to A8, A13 to A15): short label for "X is hosting the world"; the depot and key buttons no longer overflow (fixed label, value on a line below); four text keys shown raw now have texts; the timeout message of a Steam guest no longer speaks of address and port; 27 Japanese lines left in English are translated; "Add an item" with nothing to offer says so; "Server can only be started after claiming a zone" is off the title screen; the version refusal says what to do; the host's name instead of the word "Host"; no box to validate after putting a save in the depot. With the text of the hand-over message.
Compiled; trade_suite 122/122, version_suite 8/8, leave_suite 13/13, depot_suite 22/22 after. The new texts and layouts themselves are not looked at in game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D250"/>
+  <dimension ref="A1:D257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -1771,336 +1770,330 @@
     <row r="80" ht="60" customHeight="1">
       <c r="A80" t="inlineStr">
         <is>
-          <t>emp_connection_rejected</t>
+          <t>emp_dc_host_kick</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>接続が拒否されました
-ビルドバージョンが一致しません
-ホストバージョン: {0}
-クライアントバージョン: {1}</t>
-        </is>
-      </c>
-      <c r="D80" s="1" t="inlineStr">
-        <is>
-          <t>Connection rejected
-Build version mismatch
-Host version: {0}
-Client version: {1}</t>
+          <t>切断: ホストによりキックされました</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Disconnected: Kicked by host</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>emp_dc_host_kick</t>
+          <t>emp_ui_tab_client</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>切断: ホストによりキックされました</t>
+          <t>クライアント設定</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Disconnected: Kicked by host</t>
+          <t>Client Settings</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>emp_ui_tab_client</t>
+          <t>emp_tab_client</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>クライアント設定</t>
+          <t>クライアント</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Client Settings</t>
+          <t>Client</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>emp_tab_client</t>
+          <t>emp_ui_kick</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>クライアント</t>
+          <t>キック</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Kick</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>emp_ui_kick</t>
+          <t>emp_ui_ping_keymap</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>キック</t>
+          <t>ピンキー設定: {0}</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>Bind Ping Key: {0}</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>emp_ui_ping_keymap</t>
+          <t>emp_ui_ping_action</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ピンキー設定: {0}</t>
+          <t>ピン</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Bind Ping Key: {0}</t>
+          <t>Ping</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>emp_ui_ping_action</t>
+          <t>emp_ui_unknown_player</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ピン</t>
+          <t>プレイヤー {0}</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Ping</t>
+          <t>Player {0}</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>emp_ui_unknown_player</t>
+          <t>emp_ui_source_mismatch_header</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>プレイヤー {0}</t>
+          <t>ソース検証失敗 — {0} 件の不一致</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Player {0}</t>
+          <t>Source validation failed — {0} mismatches</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>emp_ui_source_mismatch_header</t>
+          <t>emp_ui_source_mismatch_sources</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ソース検証失敗 — {0} 件の不一致</t>
+          <t>ソース不一致:</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Source validation failed — {0} mismatches</t>
+          <t>Source mismatches:</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>emp_ui_source_mismatch_sources</t>
+          <t>emp_ui_source_mismatch_plugins</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ソース不一致:</t>
+          <t>プラグイン不一致:</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Source mismatches:</t>
+          <t>Plugin mismatches:</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>emp_ui_source_mismatch_plugins</t>
+          <t>emp_ui_source_mismatch_files</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>プラグイン不一致:</t>
+          <t>ファイル不一致:</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Plugin mismatches:</t>
+          <t>File mismatches:</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>emp_ui_source_mismatch_files</t>
+          <t>emp_ui_source_mismatch_more</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ファイル不一致:</t>
+          <t>… 他 {0} 件</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>File mismatches:</t>
+          <t>… and {0} more</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>emp_ui_source_mismatch_more</t>
+          <t>emp_ui_source_mismatch_continue</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>… 他 {0} 件</t>
+          <t>それでも続行しますか？</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>… and {0} more</t>
+          <t>Continue anyway?</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>emp_ui_source_mismatch_continue</t>
+          <t>emp_ui_sv_cfg_validation_sets</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>それでも続行しますか？</t>
+          <t>検証セット</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Continue anyway?</t>
+          <t>Validation Sets</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_validation_sets</t>
+          <t>emp_validation_none</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>検証セット</t>
+          <t>なし</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Validation Sets</t>
+          <t>None</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>emp_validation_none</t>
+          <t>emp_validation_sources</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>なし</t>
+          <t>ソース</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Source</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>emp_validation_sources</t>
+          <t>emp_validation_plugins</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ソース</t>
+          <t>プラグイン</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Plugin</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>emp_validation_plugins</t>
+          <t>emp_validation_all</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>プラグイン</t>
+          <t>すべて</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Plugin</t>
+          <t>All</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>emp_validation_all</t>
+          <t>emp_ui_reconnect</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>すべて</t>
+          <t>再接続</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Reconnect</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>emp_ui_reconnect</t>
+          <t>emp_dc_reconnect_request</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2110,145 +2103,128 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Reconnect</t>
+          <t>Reconnect Request</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>emp_dc_reconnect_request</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>再接続</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Reconnect Request</t>
+          <t>emp_lobby_create_failed</t>
+        </is>
+      </c>
+      <c r="C100" s="1" t="inlineStr">
+        <is>
+          <t>Steamロビーの作成に失敗しました: {Result}
+後でもう一度試してください</t>
+        </is>
+      </c>
+      <c r="D100" s="1" t="inlineStr">
+        <is>
+          <t>Failed to create Steam lobby: {Result}
+Try again later</t>
         </is>
       </c>
     </row>
     <row r="101" ht="30" customHeight="1">
       <c r="A101" t="inlineStr">
         <is>
-          <t>emp_lobby_create_failed</t>
-        </is>
-      </c>
-      <c r="C101" s="1" t="inlineStr">
-        <is>
-          <t>Steamロビーの作成に失敗しました: {Result}
-後でもう一度試してください</t>
-        </is>
-      </c>
-      <c r="D101" s="1" t="inlineStr">
-        <is>
-          <t>Failed to create Steam lobby: {Result}
-Try again later</t>
+          <t>emp_lobby_enter_failed</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Steamロビーへの参加に失敗しました: {Response}</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Failed to enter Steam lobby: {Response}</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>emp_lobby_enter_failed</t>
+          <t>emp_lobby_already_joined</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Steamロビーへの参加に失敗しました: {Response}</t>
+          <t>すでに同じロビーに参加しています</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Failed to enter Steam lobby: {Response}</t>
+          <t>Already in the same lobby</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>emp_lobby_already_joined</t>
+          <t>emp_ui_quest_client</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>すでに同じロビーに参加しています</t>
+          <t>（暫定）このクエストはクライアントプレイヤーからは開始できません。</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Already in the same lobby</t>
+          <t>(Temp) This quest cannot be started by client players.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>emp_ui_quest_client</t>
+          <t>emp_dc_version_mismatch</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>（暫定）このクエストはクライアントプレイヤーからは開始できません。</t>
+          <t>切断: 無効なVersion</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>(Temp) This quest cannot be started by client players.</t>
+          <t>Disconnected: invalid version</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>emp_dc_version_mismatch</t>
+          <t>emp_dc_act_mismatch</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>切断: 無効なVersion</t>
+          <t>切断: Act 不一致</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Disconnected: invalid version</t>
+          <t>Act mapping mismatch</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>emp_dc_act_mismatch</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>切断: Act 不一致</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>Act mapping mismatch</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="60" customHeight="1">
-      <c r="A107" t="inlineStr">
-        <is>
           <t>emp_ui_reject_acts</t>
         </is>
       </c>
-      <c r="C107" s="1" t="inlineStr">
+      <c r="C106" s="1" t="inlineStr">
         <is>
           <t>参加できません：Actマッピングが一致しません（{0}件）
 Act ID同期エラー：不一致は動作不良の原因になります。
 双方とも同じModを導入しているか確認してください。</t>
         </is>
       </c>
-      <c r="D107" s="1" t="inlineStr">
+      <c r="D106" s="1" t="inlineStr">
         <is>
           <t>Could not join: Act mapping mismatch ({0})
 Act ID is used for action sync. Game cannot run with mismatch acts.
@@ -2256,30 +2232,30 @@
         </is>
       </c>
     </row>
+    <row r="107" ht="60" customHeight="1">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>emp_ui_reject_integrity</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>参加できません：ホストの厳密チェックにより、データ整合性が不一致です（{0}件）</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Could not join: Host has strict verification enabled. Data integrity mismatch ({0})</t>
+        </is>
+      </c>
+    </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>emp_ui_reject_integrity</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>参加できません：ホストの厳密チェックにより、データ整合性が不一致です（{0}件）</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Could not join: Host has strict verification enabled. Data integrity mismatch ({0})</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="60" customHeight="1">
-      <c r="A109" t="inlineStr">
-        <is>
           <t>emp_version_rejected_host</t>
         </is>
       </c>
-      <c r="C109" s="1" t="inlineStr">
+      <c r="C108" s="1" t="inlineStr">
         <is>
           <t>{0}の接続を拒否しました
 バージョンがホストと一致しません
@@ -2287,7 +2263,7 @@
 ホストゲーム：{2}</t>
         </is>
       </c>
-      <c r="D109" s="1" t="inlineStr">
+      <c r="D108" s="1" t="inlineStr">
         <is>
           <t>Connection request from {0} rejected
 Version mismatch with host
@@ -2296,495 +2272,514 @@
         </is>
       </c>
     </row>
+    <row r="109" ht="60" customHeight="1">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>emp_version_rejected_client</t>
+        </is>
+      </c>
+      <c r="C109" s="1" t="inlineStr">
+        <is>
+          <t>参加できません：バージョン不一致
+Mod：自機 {0} ／ ホスト {1}
+ゲーム：自機 {2} ／ ホスト {3}
+古いバージョンのほうを更新してから、もう一度お試しください。</t>
+        </is>
+      </c>
+      <c r="D109" s="1" t="inlineStr">
+        <is>
+          <t>Could not join: Version mismatch
+Mod: Local {0} / Host {1}
+Game: Local {2} / Host {3}
+Whoever has the older version must update, then try again.</t>
+        </is>
+      </c>
+    </row>
     <row r="110" ht="45" customHeight="1">
       <c r="A110" t="inlineStr">
         <is>
-          <t>emp_version_rejected_client</t>
-        </is>
-      </c>
-      <c r="C110" s="1" t="inlineStr">
-        <is>
-          <t>参加できません：バージョン不一致
-Mod：自機 {0} ／ ホスト {1}
-ゲーム：自機 {2} ／ ホスト {3}</t>
-        </is>
-      </c>
-      <c r="D110" s="1" t="inlineStr">
-        <is>
-          <t>Could not join: Version mismatch
-Mod: Local {0} / Host {1}
-Game: Local {2} / Host {3}</t>
+          <t>emp_ui_sleep_request</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>全員がベッドに入るのを待っています…</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Waiting for everyone to go to bed...</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>emp_ui_sleep_request</t>
+          <t>emp_ui_sleep_wish</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>全員がベッドに入るのを待っています…</t>
+          <t>{0}が眠りたがっています（{1}/{2}）</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Waiting for everyone to go to bed...</t>
+          <t>{0} wants to sleep ({1}/{2})</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>emp_ui_sleep_wish</t>
+          <t>emp_ui_sleep_cancel</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>{0}が眠りたがっています（{1}/{2}）</t>
+          <t>{0}が目を覚ましました（{1}/{2}）</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>{0} wants to sleep ({1}/{2})</t>
+          <t>{0} woke up ({1}/{2})</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>emp_ui_sleep_cancel</t>
+          <t>emp_travel_requesting</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>{0}が目を覚ましました（{1}/{2}）</t>
+          <t>ホストに移動を申請中…</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>{0} woke up ({1}/{2})</t>
+          <t>Asking the host to travel there alone…</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>emp_travel_requesting</t>
+          <t>emp_travel_returning</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ホストに移動を申請中…</t>
+          <t>ホストのいる場所へ戻っています…</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Asking the host to travel there alone…</t>
+          <t>Returning to the host…</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>emp_travel_returning</t>
+          <t>emp_travel_disabled</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ホストのいる場所へ戻っています…</t>
+          <t>ホストが単独行動を許可していません</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Returning to the host…</t>
+          <t>The host does not allow travelling alone</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>emp_travel_disabled</t>
+          <t>emp_travel_invalid</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ホストが単独行動を許可していません</t>
+          <t>この場所へは単独で行けません</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>The host does not allow travelling alone</t>
+          <t>You cannot travel there alone</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>emp_travel_invalid</t>
+          <t>emp_travel_host_zone</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>この場所へは単独で行けません</t>
+          <t>ホストはすでにそこにいます</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>You cannot travel there alone</t>
+          <t>The host is already there</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>emp_travel_host_zone</t>
+          <t>emp_travel_occupied</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ホストはすでにそこにいます</t>
+          <t>他のプレイヤーがその場所にいます</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>The host is already there</t>
+          <t>Another player is already there</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>emp_travel_occupied</t>
+          <t>emp_travel_recalling</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>他のプレイヤーがその場所にいます</t>
+          <t>{@Peer} がその場所を返すのを待っています…</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Another player is already there</t>
+          <t>Waiting for {@Peer} to hand the zone back…</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>emp_travel_recalling</t>
+          <t>emp_travel_recalled</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>{@Peer} がその場所を返すのを待っています…</t>
+          <t>ホストが来ます。合流します…</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Waiting for {@Peer} to hand the zone back…</t>
+          <t>The host is coming, rejoining them…</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>emp_travel_recalled</t>
+          <t>emp_travel_zone_closed</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ホストが来ます。合流します…</t>
+          <t>この場所の主がいなくなりました。ホストに合流します</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>The host is coming, rejoining them…</t>
+          <t>The owner of this place is gone, rejoining the host</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>emp_travel_zone_closed</t>
+          <t>emp_travel_handoff</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>この場所の主がいなくなりました。ホストに合流します</t>
+          <t>この場所の主はあなたになりました</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>The owner of this place is gone, rejoining the host</t>
+          <t>You are now the owner of this place</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>emp_travel_handoff</t>
+          <t>emp_ui_sv_cfg_independent_travel</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>この場所の主はあなたになりました</t>
+          <t>単独行動を許可</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>You are now the owner of this place</t>
+          <t>Independent travel</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_independent_travel</t>
+          <t>emp_ui_sv_cfg_player_shipping</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>単独行動を許可</t>
+          <t>出荷はプレイヤーごと</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Independent travel</t>
+          <t>Shipping per player</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_player_shipping</t>
+          <t>emp_ui_sv_cfg_combat_time</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>出荷はプレイヤーごと</t>
+          <t>戦闘は各プレイヤーの時間で進行</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Shipping per player</t>
+          <t>Combat on each player's time</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_combat_time</t>
+          <t>emp_ui_bot_add</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>戦闘は各プレイヤーの時間で進行</t>
+          <t>Add a bot player</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Combat on each player's time</t>
+          <t>Add a bot player</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>emp_ui_bot_add</t>
+          <t>emp_ui_bot_stop</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Add a bot player</t>
+          <t>Stop the bots ({0})</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Add a bot player</t>
+          <t>Stop the bots ({0})</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>emp_ui_bot_stop</t>
+          <t>emp_ui_bot_all_actions</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Stop the bots ({0})</t>
+          <t>Bots do everything (quests, selling, digging, chests)</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Stop the bots ({0})</t>
+          <t>Bots do everything (quests, selling, digging, chests)</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>emp_ui_bot_all_actions</t>
+          <t>emp_ui_bot_need_local</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Bots do everything (quests, selling, digging, chests)</t>
+          <t>Bots need a local server: disconnect, then add a bot to start one</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Bots do everything (quests, selling, digging, chests)</t>
+          <t>Bots need a local server: disconnect, then add a bot to start one</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>emp_ui_bot_need_local</t>
+          <t>emp_ui_bot_no_launcher</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Bots need a local server: disconnect, then add a bot to start one</t>
+          <t>No second copy of the game found (see _tools/make_lab.py)</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Bots need a local server: disconnect, then add a bot to start one</t>
+          <t>No second copy of the game found (see _tools/make_lab.py)</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>emp_ui_bot_no_launcher</t>
+          <t>emp_ui_bot_started</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>No second copy of the game found (see _tools/make_lab.py)</t>
+          <t>Bot player starting, it joins in about a minute</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>No second copy of the game found (see _tools/make_lab.py)</t>
+          <t>Bot player starting, it joins in about a minute</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>emp_ui_bot_started</t>
+          <t>emp_ui_sv_cfg_personal_quests</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Bot player starting, it joins in about a minute</t>
+          <t>ランダムクエスト・名声・カルマはプレイヤーごと</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Bot player starting, it joins in about a minute</t>
+          <t>Random quests, fame and karma per player</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_personal_quests</t>
+          <t>emp_ui_sv_cfg_choose_chara</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ランダムクエスト・名声・カルマはプレイヤーごと</t>
+          <t>参加時にプレイヤーがキャラクターを選ぶ</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Random quests, fame and karma per player</t>
+          <t>Players choose their character when joining</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_choose_chara</t>
+          <t>emp_ui_chara_pick</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Players choose their character when joining</t>
+          <t>どのキャラクターで遊びますか？</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Players choose their character when joining</t>
+          <t>Who do you want to play?</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>emp_ui_chara_pick</t>
+          <t>emp_ui_chara_new</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Who do you want to play?</t>
+          <t>新しいキャラクター</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Who do you want to play?</t>
+          <t>A new character</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>emp_ui_chara_new</t>
+          <t>emp_ui_sv_cfg_player_trade</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>A new character</t>
+          <t>プレイヤー間の取引ウィンドウ</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>A new character</t>
+          <t>Trade window between players</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_player_trade</t>
+          <t>emp_act_trade</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Trade window between players</t>
+          <t>取引</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Trade window between players</t>
+          <t>Trade</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>emp_act_trade</t>
+          <t>emp_ui_trade</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Trade</t>
+          <t>取引</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -2796,1912 +2791,2031 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>emp_ui_trade</t>
+          <t>emp_trade_invite</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Trade</t>
+          <t>{0} があなたと取引したがっています</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Trade</t>
+          <t>{0} wants to trade with you</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>emp_trade_invite</t>
+          <t>emp_trade_you_offer</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>{0} wants to trade with you</t>
+          <t>あなたの提示</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>{0} wants to trade with you</t>
+          <t>You offer</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>emp_trade_you_offer</t>
+          <t>emp_trade_they_offer</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>You offer</t>
+          <t>{0} の提示</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>You offer</t>
+          <t>{0} offers</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>emp_trade_they_offer</t>
+          <t>emp_trade_nothing</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>{0} offers</t>
+          <t>（まだなし）</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>{0} offers</t>
+          <t>(nothing yet)</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>emp_trade_nothing</t>
+          <t>emp_trade_add</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>(nothing yet)</t>
+          <t>アイテムを追加</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>(nothing yet)</t>
+          <t>Add an item</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>emp_trade_add</t>
+          <t>emp_trade_gold</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Add an item</t>
+          <t>金貨: {0}</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Add an item</t>
+          <t>Gold: {0}</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>emp_trade_gold</t>
+          <t>emp_trade_clear</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Gold: {0}</t>
+          <t>すべて取り下げる</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Gold: {0}</t>
+          <t>Take everything back</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>emp_trade_clear</t>
+          <t>emp_trade_confirm</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Take everything back</t>
+          <t>確認</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Take everything back</t>
+          <t>Confirm</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>emp_trade_confirm</t>
+          <t>emp_trade_cancel</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Confirm</t>
+          <t>キャンセル</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Confirm</t>
+          <t>Cancel</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>emp_trade_cancel</t>
+          <t>emp_trade_you_ready</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>あなたは確認しました</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>You confirmed</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>emp_trade_you_ready</t>
+          <t>emp_trade_you_wait</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>You confirmed</t>
+          <t>あなたは未確認です</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>You confirmed</t>
+          <t>You have not confirmed</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>emp_trade_you_wait</t>
+          <t>emp_trade_they_ready</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>You have not confirmed</t>
+          <t>相手は確認しました</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>You have not confirmed</t>
+          <t>the other player confirmed</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>emp_trade_they_ready</t>
+          <t>emp_trade_they_wait</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>the other player confirmed</t>
+          <t>相手は未確認です</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>the other player confirmed</t>
+          <t>the other player has not confirmed</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>emp_trade_they_wait</t>
+          <t>emp_trade_pick</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>the other player has not confirmed</t>
+          <t>どのアイテム？</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>the other player has not confirmed</t>
+          <t>Which item?</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>emp_trade_pick</t>
+          <t>emp_trade_howmany</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Which item?</t>
+          <t>何個？</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Which item?</t>
+          <t>How many?</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>emp_trade_howmany</t>
+          <t>emp_trade_howmuch</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>How many?</t>
+          <t>金貨はいくら？</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>How many?</t>
+          <t>How much gold?</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>emp_trade_howmuch</t>
+          <t>emp_trade_done</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>How much gold?</t>
+          <t>取引が完了しました</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>How much gold?</t>
+          <t>Trade done</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>emp_trade_done</t>
+          <t>emp_trade_cancelled</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Trade done</t>
+          <t>取引は中止されました</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Trade done</t>
+          <t>Trade cancelled</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>emp_trade_cancelled</t>
+          <t>emp_trade_invalid</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Trade cancelled</t>
+          <t>取引中止：提示したものがもう存在しません</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Trade cancelled</t>
+          <t>Trade cancelled: something offered is not there anymore</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>emp_trade_invalid</t>
+          <t>emp_trade_far</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Trade cancelled: something offered is not there anymore</t>
+          <t>取引中止：お互いが離れすぎています</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Trade cancelled: something offered is not there anymore</t>
+          <t>Trade cancelled: too far from each other</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>emp_trade_far</t>
+          <t>emp_trade_busy</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Trade cancelled: too far from each other</t>
+          <t>そのプレイヤーはすでに取引中です</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Trade cancelled: too far from each other</t>
+          <t>That player is already trading</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>emp_trade_busy</t>
+          <t>emp_ui_sv_note_live</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>That player is already trading</t>
+          <t>ホストのルールです。変更はすぐに全員に適用されます。</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>That player is already trading</t>
+          <t>These rules are the host's. A change applies at once, for everyone.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>emp_ui_sv_note_live</t>
+          <t>emp_ui_sv_sec_players</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>ホストのルールです。変更はすぐに全員に適用されます。</t>
+          <t>プレイヤーと移動</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>These rules are the host's. A change applies at once, for everyone.</t>
+          <t>Players and travel</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>emp_ui_sv_sec_players</t>
+          <t>emp_ui_sv_sec_own</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>プレイヤーと移動</t>
+          <t>プレイヤーごとのもの</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Players and travel</t>
+          <t>To each player its own</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>emp_ui_sv_sec_own</t>
+          <t>emp_ui_sv_sec_time</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>プレイヤーごとのもの</t>
+          <t>時間と戦闘</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>To each player its own</t>
+          <t>Time and combat</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>emp_ui_sv_sec_time</t>
+          <t>emp_ui_sv_sec_checks</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>時間と戦闘</t>
+          <t>参加時の検証（上級者向け）</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Time and combat</t>
+          <t>Joining checks (advanced)</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>emp_ui_sv_sec_checks</t>
+          <t>emp_ui_sv_desc_choose_chara</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>参加時の検証（上級者向け）</t>
+          <t>参加時に、この世界の自分のキャラクターから選ぶか、新しく作る。</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Joining checks (advanced)</t>
+          <t>A joining player picks one of its characters in this world, or makes a new one.</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_choose_chara</t>
+          <t>emp_ui_sv_desc_independent_travel</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>参加時に、この世界の自分のキャラクターから選ぶか、新しく作る。</t>
+          <t>誰でも好きな場所へ、一人でも一緒でも行ける。オフ：全員がホストについて行く。</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>A joining player picks one of its characters in this world, or makes a new one.</t>
+          <t>Everyone goes where they want, alone or together. Off: everyone follows the host.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_independent_travel</t>
+          <t>emp_ui_sv_desc_personal_quests</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>誰でも好きな場所へ、一人でも一緒でも行ける。オフ：全員がホストについて行く。</t>
+          <t>各自ランダムクエスト5件、報酬・名声・カルマも各自。メインクエストは共有。</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Everyone goes where they want, alone or together. Off: everyone follows the host.</t>
+          <t>5 random quests each, with their reward, fame and karma. Story quests stay shared.</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_personal_quests</t>
+          <t>emp_ui_sv_desc_player_shipping</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>各自ランダムクエスト5件、報酬・名声・カルマも各自。メインクエストは共有。</t>
+          <t>出荷箱の売上はアイテムを入れたプレイヤーへ。オフ：すべてホストへ。</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>5 random quests each, with their reward, fame and karma. Story quests stay shared.</t>
+          <t>Shipping box money goes to the player who put the item in. Off: all to the host.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_player_shipping</t>
+          <t>emp_ui_sv_desc_player_trade</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>出荷箱の売上はアイテムを入れたプレイヤーへ。オフ：すべてホストへ。</t>
+          <t>他のプレイヤーをクリックしてアイテムと金貨を交換。双方が確認する。</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Shipping box money goes to the player who put the item in. Off: all to the host.</t>
+          <t>Click another player to trade items and gold. Both confirm.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_player_trade</t>
+          <t>emp_ui_sv_desc_combat_time</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>他のプレイヤーをクリックしてアイテムと金貨を交換。双方が確認する。</t>
+          <t>モンスターは戦っている相手が動いた時に動く。誰も待たない。ターン制より優先。</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Click another player to trade items and gold. Both confirm.</t>
+          <t>A monster acts when the player it fights acts: nobody waits. Takes over turn-based.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_combat_time</t>
+          <t>emp_ui_sv_desc_turn_combat</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>モンスターは戦っている相手が動いた時に動く。誰も待たない。ターン制より優先。</t>
+          <t>戦闘中、プレイヤーは順番に行動する。「戦闘は各プレイヤーの時間で進行」がオンの間は無効。</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>A monster acts when the player it fights acts: nobody waits. Takes over turn-based.</t>
+          <t>In a fight, players act in turn. No effect while "Combat on each player's time" is on.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_turn_combat</t>
+          <t>emp_ui_sv_desc_shared_speed</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>戦闘中、プレイヤーは順番に行動する。「戦闘は各プレイヤーの時間で進行」がオンの間は無効。</t>
+          <t>全プレイヤーが平均速度を共有。オフ：各自の速度。</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>In a fight, players act in turn. No effect while "Combat on each player's time" is on.</t>
+          <t>One speed for all players, the average. Off: each keeps its own.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_shared_speed</t>
+          <t>emp_ui_sv_desc_validation</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>全プレイヤーが平均速度を共有。オフ：各自の速度。</t>
+          <t>参加するプレイヤーのゲームがホストと一致すべきもの。「なし」：誰でも。「すべて」：データとMODが同じ。</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>One speed for all players, the average. Off: each keeps its own.</t>
+          <t>What a joining player's game must share with yours. None: anyone. All: same data and mods.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_validation</t>
+          <t>emp_ui_sv_cfg_player_clock</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>参加するプレイヤーのゲームがホストと一致すべきもの。「なし」：誰でも。「すべて」：データとMODが同じ。</t>
+          <t>各プレイヤーは自分の時計で動く</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>What a joining player's game must share with yours. None: anyone. All: same data and mods.</t>
+          <t>Each player on its own clock</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_player_clock</t>
+          <t>emp_ui_sv_desc_player_clock</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>各プレイヤーは自分の時計で動く</t>
+          <t>ゲストもホストと同じように滑らかに動く（通信の速さに左右されない）。上のオプションが必要。</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Each player on its own clock</t>
+          <t>A guest walks and acts as smoothly as the host, not at the pace of the network. Needs the option above.</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_player_clock</t>
+          <t>emp_ui_sv_cfg_step_pace</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>ゲストもホストと同じように滑らかに動く（通信の速さに左右されない）。上のオプションが必要。</t>
+          <t>各プレイヤーはソロと同じ歩調で動く</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>A guest walks and acts as smoothly as the host, not at the pace of the network. Needs the option above.</t>
+          <t>Every player walks at the pace of a solo game</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_step_pace</t>
+          <t>emp_ui_sv_desc_step_pace</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>各プレイヤーはソロと同じ歩調で動く</t>
+          <t>歩く速さが他のプレイヤーの速度に左右されなくなります。戦闘では速度は今まで通り有効。「戦闘は各プレイヤーの時間で」が必要。</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Every player walks at the pace of a solo game</t>
+          <t>The length of a step no longer depends on the other players' speed. Speed still counts in a fight. Needs combat on each player's time.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_step_pace</t>
+          <t>emp_ui_sv_cfg_import_chara</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>歩く速さが他のプレイヤーの速度に左右されなくなります。戦闘では速度は今まで通り有効。「戦闘は各プレイヤーの時間で」が必要。</t>
+          <t>自分のセーブのキャラクターで参加できる</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>The length of a step no longer depends on the other players' speed. Speed still counts in a fight. Needs combat on each player's time.</t>
+          <t>Players can bring a character from their own saves</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_import_chara</t>
+          <t>emp_ui_sv_desc_import_chara</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>自分のセーブのキャラクターで参加できる</t>
+          <t>キャラクター本人、装備、持ち物、所持金、名声、カルマ。仲間、拠点、クエスト、銀行は含まれません。セーブは読むだけで変更しません。</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Players can bring a character from their own saves</t>
+          <t>The character, its equipment, bag and gold, its fame and karma. Not its companions, base, quests or bank. The save is only read, never changed.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_import_chara</t>
+          <t>emp_ui_chara_import</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>キャラクター本人、装備、持ち物、所持金、名声、カルマ。仲間、拠点、クエスト、銀行は含まれません。セーブは読むだけで変更しません。</t>
+          <t>自分のセーブのキャラクター…</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>The character, its equipment, bag and gold, its fame and karma. Not its companions, base, quests or bank. The save is only read, never changed.</t>
+          <t>A character from one of my saves…</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import</t>
+          <t>emp_ui_chara_import_pick</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>自分のセーブのキャラクター…</t>
+          <t>どのセーブのキャラクターで参加しますか？（セーブは変更されません）</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>A character from one of my saves…</t>
+          <t>Which save to bring the character of? (the save is not changed)</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_pick</t>
+          <t>emp_ui_chara_import_back</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>どのセーブのキャラクターで参加しますか？（セーブは変更されません）</t>
+          <t>戻る</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Which save to bring the character of? (the save is not changed)</t>
+          <t>Back</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_back</t>
+          <t>emp_ui_chara_import_none</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>戻る</t>
+          <t>読み込めるセーブがありません。</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Back</t>
+          <t>No save this game can read was found.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_none</t>
+          <t>emp_ui_chara_import_fail</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>読み込めるセーブがありません。</t>
+          <t>このキャラクターは読み込めませんでした。</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>No save this game can read was found.</t>
+          <t>That character could not be brought.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_fail</t>
+          <t>emp_ui_chara_import_twice</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>このキャラクターは読み込めませんでした。</t>
+          <t>このセーブのキャラクターはすでにこの世界にいます。</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>That character could not be brought.</t>
+          <t>The character of that save is already in this world.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_twice</t>
+          <t>emp_ui_sv_cfg_world_time</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>このセーブのキャラクターはすでにこの世界にいます。</t>
+          <t>世界の時間は全員で一つ</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>The character of that save is already in this world.</t>
+          <t>One date for the whole world</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_world_time</t>
+          <t>emp_ui_sv_desc_world_time</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>世界の時間は全員で一つ</t>
+          <t>一人で別のマップにいるプレイヤーの時間も世界の時間になります。一番進んだ日付が世界の日付。オフ：ホストの日付だけ。</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>One date for the whole world</t>
+          <t>Time passed by a player alone on another map counts for everyone: the most advanced date is the world's. Off: only the host's date counts.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_world_time</t>
+          <t>emp_ui_sv_cfg_world_keeper</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>一人で別のマップにいるプレイヤーの時間も世界の時間になります。一番進んだ日付が世界の日付。オフ：ホストの日付だけ。</t>
+          <t>世界の出来事は一度だけ起きる</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Time passed by a player alone on another map counts for everyone: the most advanced date is the world's. Off: only the host's date counts.</t>
+          <t>What time does to the world happens once</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_world_keeper</t>
+          <t>emp_ui_sv_desc_world_keeper</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>世界の出来事は一度だけ起きる</t>
+          <t>天気、依頼の期限切れ、税金、給料、手紙は一つのゲームだけが処理します。オフ：マップを持つ各プレイヤーのゲームでも起きます。</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>What time does to the world happens once</t>
+          <t>Weather, expired quests, taxes, salaries and letters are handled by one game only, the same for everyone. Off: every player holding a map runs them too.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_world_keeper</t>
+          <t>emp_ui_depot_take</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>天気、依頼の期限切れ、税金、給料、手紙は一つのゲームだけが処理します。オフ：マップを持つ各プレイヤーのゲームでも起きます。</t>
+          <t>サーバーから世界を取り出してホストする</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Weather, expired quests, taxes, salaries and letters are handled by one game only, the same for everyone. Off: every player holding a map runs them too.</t>
+          <t>Take the world from the server and host it</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>emp_ui_depot_take</t>
+          <t>emp_ui_depot_put</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>サーバーから世界を取り出してホストする</t>
+          <t>このセーブをサーバーに置く</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Take the world from the server and host it</t>
+          <t>Put this save on the server</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>emp_ui_depot_put</t>
+          <t>emp_ui_depot_held</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>このセーブをサーバーに置く</t>
+          <t>{0} が世界をホスト中です。Steam で参加してください（招待してもらうか、Steam のフレンド一覧で「ゲームに参加」）。相手が抜けた直後なら、最大3分待ってください。</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Put this save on the server</t>
+          <t>{0} is hosting the world. Join them through Steam: ask for an invite, or use "Join Game" on their name in your Steam friends list. If they have just left, wait up to 3 minutes.</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>emp_ui_depot_held</t>
+          <t>emp_ui_depot_empty</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>{0} が世界をホスト中です。Steam で参加してください（招待してもらうか、Steam のフレンド一覧で「ゲームに参加」）。相手が抜けた直後なら、最大3分待ってください。</t>
+          <t>サーバーにまだ世界がありません。ゲームを開始または読み込み、このパネルの「Lobby」で「このセーブをサーバーに置く」を押してください。</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>{0} is hosting the world. Join them through Steam: ask for an invite, or use "Join Game" on their name in your Steam friends list. If they have just left, wait up to 3 minutes.</t>
+          <t>The server holds no world yet. Start or load a game, then open this panel again: Lobby tab, "Put this save on the server".</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>emp_ui_depot_empty</t>
+          <t>emp_ui_depot_fail</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>サーバーにまだ世界がありません。ゲームを開始または読み込み、このパネルの「Lobby」で「このセーブをサーバーに置く」を押してください。</t>
+          <t>デポに接続できない、または読み書きできませんでした。</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>The server holds no world yet. Start or load a game, then open this panel again: Lobby tab, "Put this save on the server".</t>
+          <t>The depot could not be reached, read or written.</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>emp_ui_depot_fail</t>
+          <t>emp_ui_depot_put_done</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>デポに接続できない、または読み書きできませんでした。</t>
+          <t>この世界はサーバーに置かれました。これからサーバーから読み込み直します。以後のセーブはすべてサーバーに送られます。</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>The depot could not be reached, read or written.</t>
+          <t>This world is now on the server. The game reloads it from there: from now on every save goes to the server.</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>emp_ui_depot_put_done</t>
+          <t>emp_ui_depot_folder</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>この世界はサーバーに置かれました。これからサーバーから読み込み直します。以後のセーブはすべてサーバーに送られます。</t>
+          <t>デポ</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>This world is now on the server. The game reloads it from there: from now on every save goes to the server.</t>
+          <t>Depot</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>emp_ui_depot_folder</t>
+          <t>emp_ui_depot_folder_ask</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>デポ（フォルダ、サーバーのアドレス、または GitHub）: {0}</t>
+          <t>セーブデポ：Elin Together Server のアドレス（ホスト:55557）、共有フォルダ、または非公開の GitHub リポジトリ（github:所有者/リポジトリ）。空欄でオフ</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Depot (folder, server address or GitHub): {0}</t>
+          <t>Save depot: the address of Elin Together Server (host:55557), a folder the whole group can reach, or a private GitHub repository (github:owner/repository). Empty for none</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>emp_ui_depot_folder_ask</t>
+          <t>emp_ui_join_address</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>セーブデポ：Elin Together Server のアドレス（ホスト:55557）、共有フォルダ、または非公開の GitHub リポジトリ（github:所有者/リポジトリ）。空欄でオフ</t>
+          <t>アドレスで参加</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Save depot: the address of Elin Together Server (host:55557), a folder the whole group can reach, or a private GitHub repository (github:owner/repository). Empty for none</t>
+          <t>Join by address</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>emp_ui_join_address</t>
+          <t>emp_ui_join_address_ask</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>アドレスで参加</t>
+          <t>サーバーのアドレス（ホスト:ポート。Elin ありは 55556、Elin なしは 55557）</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Join by address</t>
+          <t>Address of the server (host:port; the port is 55556 with Elin, 55557 without)</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>emp_ui_join_address_ask</t>
+          <t>emp_ui_depot_password</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>サーバーのアドレス（ホスト:ポート。Elin ありは 55556、Elin なしは 55557）</t>
+          <t>デポのキー</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Address of the server (host:port; the port is 55556 with Elin, 55557 without)</t>
+          <t>Depot key</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>emp_ui_depot_password</t>
+          <t>emp_ui_depot_password_ask</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>デポのパスワード／GitHub のキー: {0}</t>
+          <t>デポのパスワード（サーバーで設定した場合）、または GitHub のアクセスキー。キーは二度と表示されません。空欄のままなら現在のキーを保持します</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Depot password or GitHub key: {0}</t>
+          <t>Password of the depot (when one was set in Elin Together Server), or the GitHub access key. A key is never shown again: leave empty to keep it</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>emp_ui_depot_password_ask</t>
+          <t>emp_ui_timeout</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>デポのパスワード（サーバーで設定した場合）、または GitHub のアクセスキー。キーは二度と表示されません。空欄のままなら現在のキーを保持します</t>
+          <t>サーバーが応答しません。アドレス、ポート、サーバーのモードを確認してください。</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Password of the depot (when one was set in Elin Together Server), or the GitHub access key. A key is never shown again: leave empty to keep it</t>
+          <t>The server does not answer. Check the address, the port and the mode of the server.</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>emp_ui_timeout</t>
+          <t>emp_ui_depot_password_wrong</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>サーバーが応答しません。アドレス、ポート、サーバーのモードを確認してください。</t>
+          <t>サーバーがパスワードを拒否しました。「Client Settings」の「デポのキー」で設定してください。</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>The server does not answer. Check the address, the port and the mode of the server.</t>
+          <t>The server refused the password. Set it in Client Settings, "Depot key".</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>emp_ui_depot_password_wrong</t>
+          <t>emp_ui_depot_lost</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>サーバーがパスワードを拒否しました。「Client Settings」の「デポのパスワード」で設定してください。</t>
+          <t>接続が切れている間に {0} がサーバーの世界を引き継ぎました。ここからのプレイはサーバーに届きません。タイトルに戻って相手に参加してください。</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>The server refused the password. Set it in Client Settings, "Depot password".</t>
+          <t>{0} took over the world on the server while this game was cut off. What you play from here no longer reaches the server: go back to the title screen and join them.</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>emp_ui_depot_lost</t>
+          <t>emp_ui_depot_unsaved</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>接続が切れている間に {0} がサーバーの世界を引き継ぎました。ここからのプレイはサーバーに届きません。タイトルに戻って相手に参加してください。</t>
+          <t>このセーブはサーバーに届きませんでした。このPCには保存されています。次のセーブで再送します。</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>{0} took over the world on the server while this game was cut off. What you play from here no longer reaches the server: go back to the title screen and join them.</t>
+          <t>The server did not receive this save. It is kept on this PC; the next save tries again.</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>emp_ui_depot_unsaved</t>
+          <t>emp_ui_depot_unsent</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>このセーブはサーバーに届きませんでした。このPCには保存されています。次のセーブで再送します。</t>
+          <t>前回のプレイの最後のセーブがサーバーに届いていません。今送りますか？（はい：サーバーにある世界は別に保管されます。いいえ：このPCの分を破棄し、サーバーの世界を使います）</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>The server did not receive this save. It is kept on this PC; the next save tries again.</t>
+          <t>The last save of your previous session never reached the server. Send it now? (Yes: the world the server holds now is kept aside. No: your save is dropped and the server's world is used.)</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>emp_ui_depot_unsent</t>
+          <t>emp_quest_follow_ask</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>前回のプレイの最後のセーブがサーバーに届いていません。今送りますか？（はい：サーバーにある世界は別に保管されます。いいえ：このPCの分を破棄し、サーバーの世界を使います）</t>
+          <t>{0}がクエストに出発します。同行しますか？報酬は{0}のものです。</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>The last save of your previous session never reached the server. Send it now? (Yes: the world the server holds now is kept aside. No: your save is dropped and the server's world is used.)</t>
+          <t>{0} is leaving on a quest. Go along? The reward goes to {0}.</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>emp_quest_follow_ask</t>
+          <t>emp_quest_follow_declined</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>{0}がクエストに出発します。同行しますか？報酬は{0}のものです。</t>
+          <t>{0}は同行を断りました。</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>{0} is leaving on a quest. Go along? The reward goes to {0}.</t>
+          <t>{0} declined to come along.</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>emp_quest_follow_declined</t>
+          <t>emp_quest_follow_no_answer</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>{0}は同行を断りました。</t>
+          <t>{0}から返事がありません。</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>{0} declined to come along.</t>
+          <t>{0} did not answer.</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>emp_quest_follow_no_answer</t>
+          <t>emp_quest_follow_asked</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>{0}から返事がありません。</t>
+          <t>{0}に同行するか尋ねています…</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>{0} did not answer.</t>
+          <t>Asking {0} to come along...</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>emp_quest_follow_asked</t>
+          <t>emp_base_host_only</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>{0}に同行するか尋ねています…</t>
+          <t>今のところ、これはホストだけができます。</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Asking {0} to come along...</t>
+          <t>Only the host can do this for now.</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>emp_base_host_only</t>
+          <t>emp_trade_equipped</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>今のところ、これはホストだけができます。</t>
+          <t>取引中止：提示したアイテムが装備されています</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Only the host can do this for now.</t>
+          <t>Trade cancelled: an offered item is now equipped</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>emp_trade_equipped</t>
+          <t>emp_trade_nodrop</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>取引中止：提示したアイテムが装備されています</t>
+          <t>取引中止：提示したアイテムは手放せません</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Trade cancelled: an offered item is now equipped</t>
+          <t>Trade cancelled: an offered item cannot be dropped or given away</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>emp_trade_nodrop</t>
+          <t>emp_trade_npcprop</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>取引中止：提示したアイテムは手放せません</t>
+          <t>取引中止：提示したアイテムはNPCの所有物です</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Trade cancelled: an offered item cannot be dropped or given away</t>
+          <t>Trade cancelled: an offered item belongs to an NPC</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>emp_trade_npcprop</t>
+          <t>emp_trade_gifted</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>取引中止：提示したアイテムはNPCの所有物です</t>
+          <t>取引中止：提示したアイテムは贈り物のため取引できません</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Trade cancelled: an offered item belongs to an NPC</t>
+          <t>Trade cancelled: an offered item is a gift and cannot be traded</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>emp_trade_gifted</t>
+          <t>emp_trade_bound</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>取引中止：提示したアイテムは贈り物のため取引できません</t>
+          <t>取引中止：提示したアイテムはキャラクターに結び付いています</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Trade cancelled: an offered item is a gift and cannot be traded</t>
+          <t>Trade cancelled: an offered item is bound to a character</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>emp_trade_bound</t>
+          <t>emp_trade_full</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>取引中止：提示したアイテムはキャラクターに結び付いています</t>
+          <t>取引中止：受け取るアイテムに対してバッグの空きが足りません</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Trade cancelled: an offered item is bound to a character</t>
+          <t>Trade cancelled: a bag does not have enough free slots for what it would receive</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>emp_trade_full</t>
+          <t>emp_travel_recalled_by</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>取引中止：受け取るアイテムに対してバッグの空きが足りません</t>
+          <t>{@Peer} がこの場所に来ます。画面が再読み込みされ、合流します…</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Trade cancelled: a bag does not have enough free slots for what it would receive</t>
+          <t>{@Peer} is coming to this place: the screen will reload to rejoin them…</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>emp_travel_recalled_by</t>
+          <t>emp_ui_thing_gone</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>{@Peer} がこの場所に来ます。画面が再読み込みされ、合流します…</t>
+          <t>遅かったようです。他のプレイヤーが先に取りました</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>{@Peer} is coming to this place: the screen will reload to rejoin them…</t>
+          <t>Too late: someone else already took it</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>emp_ui_thing_gone</t>
+          <t>emp_base_refused</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>遅かったようです。他のプレイヤーが先に取りました</t>
+          <t>ホストに断られました。拠点または所持金では、もう支払えません。</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Too late: someone else already took it</t>
+          <t>The host refused: the base or your purse can no longer pay for this.</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>emp_base_refused</t>
+          <t>emp_base_pending</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>ホストに断られました。拠点または所持金では、もう支払えません。</t>
+          <t>前回の依頼はまだホストの返事を待っています。</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>The host refused: the base or your purse can no longer pay for this.</t>
+          <t>Your last request is still waiting for the host's answer.</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>emp_base_pending</t>
+          <t>emp_game_version_differs</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>前回の依頼はまだホストの返事を待っています。</t>
+          <t>{0} のElinのバージョンが異なります（{1} ／ こちら {2}）。接続は許可されます。問題が起きたら同じバージョンに揃えてください。</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Your last request is still waiting for the host's answer.</t>
+          <t>{0} runs another version of Elin ({1}, here {2}). The connection is allowed; if something goes wrong, use the same version.</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>emp_game_version_differs</t>
+          <t>emp_ui_sv_cfg_same_game_version</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>{0} のElinのバージョンが異なります（{1} ／ こちら {2}）。接続は許可されます。問題が起きたら同じバージョンに揃えてください。</t>
+          <t>同じElinバージョンを必須にする</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>{0} runs another version of Elin ({1}, here {2}). The connection is allowed; if something goes wrong, use the same version.</t>
+          <t>Require the same Elin version</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_same_game_version</t>
+          <t>emp_ui_sv_desc_same_game_version</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>同じElinバージョンを必須にする</t>
+          <t>オン：Elinのバージョンが違うプレイヤーを拒否。オフ：警告のうえ参加を許可。Modのバージョンは常に同じである必要があります。</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Require the same Elin version</t>
+          <t>On: players on another version of Elin are refused. Off: they are let in with a warning. The same version of the mod is always required.</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_same_game_version</t>
+          <t>emp_ui_sv_cfg_guest_build</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>オン：Elinのバージョンが違うプレイヤーを拒否。オフ：警告のうえ参加を許可。Modのバージョンは常に同じである必要があります。</t>
+          <t>他のプレイヤーも建築モードを使える</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>On: players on another version of Elin are refused. Off: they are let in with a warning. The same version of the mod is always required.</t>
+          <t>Other players can use build mode</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_guest_build</t>
+          <t>emp_ui_sv_desc_guest_build</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>他のプレイヤーも建築モードを使える</t>
+          <t>オン：他のプレイヤーも拠点の建築モード（床・壁・家具・採掘・伐採）を使えます。ホストのゲームが代わりに建て、費用と素材は本人が払います。オフ：ホストだけが建てられます。</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Other players can use build mode</t>
+          <t>On: the other players can use the build mode of the base (floors, walls, furniture, mining, cutting). The game of the host builds for them; they pay the gold and the materials. Off: only the host builds.</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_guest_build</t>
+          <t>emp_ui_depot_gh_help</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
-        <is>
-          <t>オン：他のプレイヤーも拠点の建築モード（床・壁・家具・採掘・伐採）を使えます。ホストのゲームが代わりに建て、費用と素材は本人が払います。オフ：ホストだけが建てられます。</t>
-        </is>
-      </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>On: the other players can use the build mode of the base (floors, walls, furniture, mining, cutting). The game of the host builds for them; they pay the gold and the materials. Off: only the host builds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>emp_ui_depot_gh_help</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
         <is>
           <t>非公開の GitHub リポジトリをデポにできます（サーバーも共有フォルダも不要、フレンドは GitHub アカウント不要）：
 1. github.com で、この世界専用の空の非公開（Private）リポジトリを作成します。
 2. そのリポジトリ用のアクセスキーを1つ作成します：Settings → Developer settings → Fine-grained tokens、このリポジトリのみ、Contents: Read and write。
-3. キーを「デポのパスワード／GitHub のキー」に貼り付け、「デポ」に github:所有者/リポジトリ と入力します。
+3. キーを「デポのキー」に貼り付け、「デポ」に github:所有者/リポジトリ と入力します。
 4. 同じ2行をフレンドに送り、フレンドもここに入力します。このキーで開けるのはこのリポジトリだけです。</t>
         </is>
       </c>
-      <c r="D228" t="inlineStr">
+      <c r="D227" t="inlineStr">
         <is>
           <t>A private GitHub repository can be the depot (no server, no shared folder, your friends need no GitHub account):
 1. On github.com, create an empty private repository, only for this world.
 2. Create one access key for it: Settings, Developer settings, Fine-grained tokens; only this repository; Contents: Read and write.
-3. Paste the key in "Depot password or GitHub key" and write github:owner/repository in "Depot".
+3. Paste the key in "Depot key" and write github:owner/repository in "Depot".
 4. Send the same two lines to your friends: they type them here too. The key only opens this one repository.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_key</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>GitHub がアクセスキーを拒否しました。キーの有効期限、このリポジトリが対象になっているか、「Contents: Read and write」の権限があるかを確認し、「Client Settings」で貼り付け直してください。</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>GitHub refused the access key. Check that it has not expired, that it covers this repository with "Contents: Read and write", then paste it again in Client Settings.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_key</t>
+          <t>emp_ui_depot_gh_missing</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>GitHub がアクセスキーを拒否しました。キーの有効期限、このリポジトリが対象になっているか、「Contents: Read and write」の権限があるかを確認し、「Client Settings」で貼り付け直してください。</t>
+          <t>GitHub でデポのリポジトリが見つかりません。「Client Settings」の名前（github:所有者/リポジトリ）と、アクセスキーがそのリポジトリを対象にしているかを確認してください。</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>GitHub refused the access key. Check that it has not expired, that it covers this repository with "Contents: Read and write", then paste it again in Client Settings.</t>
+          <t>GitHub does not find the repository of the depot. Check its name (github:owner/repository) in Client Settings, and that your access key covers it.</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_missing</t>
+          <t>emp_ui_depot_gh_public</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>GitHub でデポのリポジトリが見つかりません。「Client Settings」の名前（github:所有者/リポジトリ）と、アクセスキーがそのリポジトリを対象にしているかを確認してください。</t>
+          <t>この GitHub リポジトリは公開されています。世界とその履歴がすべて誰にでも見えてしまいます。非公開にしてから（Settings → Danger Zone → Change visibility）、もう一度お試しください。</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>GitHub does not find the repository of the depot. Check its name (github:owner/repository) in Client Settings, and that your access key covers it.</t>
+          <t>This GitHub repository is public: your world and all its history would be visible to everyone. Make it private (Settings, Danger Zone, Change visibility), then try again.</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_public</t>
+          <t>emp_ui_depot_gh_big</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>この GitHub リポジトリは公開されています。世界とその履歴がすべて誰にでも見えてしまいます。非公開にしてから（Settings → Danger Zone → Change visibility）、もう一度お試しください。</t>
+          <t>この世界は 20 MB を超えており、GitHub のデポには大きすぎます。Elin Together Server か共有フォルダを使ってください。セーブはこのPCに保存されています。</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>This GitHub repository is public: your world and all its history would be visible to everyone. Make it private (Settings, Danger Zone, Change visibility), then try again.</t>
+          <t>This world is over 20 MB: too big for a GitHub depot. Use Elin Together Server or a shared folder instead. The save is kept on this PC.</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_big</t>
+          <t>emp_ui_depot_gh_changed</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>この世界は 20 MB を超えており、GitHub のデポには大きすぎます。Elin Together Server か共有フォルダを使ってください。セーブはこのPCに保存されています。</t>
+          <t>接続が切れている間に、他のプレイヤーがデポの世界をホストしてセーブしました。あなたのセーブはこのPCに残り、デポには届きません。タイトルに戻って、もう一度世界を取り出してください。</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>This world is over 20 MB: too big for a GitHub depot. Use Elin Together Server or a shared folder instead. The save is kept on this PC.</t>
+          <t>The world in the depot changed while this game was cut off: someone else hosted it and saved. Your saves stay on this PC and no longer reach the depot. Go back to the title screen and take the world again.</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_changed</t>
+          <t>emp_ui_depot_gh_down</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>接続が切れている間に、他のプレイヤーがデポの世界をホストしてセーブしました。あなたのセーブはこのPCに残り、デポには届きません。タイトルに戻って、もう一度世界を取り出してください。</t>
+          <t>GitHub から応答がありません。接続を確認して、しばらくしてからもう一度お試しください。</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>The world in the depot changed while this game was cut off: someone else hosted it and saved. Your saves stay on this PC and no longer reach the depot. Go back to the title screen and take the world again.</t>
+          <t>GitHub does not answer. Check your connection and try again in a moment.</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_down</t>
+          <t>emp_ui_sv_cfg_player_kill</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>GitHub から応答がありません。接続を確認して、しばらくしてからもう一度お試しください。</t>
+          <t>プレイヤー同士で殺せる</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>GitHub does not answer. Check your connection and try again in a moment.</t>
+          <t>Players can kill each other</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_player_kill</t>
+          <t>emp_ui_sv_desc_player_kill</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>プレイヤー同士で殺せる</t>
+          <t>オン：プレイヤー（とその仲間）の攻撃で他のプレイヤーのキャラクターが死にます。オフ：致命的な一撃でも相手のHPは0で止まり、死にません。</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Players can kill each other</t>
+          <t>On: a strike of a player (or of its companions) can kill another player's character. Off: a strike that would kill it leaves it at 0 hit points, alive.</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_player_kill</t>
+          <t>emp_ui_sv_cfg_host_manages_base</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>オン：プレイヤー（とその仲間）の攻撃で他のプレイヤーのキャラクターが死にます。オフ：致命的な一撃でも相手のHPは0で止まり、死にません。</t>
+          <t>拠点の管理はホストだけ</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>On: a strike of a player (or of its companions) can kill another player's character. Off: a strike that would kill it leaves it at 0 hit points, alive.</t>
+          <t>Only the host manages the base</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_host_manages_base</t>
+          <t>emp_ui_sv_desc_host_manages_base</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>拠点の管理はホストだけ</t>
+          <t>オン：他のプレイヤーによる拠点の操作（研究、炉の技能、政策、名前、物の設定、住民、建築モード）は拒否されます。オフ：全員がホストと同じように拠点を管理できます。拠点の放棄は常にホストだけです。</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Only the host manages the base</t>
+          <t>On: what the other players ask of the base (research, hearth skills, policies, names, settings of an object, residents, build mode) is refused. Off: every player manages the base as the host does. Leaving the base for good always stays the host's.</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_host_manages_base</t>
+          <t>emp_ui_sv_cfg_duels</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>オン：他のプレイヤーによる拠点の操作（研究、炉の技能、政策、名前、物の設定、住民、建築モード）は拒否されます。オフ：全員がホストと同じように拠点を管理できます。拠点の放棄は常にホストだけです。</t>
+          <t>プレイヤー同士の決闘</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>On: what the other players ask of the base (research, hearth skills, policies, names, settings of an object, residents, build mode) is refused. Off: every player manages the base as the host does. Leaving the base for good always stays the host's.</t>
+          <t>Duels between players</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_duels</t>
+          <t>emp_ui_sv_desc_duels</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>プレイヤー同士の決闘</t>
+          <t>オン：相手キャラクターのメニューから決闘を申し込めます。誰も死なず、終了時に両者が回復し、何も失いません。オフ：決闘なし。</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Duels between players</t>
+          <t>On: a player can challenge another from the menu on its character. Nobody dies, both are healed, nothing is lost. Off: no duels.</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_duels</t>
+          <t>emp_act_duel</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>オン：相手キャラクターのメニューから決闘を申し込めます。誰も死なず、終了時に両者が回復し、何も失いません。オフ：決闘なし。</t>
+          <t>決闘を申し込む</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>On: a player can challenge another from the menu on its character. Nobody dies, both are healed, nothing is lost. Off: no duels.</t>
+          <t>Challenge to a duel</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>emp_act_duel</t>
+          <t>emp_duel_invite</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>決闘を申し込む</t>
+          <t>{0} が決闘を申し込んできました。誰も死なず何も失いませんが、決闘中に使ったポーション・矢・チャージは戻りません。受けますか？</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Challenge to a duel</t>
+          <t>{0} challenges you to a duel. Nobody dies and nothing is lost, but potions, arrows and charges used during the duel stay spent. Accept?</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>emp_duel_invite</t>
+          <t>emp_duel_asked</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>{0} が決闘を申し込んできました。誰も死なず何も失いませんが、決闘中に使ったポーション・矢・チャージは戻りません。受けますか？</t>
+          <t>{0} に決闘を申し込みました…</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>{0} challenges you to a duel. Nobody dies and nothing is lost, but potions, arrows and charges used during the duel stay spent. Accept?</t>
+          <t>You challenge {0} to a duel…</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>emp_duel_asked</t>
+          <t>emp_duel_countdown</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>{0} に決闘を申し込みました…</t>
+          <t>決闘：{0} 対 {1}。3秒後に開始！</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>You challenge {0} to a duel…</t>
+          <t>Duel: {0} against {1}. It starts in 3 seconds!</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>emp_duel_countdown</t>
+          <t>emp_duel_fight</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>決闘：{0} 対 {1}。3秒後に開始！</t>
+          <t>始め！</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Duel: {0} against {1}. It starts in 3 seconds!</t>
+          <t>Fight!</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>emp_duel_fight</t>
+          <t>emp_duel_won</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>始め！</t>
+          <t>{0} が {1} との決闘に勝ちました。</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Fight!</t>
+          <t>{0} won the duel against {1}.</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>emp_duel_won</t>
+          <t>emp_duel_declined</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>{0} が {1} との決闘に勝ちました。</t>
+          <t>決闘は断られました。</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>{0} won the duel against {1}.</t>
+          <t>The duel was declined.</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>emp_duel_declined</t>
+          <t>emp_duel_noanswer</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>決闘は断られました。</t>
+          <t>返事がなく、決闘は行われません。</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>The duel was declined.</t>
+          <t>No answer: no duel.</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>emp_duel_noanswer</t>
+          <t>emp_duel_busy</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>返事がなく、決闘は行われません。</t>
+          <t>そのプレイヤーは決闘中か取引中です。</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>No answer: no duel.</t>
+          <t>That player is already in a duel or a trade.</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>emp_duel_busy</t>
+          <t>emp_duel_over</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>そのプレイヤーは決闘中か取引中です。</t>
+          <t>決闘は勝者なしで終わりました。</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>That player is already in a duel or a trade.</t>
+          <t>The duel is over, without a winner.</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>emp_duel_over</t>
+          <t>emp_handover_failed</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>決闘は勝者なしで終わりました。</t>
+          <t>あなたのキャラクター {0} はこの世界で交代できませんでした（死亡しています）。セーブデータのキャラクターで遊んでいます。</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>The duel is over, without a winner.</t>
+          <t>Your character {0} could not take its place in this world (it is dead). You are playing the character of the save.</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_held_btn</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>{0} が世界をホスト中</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>{0} is hosting the world</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>emp_error_connection</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>接続できませんでした。ゲームが応答しません。まだ開いているか確認して、もう一度お試しください。</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Could not connect: the game does not answer. Check that it is still open, then try again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>emp_not_allowed</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>このゲームは、Steam のロビーから参加したプレイヤーだけを受け入れます。</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>This game only accepts players who joined through its Steam lobby.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>emp_connection_no_server</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>そのゲームはまだ開かれていません。しばらくしてからもう一度お試しください。</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>That game is not open yet. Try again in a moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>emp_zone_session_empty</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>ここには他のプレイヤーがいなくなりました</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>No other player is here anymore</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>emp_ui_timeout_steam</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>ゲームが応答しません。相手が退出したか、接続が切れた可能性があります。</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>The game does not answer: its player may have left or lost the connection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>emp_trade_nothing_to_offer</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>提示できるアイテムがありません。</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>You have nothing you can offer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
wip (not played, compiled aside in Release and Debug): boss of a dungeon gone for a player who joins another on its floor, a world taken from the depot opens its session, bank and shipping chest of a guest alone elsewhere, known players come in without being Steam friends, a guest's own waking (spellbook, pillow, recipe), a learnt recipe no longer echoes to its sender, slowness with several guests (network batch, cache sweep, fast map compression, one grouped save on a return, quest invitation to a visitor); tests written, to be played
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D270"/>
+  <dimension ref="A1:D271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5041,6 +5041,23 @@
         </is>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>emp_ui_box_far</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>この箱は世界共通で、ホストが保管しています。ホストから離れて他のプレイヤーと一緒にいる間は、入れた物はホストに届きますが、ホストのマップに戻るまで表示されません。</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>This chest belongs to the whole world and is kept by the host. With other players away from the host, what you put in arrives there, but it only shows again once you are back on the host's map.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
wip: three host checkboxes decided by council 10 (own sleep, time jumps together, auto-dump spares the belt), declared only; verdict in dev/PLAN_conseil10_verdict.md; pickup with a full bag
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D271"/>
+  <dimension ref="A1:D277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5058,6 +5058,108 @@
         </is>
       </c>
     </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_own_sleep</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>みんな自分のために眠る</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Everyone sleeps for themselves</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_own_sleep</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>オン：ベッドに入ったプレイヤーは誰も待たずにすぐ眠ります。全員が同時に眠ったときだけ、ワールドの夜が明けます。オフ：全員が互いを待ちます。</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>On: a player who goes to bed sleeps at once, without waiting for anyone. The night only passes for the world when every player is asleep at the same time. Off: everyone waits for everyone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_time_jumps_together</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>時間は全員一緒のときだけ飛ぶ</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Time only jumps when everyone jumps</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_time_jumps_together</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>オン：ワールドマップの一歩は、全プレイヤーが一緒に旅しているときだけワールドの日付を進めます。それ以外は旅人が自分のターンだけを払います。オフ：誰の一歩でも全員に3時間が加わります。</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>On: a step on the world map only moves the date of the world when all the players travel on it together. Otherwise the traveller pays its own turns and the date stays. Off: every step of anyone adds 3 hours for all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_dump_spares_belt</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>自動収納は手とベルトに触れない</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Auto-dump spares hand and tool belt</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_dump_spares_belt</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>オン：自動収納は、手に持っている物とツールベルトの中身を収納しません（ホットバーと同じ）。オフ：ゲーム本来の動作。</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>On: auto-dump leaves what you hold and what is in your tool belt, as it leaves the hotbar. Off: as in the game.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
wip (not played): council 10 (iv), the date: a quest timer no longer takes another player's time, a step on the world map moves the date only when all travel together, a guest beside the host pays its own step
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D277"/>
+  <dimension ref="A1:D278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5160,6 +5160,23 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>emp_ui_travel_no_date</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>仲間は別の場所にいる。この旅では日付は進まない。</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Your friends are elsewhere: your trip does not move the date.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
wip (not played): council 10 (i) auto-dump spares the held item and the tool belt, (v) a guest can pay a bill, once, with its own gold, and everyone reads who paid
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D278"/>
+  <dimension ref="A1:D280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5177,6 +5177,40 @@
         </is>
       </c>
     </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>emp_ui_bill_paid</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>{0}が請求書を支払いました：{1}（{2}）</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>{0} paid a bill: {1} ({2})</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>emp_ui_bill_already_paid</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>この請求書はすでに支払い済みです。所持金は減っていません。</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>This bill is already paid: nothing was taken from you.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
wip (not played): council 10 (iii), the night: each player sleeps for itself at once, the world's night passes when all sleep; a host alone lives the solo game (14 conditions); desync inquiry
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D280"/>
+  <dimension ref="A1:D283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5211,6 +5211,57 @@
         </is>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>emp_ui_sleep_alone</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>眠った。世界の時間は進まなかった：{0} がまだ起きている。</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>You slept. The world did not move on: {0} still awake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>emp_ui_sleep_count</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>{0} は眠っている（{1}/{2}）</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>{0} is asleep ({1} of {2})</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>emp_ui_sleep_all</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>全員が眠った：夜が過ぎていく。</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Everyone is asleep: the night passes.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
wip (not played): desync detector (a few sums per map compared every 2 s, a warning in both logs, the map loaded again by itself, host checkbox AutoResync)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D283"/>
+  <dimension ref="A1:D286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5262,6 +5262,57 @@
         </is>
       </c>
     </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>emp_ui_resync</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>マップを同期し直しています…</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Bringing the map up to date…</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_auto_resync</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>マップを自動で修復</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Repair the map by itself</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_auto_resync</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>オン：マップがホストと食い違ったプレイヤー（アイテムやキャラクターの欠落）は、自動でマップを読み込み直します（30秒に1回まで）。オフ：食い違いはログに書かれるだけです。</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>On: a player whose map no longer matches the host's (a missing item or character) loads it again by itself, at most once every 30 seconds. Off: the difference is only written to the log.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
wip (not played): training dummy for a guest, a bag that differs is asked again from its keeper, hand-over between guests, guests keep a copy of the world (council 9, step 3), bank (a taken item is kept until the guest has it, deposits and withdrawals told to all), tax on the highest fame (host checkbox SharedTax), a guest alone elsewhere pays a bill
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D286"/>
+  <dimension ref="A1:D292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5313,6 +5313,108 @@
         </is>
       </c>
     </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>emp_ui_bank_deposit</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>{0}が銀行に{1}を預けました</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>{0} put {1} in the bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>emp_ui_bank_withdraw</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>{0}が銀行から{1}を引き出しました</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>{0} took {1} out of the bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_world_copy</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>他のプレイヤーがワールドのコピーを保持する</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>The other players keep a copy of the world</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_world_copy</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>オン：自動セーブのたびに、各プレイヤーのPCが自分のセーブとは別の場所にワールドのコピーを保存します。オフ：ワールドはホストのPCにしかありません。</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>On: after each automatic save, every player's PC keeps a copy of the world, outside its own saves. Off: the world is on the host's PC only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_shared_tax</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>税金は最も名声の高いプレイヤーで計算</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Tax on the most famous player</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_shared_tax</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>オン：毎月の税金は、接続中のプレイヤーの中で最も高い名声で計算されます。オフ：ホストの名声で計算されます（ゲーム本来の動作）。</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>On: the monthly tax is computed on the highest fame among the connected players. Off: on the host's fame, as the game does.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
wip (compiled, never run, NOT to publish before the bench): soft recall, council 11 slice 1: when the host comes to a map a guest holds alone, the guest keeps its scene and becomes a client again in place instead of reloading the whole world; rule SoftRecall (23), unticked by default, every flow unchanged while it is off; falls back to the map alone, then to the world copy; plan and 18 points to check in dev/PLAN_retour_sur_place.md
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D292"/>
+  <dimension ref="A1:D294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5415,6 +5415,40 @@
         </is>
       </c>
     </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_soft_recall</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>ホストが来てもワールドを読み込み直さない（新機能）</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>No world reload when the host joins a player (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_soft_recall</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>オン：ホストが、プレイヤーが一人でいるマップに入っても、そのプレイヤーはその場に残り、ワールド全体を読み込み直しません。食い違いがあれば、これまでどおりワールドを読み込みます。オフ：そのたびにワールドを読み込み直します。</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>On: when the host walks onto the map a player is on alone, that player stays where it is and does not load the whole world again. Should anything not match, the world is loaded as before. Off: the world is loaded again each time.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
wip soft return, council 11 slice 2 (rule SoftRecall, unticked by default): a guest that walks to the host's map keeps its game and loads only that map; played on the bench for the first time: floors_suite --soft 6 floors, 0 whole-world copy (4 before the rule, 2 with slice 1 alone), 72/72: map sums equal, objects and moves seen both ways, bags unchanged, no duplicate uid
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -5423,12 +5423,12 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>ホストが来てもワールドを読み込み直さない（新機能）</t>
+          <t>ホストと合流してもワールドを読み込み直さない（新機能）</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>No world reload when the host joins a player (new)</t>
+          <t>No world reload when the host and a player meet again (new)</t>
         </is>
       </c>
     </row>
@@ -5440,12 +5440,12 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>オン：ホストが、プレイヤーが一人でいるマップに入っても、そのプレイヤーはその場に残り、ワールド全体を読み込み直しません。食い違いがあれば、これまでどおりワールドを読み込みます。オフ：そのたびにワールドを読み込み直します。</t>
+          <t>オン：ホストが、プレイヤーが一人でいるマップに入るとき、またはそのプレイヤーがホストのいるマップに入るとき、ワールド全体を読み込み直しません（その場に残るか、そのマップだけを読み込みます）。食い違いがあれば、これまでどおりワールドを読み込みます。オフ：そのたびにワールドを読み込み直します。</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>On: when the host walks onto the map a player is on alone, that player stays where it is and does not load the whole world again. Should anything not match, the world is loaded as before. Off: the world is loaded again each time.</t>
+          <t>On: when the host walks onto the map a player is on alone, or that player walks into the map the host is on, the player does not load the whole world again: it stays where it is, or loads that one map. Should anything not match, the world is loaded as before. Off: the world is loaded again each time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
wip (compiled, never run, NOT in 0.26.584, not reviewed): the mods of the world known and compared when hosting from the depot or joining (PublishMods, on: list in the lobby and the handshake, messages naming the mods), and fetched without subscribing then a restart and a return by itself (FetchMods, client side, off); depot_github_test 85/85; modlist_suite written, not run
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D294"/>
+  <dimension ref="A1:D310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5449,6 +5449,278 @@
         </is>
       </c>
     </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_publish_mods</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>ゲームのMod一覧を公開する</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Show the mods of the game to the players</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_publish_mods</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>オン：参加前（ゲーム一覧）と参加時にMod一覧が伝えられ、拒否された場合はどのModが違うかが名前で表示されます。デポから取ったワールドではデポの一覧（modlist.txt）を使います。オフ：何も伝えません。</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>On: the list of mods is known before joining (list of games) and when joining, and a player who is refused is told which mods differ, by name. For a world taken from a depot it is the depot's list (modlist.txt). Off: nothing is said.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_fetch_mods</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>ゲームのModを自動で取得する（新機能）</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Fetch the mods of the game by itself (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_desc_fetch_mods</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>オン：参加するゲームにあってここに無いワークショップModを、サブスクライブせずにダウンロードし、そのゲームのModだけでElinを1回再起動して自動で戻ります。次の起動で自分のMod一覧に戻ります。オフ：違うModの名前が表示されるだけです。</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>On: Workshop mods of the game you join that are missing here are downloaded without subscribing, Elin restarts once with exactly the mods of that game and comes back by itself. Your own mod list is back at the next start. Off: you are only told which mods differ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_lobby</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Mod {0} 個</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>{0} mods</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_lobby_missing</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Mod {0} 個、うち {1} 個がここにありません</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>{0} mods, {1} missing here</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_world</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>このワールドのModのうち {0} 個がここで読み込まれていません：{1}。一覧はログにあります。</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>{0} mods of this world are not loaded here: {1}. The list is in the log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_missing</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>ここに無いホストのMod（{0}）：{1}</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Mods of the host missing here ({0}): {1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_hand</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>手動で入れる必要があるMod（{0}）：{1}</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Mods to install by hand ({0}): {1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_extra</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>ホストに無いここのMod（{0}）：{1}</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Mods only here, not on the host ({0}): {1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_fetching</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>ゲームのModをダウンロード中 {0}/{1}：{2} {3}%（Escで中止）</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Downloading the mods of the game {0}/{1}: {2} {3}% (Esc to cancel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_fetch_failed</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>ゲームのModをダウンロードできませんでした。何も変更していません。</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>The mods of the game could not be downloaded. Nothing was changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_restart</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>ElinはゲームのModで再起動し、自動でゲームに戻ります。再起動しない場合は、Elinをもう一度起動してください。</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Elin restarts with the mods of the game and comes back to it by itself. If it does not start, start Elin again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_restart_manual</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Elinを閉じます。もう一度起動してください：ゲームのModで自動的にゲームへ戻ります。</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Elin closes. Start it again: it comes back to the game by itself, with its mods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_session</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>今回のElinはマルチプレイのゲームのModで動いています。次の起動で自分のMod一覧に戻ります。</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Elin runs with the mods of the multiplayer game this time. Your own mod list is back at the next start.</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>emp_ui_mods_session_locked</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>このセッション中はMod一覧を保存しません。次の起動で自分の一覧に戻ります。</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>The mod list is not saved during this session: your own is back at the next start of Elin.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(mods), compiled, never run: client setting KeepMods (off), Keep the mods of the game (subscribe on the Workshop). Ticked, the mods missing when joining are subscribed to and switched on in the player's own list instead of hidden in it: Elin still restarts once, then joining the same game again needs no restart, even after closing Elin (asked by the user after a real evening where a guest's Elin restarted at every start). The message of a session run says how to skip the restart. Texts in EN, JP, CN. Not in 0.26.605
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9510" yWindow="2685" windowWidth="31695" windowHeight="18195" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="General" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D310"/>
+  <dimension ref="A1:D312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5695,12 +5695,12 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>今回のElinはマルチプレイのゲームのModで動いています。次の起動で自分のMod一覧に戻ります。</t>
+          <t>今回のElinはマルチプレイのゲームのModで動いています。次の起動では自分のMod一覧に戻ります。この再起動を次回からなくすには、クライアント設定の「ゲームのModを残す」をオンにしてください。</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Elin runs with the mods of the multiplayer game this time. Your own mod list is back at the next start.</t>
+          <t>Elin runs with the mods of the multiplayer game this time. Your own mod list is back at the next start. To skip this restart next time, tick "Keep the mods of the game" in Client Settings.</t>
         </is>
       </c>
     </row>
@@ -5718,6 +5718,40 @@
       <c r="D310" t="inlineStr">
         <is>
           <t>The mod list is not saved during this session: your own is back at the next start of Elin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_keep_mods</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>ゲームのModを残す（ワークショップでサブスクライブ）</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Keep the mods of the game (subscribe on the Workshop)</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_desc_keep_mods</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>オン：参加したゲームのModをSteamアカウントでサブスクライブし、自分のMod一覧でも有効のままにします。最初の一回だけElinが再起動し、その後はElinを閉じても同じゲームに再起動なしで参加できます。やめるには、ワークショップでサブスクライブを解除してください。オフ：サブスクライブせずに取得し、Elinを起動するたびに最初の参加で再起動します。</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>On: your Steam account subscribes to the mods of the game you join and they stay on in your own mod list. Elin still restarts once, the first time; after that you join the same game again with no restart, even after closing Elin. To undo, unsubscribe on the Workshop. Off: they are fetched without subscribing and Elin restarts at the first join of every start.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: what a shop sells once per world is sold once per player (limited stock: skill books, recipes, a few merchants' weapons). The item in the merchant's chest keeps who bought how many; the game that keeps the shop lays the whole stack again when some leave for a player; at a restock the limited items are made again, so a world played before finds them back. oct10_suite l1 21/21 on two windows (Fiama), the whole suite 38/39 (the red was the test replayed in the same world, corrected, not replayed). Not played: travelling merchant, mod merchants, a map kept by a guest, the real click (drag). Audit of the other once-per-world things in dev/PLAN_une_fois_par_monde.md
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9510" yWindow="2685" windowWidth="31695" windowHeight="18195" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="General" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D316"/>
+  <dimension ref="A1:D317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5823,6 +5823,23 @@
         </is>
       </c>
     </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>emp_ui_limited_bought</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>それはもう買いました。</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>You already bought this one.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: a share for everyone (council 14, slice 1): what a story quest or a dialog gives is given to every other player of the world, at its feet when it is on the map, else as a parcel in its name in the base's mail; recipes, deeds and artifacts are not multiplied (the bag of holding is). New host checkbox 'Once per world = once per player' (session rule 25, on), which also covers the limited stock of shops. oct10_suite 58/58 (host completes the curry quest: same seeds for the guest in both games, nothing for a non-story drop, nothing with the checkbox off, a parcel for a guest away). Not played: a guest as the one who completes, a real dialog, three players. Not done: catching up a late player and worlds already played
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D317"/>
+  <dimension ref="A1:D320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5840,6 +5840,57 @@
         </is>
       </c>
     </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>emp_story_share</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>{0}の分け前</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>{0}'s share</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_once_per_player</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>一度きりのものを各プレイヤーに</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Once per world = once per player</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_once_per_player</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>オン：店の限定商品とストーリーの報酬を、各プレイヤーが一度ずつ得られます。オフ：最初のプレイヤーだけ（原作通り）。</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>On: what a shop sells only once and what the story gives (quest rewards, dialog gifts) go once to each player. Off: only the first player, as the game does.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Takeover R6: a former host that loads its world again joins the game that took it over
Lobby data EmpWorld / EmpHandover (Steam) and a local announce file (same machine); EmpAutoHost and
WorldHandover.Watch join the newer host as a guest instead of hosting a second world. Nothing is deleted.
Test: takeover_trio 16/16 (three windows, local port). By Steam between real PCs: not played.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D320"/>
+  <dimension ref="A1:D321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5891,6 +5891,23 @@
         </is>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>emp_takeover_rejoin</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>別のプレイヤーがこの世界を引き継ぎました。そのゲームに参加します…</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Another player took this world over. Joining its game…</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Une part pour chacun : le joueur qui recoit sa part le lit dans son journal
TellShare : MsgSayDelta a ce joueur seul, Msg.SayRaw chez l'host. oct10_suite s1 17/17 (invite present).
Pas joue : la ligne du colis, la ligne chez l'host. Texte dans la langue du jeu qui heberge.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D321"/>
+  <dimension ref="A1:D323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5908,6 +5908,40 @@
         </is>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>emp_story_share_got</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>物語の報酬の分け前を受け取った：{0}</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>You receive your share of what the story gave: {0}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>emp_story_share_mail</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>物語の報酬の分け前（{0}）が拠点の郵便受けに届く。</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Your share of what the story gave ({0}) is sent to the mail of the base.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Bouton « Prepare a bug report » : un zip des journaux du jeu et du mod sur le bureau
Helper/BugReport.cs, onglet Client Settings. Ni sauvegarde ni fichier de reglages. Joue par reflexion dans les
deux jeux (contenu des zips lu), bouton present dans l'onglet ; le clic n'est pas joue.
together_suite : note ce que disent les deux jeux si l'invite n'arrive pas a tuer le dernier monstre.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D323"/>
+  <dimension ref="A1:D327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5942,6 +5942,74 @@
         </is>
       </c>
     </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>emp_ui_report</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>不具合レポートを作成</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Prepare a bug report</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>emp_ui_report_desc</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>ゲームとModのログをまとめたzipをデスクトップに作成します（セーブデータや設定ファイルは含みません）。問題を報告するときに送ってください。</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Writes one zip on your desktop with the logs of the game and of the mod (no save, no settings file). Send it when you report a problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>emp_ui_report_done</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>レポートを作成しました：{0}</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Bug report written: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>emp_ui_report_failed</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>レポートを作成できませんでした。</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>The bug report could not be written.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Factures fantomes : le compteur des factures impayees est ramene aux factures qui existent
Avant la 0.26.652 une facture payee par un joueur seul ailleurs n'etait pas toujours comptee : le compteur du
monde restait au-dessus des factures existantes, sans rien a payer pour le faire descendre, avec 50 de karma en
moins chaque mois. ElinNetHostBills : ramene aux factures trouvees (sacs de tous les personnages, courrier,
banque, expedition, carte affichee), jamais releve ; une fois par monde au lancement, et par un bouton de
l'onglet de l'host. oct10_suite z1 4/4, clic du bouton joue (2 -> 0). t1 : drapeaux du banc remis a zero.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D327"/>
+  <dimension ref="A1:D331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6010,6 +6010,74 @@
         </is>
       </c>
     </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_bills</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>未払いの税金請求書：カウント {0}、実在 {1}（修復する）</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Unpaid tax bills: counted {0}, existing {1} (repair)</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_bills_desc</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>カウントが実在する請求書より多い場合（以前の不具合）、実在する数まで下げます。増えることはありません。</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>When the count is above the bills that exist (an old defect), it is brought down to them. It is never raised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_bills_done</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>支払えない請求書 {0} 件をカウントから外しました。</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>{0} bill(s) that nothing could pay were taken off the count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_bills_none</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>カウントは実在する請求書と一致しています。</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>The count matches the bills that exist.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tente amelioree a la cle : connue de tous les jeux ; un invite peut supprimer un de ses personnages
TentZoneDelta (855) : la cle change la zone de la tente, que rien ne transmettait. x5 rouge sans le correctif,
8/8 avec. Suppression d'un personnage depuis la liste de connexion (case host, textes 4 langues) ; x6 3/3
cote host, boites cote invite pas jouees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D331"/>
+  <dimension ref="A1:D336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6078,6 +6078,91 @@
         </is>
       </c>
     </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_delete</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>キャラクターを削除する</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Delete a character</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_delete_confirm</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>#1 を削除しますか？持ち物も一緒に消えます。仲間はこの世界に残ります。</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Delete #1? What it carries goes with it. Its companions stay in this world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_deleted</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>キャラクターを削除しました。</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>The character was deleted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_delete_chara</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>プレイヤーが自分のキャラクターを削除できる</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Players can delete their characters</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_delete_chara</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>キャラクター選択の一覧から（二度確認）。持ち物も消え、仲間は世界に残る。</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>From the list of characters (asked twice). What it carries goes too; its companions stay in the world.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reglages du monde : ceux de l'host, pour tous (WorldPrincipalDelta 858)
Conseil du 19 octobre : un invite qui changeait les reglages du monde (protection de la penalite de mort,
benediction du vide, mort definitive...) ne les changeait que dans son jeu, qui appliquait alors d'autres regles.
Maintenant la fenetre s'ouvre pour tous, mais chez un invite ses changements ne sont pas gardes (message
emp_world_setting_host, japonais/anglais/chinois) ; l'host envoie ses reglages a tous apres chaque changement
(a la connexion ils arrivent deja avec le monde).
Test settings2_suite p19 (fenetre ouverte par eval, un reglage bascule, fermee) : rouge sur l'ancien build (l'invite
gardait le sien), vert ; serie entiere 45/45. Relu (sonnet) : rien de bloquant.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D336"/>
+  <dimension ref="A1:D337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6163,6 +6163,23 @@
         </is>
       </c>
     </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>emp_world_setting_host</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>ワールド設定はホストが決めます。変更は保存されませんでした。</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>World settings are the host's: your changes were not kept.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Texts: drop the old trade window's texts, plainer disconnect message
The ten texts of the old list-style trade window are unused since the trade moved to the game's container windows.
"Disconnected: client cancelled" now reads "Disconnected: you cancelled the connection."

Checked in game: the new text loads; trade_suite 138/138 on the world copy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D324"/>
+  <dimension ref="A1:D314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Disconnected: client cancelled</t>
+          <t>Disconnected: you cancelled the connection.</t>
         </is>
       </c>
     </row>
@@ -2365,1523 +2365,1370 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>emp_ui_trade</t>
+          <t>emp_trade_invite</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>取引</t>
+          <t>{0} があなたと取引したがっています</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Trade</t>
+          <t>{0} wants to trade with you</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>emp_trade_invite</t>
+          <t>emp_trade_gold</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>{0} があなたと取引したがっています</t>
+          <t>金貨: {0}</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>{0} wants to trade with you</t>
+          <t>Gold: {0}</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>emp_trade_you_offer</t>
+          <t>emp_trade_confirm</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>あなたの提示</t>
+          <t>確定する</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>You offer</t>
+          <t>Validate</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>emp_trade_they_offer</t>
+          <t>emp_trade_cancel</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>{0} の提示</t>
+          <t>キャンセル</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>{0} offers</t>
+          <t>Cancel</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>emp_trade_nothing</t>
+          <t>emp_trade_you_ready</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>（まだなし）</t>
+          <t>確定済み</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>(nothing yet)</t>
+          <t>Validated</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>emp_trade_add</t>
+          <t>emp_trade_they_ready</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>アイテムを追加</t>
+          <t>確定済み</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Add an item</t>
+          <t>validated</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>emp_trade_gold</t>
+          <t>emp_trade_they_wait</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>金貨: {0}</t>
+          <t>まだ確定していない</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Gold: {0}</t>
+          <t>not validated yet</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>emp_trade_clear</t>
+          <t>emp_trade_howmuch</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>すべて取り下げる</t>
+          <t>金貨はいくら？</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Take everything back</t>
+          <t>How much gold?</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>emp_trade_confirm</t>
+          <t>emp_trade_done</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>確定する</t>
+          <t>取引が完了しました</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Validate</t>
+          <t>Trade done</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>emp_trade_cancel</t>
+          <t>emp_trade_cancelled</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>キャンセル</t>
+          <t>取引は中止されました</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>Trade cancelled</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>emp_trade_you_ready</t>
+          <t>emp_trade_invalid</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>確定済み</t>
+          <t>取引は中止されました：渡すはずの物がもうありません</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Validated</t>
+          <t>Trade cancelled: an item is gone.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>emp_trade_you_wait</t>
+          <t>emp_trade_far</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>あなたは未確認です</t>
+          <t>取引は中止されました：離れすぎです</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>You have not confirmed</t>
+          <t>Trade cancelled: you are too far apart.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>emp_trade_they_ready</t>
+          <t>emp_trade_busy</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>確定済み</t>
+          <t>そのプレイヤーは取引中です</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>validated</t>
+          <t>That player is already trading.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>emp_trade_they_wait</t>
+          <t>emp_ui_sv_note_live</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>まだ確定していない</t>
+          <t>これはホストのルールです。変更はすぐ全員に反映されます。</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>not validated yet</t>
+          <t>These are the host's rules. Changes apply to everyone at once.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>emp_trade_pick</t>
+          <t>emp_ui_sv_sec_players</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>どのアイテム？</t>
+          <t>プレイヤーと移動</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Which item?</t>
+          <t>Players and travel</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>emp_trade_howmany</t>
+          <t>emp_ui_sv_sec_own</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>何個？</t>
+          <t>プレイヤーごとのもの</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>How many?</t>
+          <t>One for each player</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>emp_trade_howmuch</t>
+          <t>emp_ui_sv_sec_time</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>金貨はいくら？</t>
+          <t>時間と戦闘</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>How much gold?</t>
+          <t>Time and combat</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>emp_trade_done</t>
+          <t>emp_ui_sv_sec_checks</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>取引が完了しました</t>
+          <t>参加チェック</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Trade done</t>
+          <t>Joining checks</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>emp_trade_cancelled</t>
+          <t>emp_ui_sv_desc_choose_chara</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>取引は中止されました</t>
+          <t>参加するとき、この世界での自分のキャラを選ぶか、新しく作ります。</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Trade cancelled</t>
+          <t>Joining players pick one of their characters in this world, or make a new one.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>emp_trade_invalid</t>
+          <t>emp_ui_sv_desc_independent_travel</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>取引は中止されました：渡すはずの物がもうありません</t>
+          <t>好きな場所へ、ひとりでも仲間とでも行けます。オフ：全員がホストについていきます。</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Trade cancelled: an item is gone.</t>
+          <t>Players can go anywhere, alone or together. Unticked, everyone follows the host.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>emp_trade_far</t>
+          <t>emp_ui_sv_desc_personal_quests</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>取引は中止されました：離れすぎです</t>
+          <t>依頼は1人5件ずつ。報酬・名声・カルマも別々です。ストーリーは共通です。</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Trade cancelled: you are too far apart.</t>
+          <t>Each player gets 5 quests, with their own reward, fame and karma. Story quests stay shared.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>emp_trade_busy</t>
+          <t>emp_ui_sv_desc_player_shipping</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>そのプレイヤーは取引中です</t>
+          <t>出荷箱のお金は、入れたプレイヤーのものに。オフ：すべてホストへ。</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>That player is already trading.</t>
+          <t>Shipping money goes to the player who put the item in. Unticked, the host gets it all.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>emp_ui_sv_note_live</t>
+          <t>emp_ui_sv_desc_player_trade</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>これはホストのルールです。変更はすぐ全員に反映されます。</t>
+          <t>ほかのプレイヤーをクリックすると、アイテムやお金を取引できます。双方の確認が必要です。</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>These are the host's rules. Changes apply to everyone at once.</t>
+          <t>Click another player to trade items and gold. Both must confirm.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>emp_ui_sv_sec_players</t>
+          <t>emp_ui_sv_desc_combat_time</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>プレイヤーと移動</t>
+          <t>モンスターは、戦っているプレイヤーが動くときに動きます。誰も待ちません。ターン制より優先されます。</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Players and travel</t>
+          <t>A monster acts when the player it fights acts. Nobody waits. This comes before turn-based combat.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>emp_ui_sv_sec_own</t>
+          <t>emp_ui_sv_desc_turn_combat</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>プレイヤーごとのもの</t>
+          <t>戦闘中、プレイヤーは順番に動きます。「戦闘はプレイヤーごとの時間で」がオンのときは無効です。</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>One for each player</t>
+          <t>In a fight, players take turns. Does nothing while "Combat at each player's pace" is ticked.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>emp_ui_sv_sec_time</t>
+          <t>emp_ui_sv_desc_shared_speed</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>時間と戦闘</t>
+          <t>全員が平均の速さで動きます。オフ：それぞれの速さのまま。</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Time and combat</t>
+          <t>Everyone moves at the average speed. Unticked, each keeps their own.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>emp_ui_sv_sec_checks</t>
+          <t>emp_ui_sv_desc_validation</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>参加チェック</t>
+          <t>参加するプレイヤーのゲームが、ホストと同じであるべきもの。「なし」：誰でも。「すべて」：データとMODが同じ。</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Joining checks</t>
+          <t>What a joining player's game must share with yours. None: anyone. All: same data and mods.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_choose_chara</t>
+          <t>emp_ui_sv_cfg_player_clock</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>参加するとき、この世界での自分のキャラを選ぶか、新しく作ります。</t>
+          <t>プレイヤーごとの時間で動く</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Joining players pick one of their characters in this world, or make a new one.</t>
+          <t>Each player moves at their own pace</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_independent_travel</t>
+          <t>emp_ui_sv_desc_player_clock</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>好きな場所へ、ひとりでも仲間とでも行けます。オフ：全員がホストについていきます。</t>
+          <t>ゲストも、ホストと同じなめらかさで動けます。上の項目がオンのときに使えます。</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Players can go anywhere, alone or together. Unticked, everyone follows the host.</t>
+          <t>Guests move as smoothly as the host. Needs the option above.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_personal_quests</t>
+          <t>emp_ui_sv_cfg_step_pace</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>依頼は1人5件ずつ。報酬・名声・カルマも別々です。ストーリーは共通です。</t>
+          <t>全員がひとり用の速さで歩く</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Each player gets 5 quests, with their own reward, fame and karma. Story quests stay shared.</t>
+          <t>Everyone walks as in a solo game</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_player_shipping</t>
+          <t>emp_ui_sv_desc_step_pace</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>出荷箱のお金は、入れたプレイヤーのものに。オフ：すべてホストへ。</t>
+          <t>歩く速さが、ほかのプレイヤーの速さに左右されません。戦闘では速さが効きます。「戦闘はプレイヤーごとの時間で」が必要です。</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Shipping money goes to the player who put the item in. Unticked, the host gets it all.</t>
+          <t>A step no longer depends on the others' speed. Speed still counts in a fight. Needs "Combat at each player's pace".</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_player_trade</t>
+          <t>emp_ui_sv_cfg_import_chara</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ほかのプレイヤーをクリックすると、アイテムやお金を取引できます。双方の確認が必要です。</t>
+          <t>自分のセーブのキャラを連れてこられる</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Click another player to trade items and gold. Both must confirm.</t>
+          <t>Players can bring a character from their saves</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_combat_time</t>
+          <t>emp_ui_sv_desc_import_chara</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>モンスターは、戦っているプレイヤーが動くときに動きます。誰も待ちません。ターン制より優先されます。</t>
+          <t>キャラ本人、装備、バッグ、お金、名声とカルマ。仲間、拠点、依頼、銀行は含みません。セーブは読むだけで、変更されません。</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>A monster acts when the player it fights acts. Nobody waits. This comes before turn-based combat.</t>
+          <t>The character, gear, bag, gold, fame and karma. Not companions, base, quests or bank. The save is never changed.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_turn_combat</t>
+          <t>emp_ui_chara_import</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>戦闘中、プレイヤーは順番に動きます。「戦闘はプレイヤーごとの時間で」がオンのときは無効です。</t>
+          <t>自分のセーブのキャラ…</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>In a fight, players take turns. Does nothing while "Combat at each player's pace" is ticked.</t>
+          <t>A character from my saves…</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_shared_speed</t>
+          <t>emp_ui_chara_import_pick</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>全員が平均の速さで動きます。オフ：それぞれの速さのまま。</t>
+          <t>どのセーブのキャラを連れてきますか？（セーブは変更されません）</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Everyone moves at the average speed. Unticked, each keeps their own.</t>
+          <t>Which save? It will not be changed.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_validation</t>
+          <t>emp_ui_chara_import_back</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>参加するプレイヤーのゲームが、ホストと同じであるべきもの。「なし」：誰でも。「すべて」：データとMODが同じ。</t>
+          <t>戻る</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>What a joining player's game must share with yours. None: anyone. All: same data and mods.</t>
+          <t>Back</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_player_clock</t>
+          <t>emp_ui_chara_import_none</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>プレイヤーごとの時間で動く</t>
+          <t>読み込めるセーブが見つかりません。</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Each player moves at their own pace</t>
+          <t>No save was found.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_player_clock</t>
+          <t>emp_ui_chara_import_fail</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>ゲストも、ホストと同じなめらかさで動けます。上の項目がオンのときに使えます。</t>
+          <t>そのキャラを連れてこられませんでした。</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Guests move as smoothly as the host. Needs the option above.</t>
+          <t>That character can't be brought.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_step_pace</t>
+          <t>emp_ui_chara_import_twice</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>全員がひとり用の速さで歩く</t>
+          <t>そのセーブのキャラは、すでにこの世界にいます。</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Everyone walks as in a solo game</t>
+          <t>That character is already in this world.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_step_pace</t>
+          <t>emp_ui_sv_cfg_world_time</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>歩く速さが、ほかのプレイヤーの速さに左右されません。戦闘では速さが効きます。「戦闘はプレイヤーごとの時間で」が必要です。</t>
+          <t>世界で日付をひとつにする</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>A step no longer depends on the others' speed. Speed still counts in a fight. Needs "Combat at each player's pace".</t>
+          <t>One date for the whole world</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_import_chara</t>
+          <t>emp_ui_sv_desc_world_time</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>自分のセーブのキャラを連れてこられる</t>
+          <t>別のマップにひとりでいるプレイヤーの時間も、全員に反映されます。いちばん進んだ日付が世界の日付です。オフ：ホストの日付のみ。</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Players can bring a character from their saves</t>
+          <t>Time spent alone on another map counts for everyone. The latest date is the world's. Unticked, only the host's date counts.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_import_chara</t>
+          <t>emp_ui_sv_cfg_world_keeper</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>キャラ本人、装備、バッグ、お金、名声とカルマ。仲間、拠点、依頼、銀行は含みません。セーブは読むだけで、変更されません。</t>
+          <t>時間の影響を一度だけ起こす</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>The character, gear, bag, gold, fame and karma. Not companions, base, quests or bank. The save is never changed.</t>
+          <t>Time affects the world only once</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import</t>
+          <t>emp_ui_sv_desc_world_keeper</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>自分のセーブのキャラ…</t>
+          <t>天気、依頼の期限切れ、税金、給料、手紙は、ひとりのゲームだけが処理します。オフ：マップを持つ全員が処理します。</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>A character from my saves…</t>
+          <t>Weather, expired quests, taxes, salaries and letters are handled by one player only. Unticked, every player holding a map handles them.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_pick</t>
+          <t>emp_ui_depot_take</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>どのセーブのキャラを連れてきますか？（セーブは変更されません）</t>
+          <t>デポから世界を取り出してホストする</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Which save? It will not be changed.</t>
+          <t>Take the world from the depot and host it</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_back</t>
+          <t>emp_ui_depot_put</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>戻る</t>
+          <t>このセーブをデポに置く</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Back</t>
+          <t>Put this save in the depot</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_none</t>
+          <t>emp_ui_depot_held</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>読み込めるセーブが見つかりません。</t>
+          <t>{0} が世界をホスト中です。Steam で参加してください。招待してもらうか、Steam のフレンド一覧で「ゲームに参加」を選びます。抜けた直後なら、3分ほど待ってください。</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>No save was found.</t>
+          <t>{0} is hosting the world. Join through Steam: ask for an invite, or use "Join Game" on their name in your friends list. If they just left, wait up to 3 minutes.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_fail</t>
+          <t>emp_ui_depot_empty</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>そのキャラを連れてこられませんでした。</t>
+          <t>デポにはまだ世界がありません。ゲームを始めるかロードして、このパネルをもう一度開き、ロビーのタブで「このセーブをデポに置く」を選んでください。</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>That character can't be brought.</t>
+          <t>The depot has no world yet. Start or load a game, then open this panel again and use "Put this save in the depot" in the Lobby tab.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>emp_ui_chara_import_twice</t>
+          <t>emp_ui_depot_fail</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>そのセーブのキャラは、すでにこの世界にいます。</t>
+          <t>デポに接続できませんでした。</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>That character is already in this world.</t>
+          <t>Could not reach the depot.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_world_time</t>
+          <t>emp_ui_depot_put_done</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>世界で日付をひとつにする</t>
+          <t>この世界をデポに置きました。ゲームはそこから読み込み直します。これからのセーブはすべてデポに送られます。</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>One date for the whole world</t>
+          <t>The world is now in the depot. The game loads it again from there. From now on, every save goes to the depot.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_world_time</t>
+          <t>emp_ui_depot_folder</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>別のマップにひとりでいるプレイヤーの時間も、全員に反映されます。いちばん進んだ日付が世界の日付です。オフ：ホストの日付のみ。</t>
+          <t>デポ</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Time spent alone on another map counts for everyone. The latest date is the world's. Unticked, only the host's date counts.</t>
+          <t>Depot</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_world_keeper</t>
+          <t>emp_ui_depot_folder_ask</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>時間の影響を一度だけ起こす</t>
+          <t>セーブの置き場所：Elin Together Server のアドレス（ホスト:55557）、全員が使えるフォルダ、または非公開の GitHub リポジトリ（github:ユーザー/リポジトリ）。空欄なら使いません</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Time affects the world only once</t>
+          <t>Where the world is kept: the address of Elin Together Server (host:55557), a folder everyone can reach, or a private GitHub repository (github:owner/repository). Leave empty for none.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_world_keeper</t>
+          <t>emp_ui_join_address</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>天気、依頼の期限切れ、税金、給料、手紙は、ひとりのゲームだけが処理します。オフ：マップを持つ全員が処理します。</t>
+          <t>アドレスで参加</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Weather, expired quests, taxes, salaries and letters are handled by one player only. Unticked, every player holding a map handles them.</t>
+          <t>Join by address</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>emp_ui_depot_take</t>
+          <t>emp_ui_join_address_ask</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>デポから世界を取り出してホストする</t>
+          <t>サーバーのアドレス（ホスト:ポート。Elin ありは 55556、なしは 55557）</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Take the world from the depot and host it</t>
+          <t>Server address (host:port). The port is 55556 with Elin, 55557 without.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>emp_ui_depot_put</t>
+          <t>emp_ui_depot_password</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>このセーブをデポに置く</t>
+          <t>デポのキー</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Put this save in the depot</t>
+          <t>Depot key</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>emp_ui_depot_held</t>
+          <t>emp_ui_depot_password_ask</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>{0} が世界をホスト中です。Steam で参加してください。招待してもらうか、Steam のフレンド一覧で「ゲームに参加」を選びます。抜けた直後なら、3分ほど待ってください。</t>
+          <t>デポのパスワード（設定した場合）、または GitHub のアクセスキー。キーは二度と表示されません。変えないなら空欄のままにしてください</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>{0} is hosting the world. Join through Steam: ask for an invite, or use "Join Game" on their name in your friends list. If they just left, wait up to 3 minutes.</t>
+          <t>The depot password (if one was set), or the GitHub key. A key is never shown again. Leave empty to keep it.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>emp_ui_depot_empty</t>
+          <t>emp_ui_timeout</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>デポにはまだ世界がありません。ゲームを始めるかロードして、このパネルをもう一度開き、ロビーのタブで「このセーブをデポに置く」を選んでください。</t>
+          <t>サーバーが応答しません。アドレスとポートを確認してください。</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>The depot has no world yet. Start or load a game, then open this panel again and use "Put this save in the depot" in the Lobby tab.</t>
+          <t>The server does not answer. Check the address and the port.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>emp_ui_depot_fail</t>
+          <t>emp_ui_depot_password_wrong</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>デポに接続できませんでした。</t>
+          <t>サーバーにパスワードを断られました。クライアント設定の「デポのキー」で設定してください。</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Could not reach the depot.</t>
+          <t>The server refused the password. Set it in Client Settings, under "Depot key".</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>emp_ui_depot_put_done</t>
+          <t>emp_ui_depot_lost</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>この世界をデポに置きました。ゲームはそこから読み込み直します。これからのセーブはすべてデポに送られます。</t>
+          <t>接続が切れている間に、{0} がデポの世界を引き継ぎました。これ以降のプレイはデポに届きません。タイトルに戻って、その人のゲームに参加してください。</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>The world is now in the depot. The game loads it again from there. From now on, every save goes to the depot.</t>
+          <t>{0} took over the world while you were cut off. What you play now won't reach the depot. Go back to the title screen and join them.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>emp_ui_depot_folder</t>
+          <t>emp_ui_depot_unsaved</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>デポ</t>
+          <t>デポにセーブが届きませんでした。このPCに残してあり、次のセーブでもう一度送ります。</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Depot</t>
+          <t>The save didn't reach the depot. It is kept on this PC and sent again at the next save.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>emp_ui_depot_folder_ask</t>
+          <t>emp_ui_depot_unsent</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>セーブの置き場所：Elin Together Server のアドレス（ホスト:55557）、全員が使えるフォルダ、または非公開の GitHub リポジトリ（github:ユーザー/リポジトリ）。空欄なら使いません</t>
+          <t>前回の最後のセーブが、デポに届いていません。今送りますか？（はい：デポにある世界は別に取っておきます。いいえ：このセーブは捨てて、デポの世界を使います。）</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Where the world is kept: the address of Elin Together Server (host:55557), a folder everyone can reach, or a private GitHub repository (github:owner/repository). Leave empty for none.</t>
+          <t>Your last save never reached the depot. Send it now? Yes keeps the depot's world aside. No drops your save and uses the depot's world.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>emp_ui_join_address</t>
+          <t>emp_quest_follow_ask</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>アドレスで参加</t>
+          <t>{0} が依頼に出かけます。ついていきますか？報酬は {0} のものになります。</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Join by address</t>
+          <t>{0} is leaving on a quest. Go along? The reward goes to {0}.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>emp_ui_join_address_ask</t>
+          <t>emp_quest_follow_declined</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>サーバーのアドレス（ホスト:ポート。Elin ありは 55556、なしは 55557）</t>
+          <t>{0} は同行を断りました。</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Server address (host:port). The port is 55556 with Elin, 55557 without.</t>
+          <t>{0} won't come along.</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>emp_ui_depot_password</t>
+          <t>emp_quest_follow_no_answer</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>デポのキー</t>
+          <t>{0} から返事がありません。</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Depot key</t>
+          <t>{0} didn't answer.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>emp_ui_depot_password_ask</t>
+          <t>emp_quest_follow_asked</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>デポのパスワード（設定した場合）、または GitHub のアクセスキー。キーは二度と表示されません。変えないなら空欄のままにしてください</t>
+          <t>{0} に同行を頼んでいます…</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>The depot password (if one was set), or the GitHub key. A key is never shown again. Leave empty to keep it.</t>
+          <t>Asking {0} to come along...</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>emp_ui_timeout</t>
+          <t>emp_base_host_only</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>サーバーが応答しません。アドレスとポートを確認してください。</t>
+          <t>今はホストだけができます。</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>The server does not answer. Check the address and the port.</t>
+          <t>Only the host can do this for now.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>emp_ui_depot_password_wrong</t>
+          <t>emp_trade_equipped</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>サーバーにパスワードを断られました。クライアント設定の「デポのキー」で設定してください。</t>
+          <t>取引は中止されました：渡す物が装備中です</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>The server refused the password. Set it in Client Settings, under "Depot key".</t>
+          <t>Trade cancelled: an item is equipped.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>emp_ui_depot_lost</t>
+          <t>emp_trade_nodrop</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>接続が切れている間に、{0} がデポの世界を引き継ぎました。これ以降のプレイはデポに届きません。タイトルに戻って、その人のゲームに参加してください。</t>
+          <t>取引は中止されました：捨てられない物、渡せない物があります</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>{0} took over the world while you were cut off. What you play now won't reach the depot. Go back to the title screen and join them.</t>
+          <t>Trade cancelled: an item can't be given away.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>emp_ui_depot_unsaved</t>
+          <t>emp_trade_npcprop</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>デポにセーブが届きませんでした。このPCに残してあり、次のセーブでもう一度送ります。</t>
+          <t>取引は中止されました：NPCの持ち物が含まれています</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>The save didn't reach the depot. It is kept on this PC and sent again at the next save.</t>
+          <t>Trade cancelled: an item belongs to an NPC.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>emp_ui_depot_unsent</t>
+          <t>emp_trade_gifted</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>前回の最後のセーブが、デポに届いていません。今送りますか？（はい：デポにある世界は別に取っておきます。いいえ：このセーブは捨てて、デポの世界を使います。）</t>
+          <t>取引は中止されました：贈り物は取引できません</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Your last save never reached the depot. Send it now? Yes keeps the depot's world aside. No drops your save and uses the depot's world.</t>
+          <t>Trade cancelled: a gift can't be traded.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>emp_quest_follow_ask</t>
+          <t>emp_trade_bound</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>{0} が依頼に出かけます。ついていきますか？報酬は {0} のものになります。</t>
+          <t>取引は中止されました：キャラに結びついた物があります</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>{0} is leaving on a quest. Go along? The reward goes to {0}.</t>
+          <t>Trade cancelled: an item is bound to a character.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>emp_quest_follow_declined</t>
+          <t>emp_trade_full</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>{0} は同行を断りました。</t>
+          <t>取引は中止されました：バッグの空きが足りません</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>{0} won't come along.</t>
+          <t>Trade cancelled: a bag is full.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>emp_quest_follow_no_answer</t>
+          <t>emp_travel_recalled_by</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>{0} から返事がありません。</t>
+          <t>{@Peer} がここに来ます。合流のため画面を読み込み直します…</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>{0} didn't answer.</t>
+          <t>{@Peer} is coming here. The screen reloads to join them…</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>emp_quest_follow_asked</t>
+          <t>emp_ui_thing_gone</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>{0} に同行を頼んでいます…</t>
+          <t>遅かった：ほかの人が先に取りました</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Asking {0} to come along...</t>
+          <t>Too late. Someone else took it.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>emp_base_host_only</t>
+          <t>emp_base_refused</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>今はホストだけができます。</t>
+          <t>ホストに断られました：拠点か所持金では払えません。</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Only the host can do this for now.</t>
+          <t>The host refused. The base or your purse can't pay for this.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>emp_trade_equipped</t>
+          <t>emp_base_pending</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>取引は中止されました：渡す物が装備中です</t>
+          <t>前の頼みが、まだホストの返事待ちです。</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Trade cancelled: an item is equipped.</t>
+          <t>Your last request is still waiting for the host.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>emp_trade_nodrop</t>
+          <t>emp_game_version_differs</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>取引は中止されました：捨てられない物、渡せない物があります</t>
+          <t>{0} の Elin はバージョンが違います（{1}、自分は {2}）。接続はできます。問題が起きたら同じバージョンにしてください。</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Trade cancelled: an item can't be given away.</t>
+          <t>{0} has another version of Elin ({1}, yours is {2}). You can still join. If something goes wrong, use the same version.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>emp_trade_npcprop</t>
+          <t>emp_ui_sv_cfg_same_game_version</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>取引は中止されました：NPCの持ち物が含まれています</t>
+          <t>同じ Elin のバージョンを必須にする</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Trade cancelled: an item belongs to an NPC.</t>
+          <t>Require the same Elin version</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>emp_trade_gifted</t>
+          <t>emp_ui_sv_desc_same_game_version</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>取引は中止されました：贈り物は取引できません</t>
+          <t>Elin のバージョンが違うプレイヤーは入れません。オフ：警告つきで入れます。MODのバージョンは常に同じである必要があります。</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Trade cancelled: a gift can't be traded.</t>
+          <t>Players with another Elin version can't join. Unticked, they join with a warning. The mod version must always match.</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>emp_trade_bound</t>
+          <t>emp_ui_sv_cfg_guest_build</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>取引は中止されました：キャラに結びついた物があります</t>
+          <t>ほかのプレイヤーも建築できる</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Trade cancelled: an item is bound to a character.</t>
+          <t>Other players can build</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>emp_trade_full</t>
+          <t>emp_ui_sv_desc_guest_build</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>取引は中止されました：バッグの空きが足りません</t>
+          <t>拠点の建築モード（床、壁、家具、採掘、伐採）を使えます。お金と素材は本人が払います。オフ：建築できるのはホストだけ。</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Trade cancelled: a bag is full.</t>
+          <t>Others can use build mode in the base: floors, walls, furniture, mining, cutting. They pay the gold and materials. Unticked, only the host builds.</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>emp_travel_recalled_by</t>
+          <t>emp_ui_depot_gh_help</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
-        <is>
-          <t>{@Peer} がここに来ます。合流のため画面を読み込み直します…</t>
-        </is>
-      </c>
-      <c r="D194" t="inlineStr">
-        <is>
-          <t>{@Peer} is coming here. The screen reloads to join them…</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>emp_ui_thing_gone</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>遅かった：ほかの人が先に取りました</t>
-        </is>
-      </c>
-      <c r="D195" t="inlineStr">
-        <is>
-          <t>Too late. Someone else took it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>emp_base_refused</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>ホストに断られました：拠点か所持金では払えません。</t>
-        </is>
-      </c>
-      <c r="D196" t="inlineStr">
-        <is>
-          <t>The host refused. The base or your purse can't pay for this.</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>emp_base_pending</t>
-        </is>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>前の頼みが、まだホストの返事待ちです。</t>
-        </is>
-      </c>
-      <c r="D197" t="inlineStr">
-        <is>
-          <t>Your last request is still waiting for the host.</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>emp_game_version_differs</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>{0} の Elin はバージョンが違います（{1}、自分は {2}）。接続はできます。問題が起きたら同じバージョンにしてください。</t>
-        </is>
-      </c>
-      <c r="D198" t="inlineStr">
-        <is>
-          <t>{0} has another version of Elin ({1}, yours is {2}). You can still join. If something goes wrong, use the same version.</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>emp_ui_sv_cfg_same_game_version</t>
-        </is>
-      </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>同じ Elin のバージョンを必須にする</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr">
-        <is>
-          <t>Require the same Elin version</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>emp_ui_sv_desc_same_game_version</t>
-        </is>
-      </c>
-      <c r="C200" t="inlineStr">
-        <is>
-          <t>Elin のバージョンが違うプレイヤーは入れません。オフ：警告つきで入れます。MODのバージョンは常に同じである必要があります。</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>Players with another Elin version can't join. Unticked, they join with a warning. The mod version must always match.</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>emp_ui_sv_cfg_guest_build</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>ほかのプレイヤーも建築できる</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>Other players can build</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>emp_ui_sv_desc_guest_build</t>
-        </is>
-      </c>
-      <c r="C202" t="inlineStr">
-        <is>
-          <t>拠点の建築モード（床、壁、家具、採掘、伐採）を使えます。お金と素材は本人が払います。オフ：建築できるのはホストだけ。</t>
-        </is>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>Others can use build mode in the base: floors, walls, furniture, mining, cutting. They pay the gold and materials. Unticked, only the host builds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>emp_ui_depot_gh_help</t>
-        </is>
-      </c>
-      <c r="C203" t="inlineStr">
         <is>
           <t>非公開の GitHub リポジトリを、デポにできます。サーバーも共有フォルダも要らず、友達に GitHub アカウントも要りません。
 1. github.com で、この世界専用の空の非公開リポジトリを作ります。
@@ -3890,7 +3737,7 @@
 4. 同じ2行を友達に送ります。友達もここに入力します。キーで開けるのはこのリポジトリだけです。</t>
         </is>
       </c>
-      <c r="D203" t="inlineStr">
+      <c r="D194" t="inlineStr">
         <is>
           <t>A private GitHub repository can be the depot. No server, no shared folder, and your friends need no GitHub account.
 1. On github.com, create an empty private repository just for this world.
@@ -3900,2058 +3747,2041 @@
         </is>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_key</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>GitHub にアクセスキーを断られました。期限切れでないか、このリポジトリを含み「Contents: Read and write」であるかを確認して、クライアント設定でもう一度貼ってください。</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>GitHub refused the key. Check that it hasn't expired and covers this repository with "Contents: Read and write", then paste it again in Client Settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_missing</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>GitHub でこのリポジトリが見つかりません。クライアント設定で名前（github:ユーザー/リポジトリ）を確認し、アクセスキーがそれを含んでいるか確認してください。</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>GitHub can't find the repository. Check its name (github:owner/repository) in Client Settings, and that your key covers it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_public</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>この GitHub リポジトリは公開です。世界とその履歴が誰にでも見えてしまいます。非公開に変えて（Settings、Danger Zone、Change visibility）、もう一度試してください。</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>This GitHub repository is public. Everyone could see your world and its history. Make it private (Settings, Danger Zone, Change visibility), then try again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_big</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>この世界は20MBを超えていて、GitHub には大きすぎます。Elin Together Server か共有フォルダを使ってください。セーブはこのPCに残っています。</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>This world is over 20 MB, too big for GitHub. Use Elin Together Server or a shared folder. The save stays on this PC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_changed</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>接続が切れている間に、別の人が世界をホストしてセーブしました。あなたのセーブはこのPCに残り、これ以上デポに送られません。タイトルに戻って、世界を取り直してください。</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Someone else hosted the world and saved while you were cut off. Your saves stay on this PC and no longer reach the depot. Go back to the title screen and take the world again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>emp_ui_depot_gh_down</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>GitHub が応答しません。接続を確認して、少し待ってからもう一度試してください。</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>GitHub does not answer. Check your connection and try again in a moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_player_kill</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>プレイヤー同士で倒せる</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Players can kill each other</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_player_kill</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>プレイヤーや仲間の攻撃で、ほかのプレイヤーを倒せます。オフ：致命傷でもHP0で生き残ります。</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Players and their companions can kill other players. Unticked, a deadly blow leaves them alive at 0 HP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_host_manages_base</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>拠点を管理できるのはホストだけ</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Only the host manages the base</t>
+        </is>
+      </c>
+    </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_key</t>
+          <t>emp_ui_sv_desc_host_manages_base</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>GitHub にアクセスキーを断られました。期限切れでないか、このリポジトリを含み「Contents: Read and write」であるかを確認して、クライアント設定でもう一度貼ってください。</t>
+          <t>ほかのプレイヤーの拠点操作（研究、炉の技能、方針、名前、設定、住人、建築）は断られます。オフ：全員がホストと同じように管理できます。拠点を完全に手放せるのは常にホストだけです。</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>GitHub refused the key. Check that it hasn't expired and covers this repository with "Contents: Read and write", then paste it again in Client Settings.</t>
+          <t>Others can't change the base: research, hearth skills, policies, names, settings, residents, build mode. Unticked, all can. Only the host can give up the base for good.</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_missing</t>
+          <t>emp_ui_sv_cfg_duels</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>GitHub でこのリポジトリが見つかりません。クライアント設定で名前（github:ユーザー/リポジトリ）を確認し、アクセスキーがそれを含んでいるか確認してください。</t>
+          <t>プレイヤー同士の決闘</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>GitHub can't find the repository. Check its name (github:owner/repository) in Client Settings, and that your key covers it.</t>
+          <t>Duels between players</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_public</t>
+          <t>emp_ui_sv_desc_duels</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>この GitHub リポジトリは公開です。世界とその履歴が誰にでも見えてしまいます。非公開に変えて（Settings、Danger Zone、Change visibility）、もう一度試してください。</t>
+          <t>相手のキャラのメニューから決闘を申し込めます。誰も死なず、終わると全員回復し、何も失いません。</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>This GitHub repository is public. Everyone could see your world and its history. Make it private (Settings, Danger Zone, Change visibility), then try again.</t>
+          <t>Challenge another player from the menu on their character. Nobody dies, both are healed and nothing is lost.</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_big</t>
+          <t>emp_act_duel</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>この世界は20MBを超えていて、GitHub には大きすぎます。Elin Together Server か共有フォルダを使ってください。セーブはこのPCに残っています。</t>
+          <t>決闘を申し込む</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>This world is over 20 MB, too big for GitHub. Use Elin Together Server or a shared folder. The save stays on this PC.</t>
+          <t>Challenge to a duel</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_changed</t>
+          <t>emp_duel_invite</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>接続が切れている間に、別の人が世界をホストしてセーブしました。あなたのセーブはこのPCに残り、これ以上デポに送られません。タイトルに戻って、世界を取り直してください。</t>
+          <t>{0}が決闘を申し込んできた。誰も死なないが、使った物は戻らない。受けますか？</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Someone else hosted the world and saved while you were cut off. Your saves stay on this PC and no longer reach the depot. Go back to the title screen and take the world again.</t>
+          <t>{0} challenges you to a duel. Nobody dies, but what you use up stays used. Accept?</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>emp_ui_depot_gh_down</t>
+          <t>emp_duel_asked</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>GitHub が応答しません。接続を確認して、少し待ってからもう一度試してください。</t>
+          <t>{0} に決闘を申し込みました…</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>GitHub does not answer. Check your connection and try again in a moment.</t>
+          <t>You challenge {0} to a duel…</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_player_kill</t>
+          <t>emp_duel_countdown</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>プレイヤー同士で倒せる</t>
+          <t>{0} と {1} が向かい合います。3秒後に決闘開始。</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Players can kill each other</t>
+          <t>{0} and {1} face each other. The duel starts in 3 seconds.</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_player_kill</t>
+          <t>emp_duel_fight</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>プレイヤーや仲間の攻撃で、ほかのプレイヤーを倒せます。オフ：致命傷でもHP0で生き残ります。</t>
+          <t>始め！</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Players and their companions can kill other players. Unticked, a deadly blow leaves them alive at 0 HP.</t>
+          <t>Fight!</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_host_manages_base</t>
+          <t>emp_duel_declined</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>拠点を管理できるのはホストだけ</t>
+          <t>決闘を断られました。</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Only the host manages the base</t>
+          <t>Your challenge was declined.</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_host_manages_base</t>
+          <t>emp_duel_noanswer</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>ほかのプレイヤーの拠点操作（研究、炉の技能、方針、名前、設定、住人、建築）は断られます。オフ：全員がホストと同じように管理できます。拠点を完全に手放せるのは常にホストだけです。</t>
+          <t>決闘の返事がありません。</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Others can't change the base: research, hearth skills, policies, names, settings, residents, build mode. Unticked, all can. Only the host can give up the base for good.</t>
+          <t>Nobody answered your challenge.</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_duels</t>
+          <t>emp_duel_busy</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>プレイヤー同士の決闘</t>
+          <t>そのプレイヤーは決闘中か取引中です。</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Duels between players</t>
+          <t>That player is busy in a duel or a trade.</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_duels</t>
+          <t>emp_duel_over</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>相手のキャラのメニューから決闘を申し込めます。誰も死なず、終わると全員回復し、何も失いません。</t>
+          <t>決闘は引き分けです。</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Challenge another player from the menu on their character. Nobody dies, both are healed and nothing is lost.</t>
+          <t>The duel ends in a draw.</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>emp_act_duel</t>
+          <t>emp_handover_failed</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>決闘を申し込む</t>
+          <t>キャラ {0} はこの世界に入れませんでした（死亡しています）。セーブのキャラで遊びます。</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Challenge to a duel</t>
+          <t>Your character {0} can't join this world because it is dead. You play the character of the save.</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>emp_duel_invite</t>
+          <t>emp_ui_depot_held_btn</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>{0}が決闘を申し込んできた。誰も死なないが、使った物は戻らない。受けますか？</t>
+          <t>{0} が世界をホスト中</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>{0} challenges you to a duel. Nobody dies, but what you use up stays used. Accept?</t>
+          <t>{0} is hosting the world</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>emp_duel_asked</t>
+          <t>emp_error_connection</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>{0} に決闘を申し込みました…</t>
+          <t>接続できません：ゲームが応答しません。ゲームが開いているか確認して、もう一度試してください。</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>You challenge {0} to a duel…</t>
+          <t>Could not connect. The game does not answer. Check that it is open, then try again.</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>emp_duel_countdown</t>
+          <t>emp_not_allowed</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>{0} と {1} が向かい合います。3秒後に決闘開始。</t>
+          <t>このゲームには、Steam ロビーから参加したプレイヤーしか入れません。</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>{0} and {1} face each other. The duel starts in 3 seconds.</t>
+          <t>Only players who join through its Steam lobby can enter this game.</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>emp_duel_fight</t>
+          <t>emp_connection_no_server</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>始め！</t>
+          <t>そのゲームはまだ開いていません。少し待ってからもう一度試してください。</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Fight!</t>
+          <t>That game is not open yet. Try again in a moment.</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>emp_duel_declined</t>
+          <t>emp_zone_session_empty</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>決闘を断られました。</t>
+          <t>ここにはもう誰もいません</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Your challenge was declined.</t>
+          <t>Nobody else is here anymore.</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>emp_duel_noanswer</t>
+          <t>emp_ui_timeout_steam</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>決闘の返事がありません。</t>
+          <t>ゲームが応答しません。相手が抜けたか、接続が切れたのかもしれません。</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Nobody answered your challenge.</t>
+          <t>The game does not answer. The player may have left or lost the connection.</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>emp_duel_busy</t>
+          <t>emp_ui_reconnecting</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>そのプレイヤーは決闘中か取引中です。</t>
+          <t>接続が切れました。ゲームに戻っています…</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>That player is busy in a duel or a trade.</t>
+          <t>Connection lost. Going back into the game…</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>emp_duel_over</t>
+          <t>emp_ui_reconnect_cancel</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>決闘は引き分けです。</t>
+          <t>キャンセル</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>The duel ends in a draw.</t>
+          <t>Cancel</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>emp_handover_failed</t>
+          <t>emp_ui_reconnect_failed</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>キャラ {0} はこの世界に入れませんでした（死亡しています）。セーブのキャラで遊びます。</t>
+          <t>ゲームに戻れませんでした。3分間応答がなく、終わった可能性があります。</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Your character {0} can't join this world because it is dead. You play the character of the save.</t>
+          <t>Could not get back into the game. It didn't answer for 3 minutes and may be over.</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>emp_ui_depot_held_btn</t>
+          <t>emp_ui_save_kept</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>{0} が世界をホスト中</t>
+          <t>進行状況は、参加したゲームが保存します。</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>{0} is hosting the world</t>
+          <t>The game you joined keeps your progress.</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>emp_error_connection</t>
+          <t>emp_ui_sv_cfg_auto_reconnect</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>接続できません：ゲームが応答しません。ゲームが開いているか確認して、もう一度試してください。</t>
+          <t>切れたプレイヤーは自動で戻る</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Could not connect. The game does not answer. Check that it is open, then try again.</t>
+          <t>Players rejoin by themselves after a drop</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>emp_not_allowed</t>
+          <t>emp_ui_sv_desc_auto_reconnect</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>このゲームには、Steam ロビーから参加したプレイヤーしか入れません。</t>
+          <t>接続が切れたプレイヤーは、3分間自動で再参加を試みます。オフ：タイトルに戻ります。</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Only players who join through its Steam lobby can enter this game.</t>
+          <t>A player who drops tries to rejoin for 3 minutes. Unticked, they go back to the title screen.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>emp_connection_no_server</t>
+          <t>emp_ui_sv_cfg_auto_host</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>そのゲームはまだ開いていません。少し待ってからもう一度試してください。</t>
+          <t>世界を読み込むと自動でフレンドに公開</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>That game is not open yet. Try again in a moment.</t>
+          <t>Open the game to friends when a world loads</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>emp_zone_session_empty</t>
+          <t>emp_ui_sv_desc_auto_host</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>ここにはもう誰もいません</t>
+          <t>世界を読み込むとすぐ、サーバーを手で始めなくてもフレンドが参加できます（所有した土地が必要）。オフ：ホストが自分でサーバーを始めます。</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Nobody else is here anymore.</t>
+          <t>Friends can join as soon as the world loads, with no need to start the server. The world needs a claimed land. Unticked, the host starts the server.</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>emp_ui_timeout_steam</t>
+          <t>emp_ui_sv_cfg_auto_save</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>ゲームが応答しません。相手が抜けたか、接続が切れたのかもしれません。</t>
+          <t>他のプレイヤーがいる間は自動でセーブ</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>The game does not answer. The player may have left or lost the connection.</t>
+          <t>Save automatically while others play</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>emp_trade_nothing_to_offer</t>
+          <t>emp_ui_sv_desc_auto_save</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>渡せる物がありません。</t>
+          <t>他のプレイヤーがいる間は2分ごと（遅いときは5分ごと）と、最後の人が抜けたときにセーブします。オフ：ホストがセーブしたときだけ。</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>You have nothing to offer.</t>
+          <t>Saves every 2 minutes while others are in the game (5 if saving is slow), and when the last one leaves. Unticked, only when the host saves.</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>emp_ui_reconnecting</t>
+          <t>emp_ui_load_blocked</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>接続が切れました。ゲームに戻っています…</t>
+          <t>みんなで遊んでいる間は、セーブをロードできません。</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Connection lost. Going back into the game…</t>
+          <t>You can't load a save while players are together.</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>emp_ui_reconnect_cancel</t>
+          <t>emp_ui_depot_join_btn</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>キャンセル</t>
+          <t>{0} に参加</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>Join {0}</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>emp_ui_reconnect_failed</t>
+          <t>emp_ui_depot_join_fail</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>ゲームに戻れませんでした。3分間応答がなく、終わった可能性があります。</t>
+          <t>{0} が世界を持っていますが、そのゲームはまだ開いていません。少し待ってからもう一度試してください。ゲームが止まっていたら、3分以内に世界は空きます。</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Could not get back into the game. It didn't answer for 3 minutes and may be over.</t>
+          <t>{0} has the world, but their game is not open yet. Try again in a moment. If their game stopped, the world is free again within 3 minutes.</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>emp_ui_save_kept</t>
+          <t>emp_ui_box_far</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>進行状況は、参加したゲームが保存します。</t>
+          <t>この箱は世界全体のもので、ホストが預かっています。ホストから離れていても入れた物はホストに届きますが、ホストのマップに戻るまで表示されません。</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>The game you joined keeps your progress.</t>
+          <t>This chest belongs to the whole world and the host keeps it. If you are away from the host, what you put in still arrives, but you only see it again back on the host's map.</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_auto_reconnect</t>
+          <t>emp_ui_sv_cfg_own_sleep</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>切れたプレイヤーは自動で戻る</t>
+          <t>各自で眠る</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Players rejoin by themselves after a drop</t>
+          <t>Everyone sleeps on their own</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_auto_reconnect</t>
+          <t>emp_ui_sv_desc_own_sleep</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>接続が切れたプレイヤーは、3分間自動で再参加を試みます。オフ：タイトルに戻ります。</t>
+          <t>ベッドに入ったプレイヤーはすぐ眠れます。夜が明けるのは、全員が同時に眠っているときだけです。オフ：全員が揃うまで待ちます。</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>A player who drops tries to rejoin for 3 minutes. Unticked, they go back to the title screen.</t>
+          <t>A player in bed sleeps at once. The night passes only when everyone sleeps at the same time. Unticked, everyone waits for everyone.</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_auto_host</t>
+          <t>emp_ui_sv_cfg_time_jumps_together</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>世界を読み込むと自動でフレンドに公開</t>
+          <t>全員一緒のときだけ時間が進む</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Open the game to friends when a world loads</t>
+          <t>Time moves only when all travel together</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_auto_host</t>
+          <t>emp_ui_sv_desc_time_jumps_together</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>世界を読み込むとすぐ、サーバーを手で始めなくてもフレンドが参加できます（所有した土地が必要）。オフ：ホストが自分でサーバーを始めます。</t>
+          <t>ワールドマップの一歩で日付が進むのは、全員が一緒に旅しているときだけです。そうでなければ旅人だけがターンを消費します。オフ：誰かの一歩ごとに全員が3時間進みます。</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Friends can join as soon as the world loads, with no need to start the server. The world needs a claimed land. Unticked, the host starts the server.</t>
+          <t>On the world map, the date moves only when all players travel together. Otherwise only the traveller's turns pass. Unticked, every step by anyone adds 3 hours for all.</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_auto_save</t>
+          <t>emp_ui_sv_cfg_dump_spares_belt</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>他のプレイヤーがいる間は自動でセーブ</t>
+          <t>自動整理で手持ちとツールベルトを残す</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Save automatically while others play</t>
+          <t>Auto-dump leaves your hands and tool belt alone</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_auto_save</t>
+          <t>emp_ui_sv_desc_dump_spares_belt</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>他のプレイヤーがいる間は2分ごと（遅いときは5分ごと）と、最後の人が抜けたときにセーブします。オフ：ホストがセーブしたときだけ。</t>
+          <t>手に持っている物とツールベルトの中身は、ホットバーと同じように、まとめて入れても残ります。オフ：元のゲームと同じ。</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Saves every 2 minutes while others are in the game (5 if saving is slow), and when the last one leaves. Unticked, only when the host saves.</t>
+          <t>Dump spares keeps what you hold and what is in your tool belt, like the hotbar. Unticked, it works as in the base game.</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>emp_ui_load_blocked</t>
+          <t>emp_ui_travel_no_date</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>みんなで遊んでいる間は、セーブをロードできません。</t>
+          <t>仲間は別の場所にいます。あなたの旅では日付は進みません。</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>You can't load a save while players are together.</t>
+          <t>Your friends are elsewhere. Your trip doesn't move the date.</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>emp_ui_depot_join_btn</t>
+          <t>emp_ui_bill_paid</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>{0} に参加</t>
+          <t>{0}が請求書を支払いました：{1}（{2}）</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Join {0}</t>
+          <t>{0} paid a bill: {1} ({2})</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>emp_ui_depot_join_fail</t>
+          <t>emp_ui_bill_already_paid</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>{0} が世界を持っていますが、そのゲームはまだ開いていません。少し待ってからもう一度試してください。ゲームが止まっていたら、3分以内に世界は空きます。</t>
+          <t>この請求書はもう払われています。お金は引かれていません。</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>{0} has the world, but their game is not open yet. Try again in a moment. If their game stopped, the world is free again within 3 minutes.</t>
+          <t>This bill is already paid. Nothing was taken from you.</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>emp_ui_box_far</t>
+          <t>emp_ui_sleep_alone</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>この箱は世界全体のもので、ホストが預かっています。ホストから離れていても入れた物はホストに届きますが、ホストのマップに戻るまで表示されません。</t>
+          <t>あなたは眠りました。世界は進みません：{0} がまだ起きています。</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>This chest belongs to the whole world and the host keeps it. If you are away from the host, what you put in still arrives, but you only see it again back on the host's map.</t>
+          <t>You slept. The world did not move on, as {0} is still awake.</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_own_sleep</t>
+          <t>emp_ui_sleep_count</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>各自で眠る</t>
+          <t>{0} は眠っている（{1}/{2}）</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Everyone sleeps on their own</t>
+          <t>{0} is asleep ({1} of {2})</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_own_sleep</t>
+          <t>emp_ui_sleep_all</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>ベッドに入ったプレイヤーはすぐ眠れます。夜が明けるのは、全員が同時に眠っているときだけです。オフ：全員が揃うまで待ちます。</t>
+          <t>全員が眠りました。夜が明けます。</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>A player in bed sleeps at once. The night passes only when everyone sleeps at the same time. Unticked, everyone waits for everyone.</t>
+          <t>Everyone is asleep. The night passes.</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_time_jumps_together</t>
+          <t>emp_ui_resync</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>全員一緒のときだけ時間が進む</t>
+          <t>マップを整えています…</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Time moves only when all travel together</t>
+          <t>Fixing the map…</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_time_jumps_together</t>
+          <t>emp_ui_sv_cfg_auto_resync</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>ワールドマップの一歩で日付が進むのは、全員が一緒に旅しているときだけです。そうでなければ旅人だけがターンを消費します。オフ：誰かの一歩ごとに全員が3時間進みます。</t>
+          <t>マップを自動で直す</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>On the world map, the date moves only when all players travel together. Otherwise only the traveller's turns pass. Unticked, every step by anyone adds 3 hours for all.</t>
+          <t>Fix the map automatically</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_dump_spares_belt</t>
+          <t>emp_ui_sv_desc_auto_resync</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>自動整理で手持ちとツールベルトを残す</t>
+          <t>マップがホストと食い違う（物やキャラが足りない）と、自動で読み込み直します。30秒に1回まで。オフ：違いはログに書くだけ。</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Auto-dump leaves your hands and tool belt alone</t>
+          <t>If a player's map differs from the host's, with an item or character missing, it loads again by itself, at most every 30 seconds. Unticked, the difference is only logged.</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_dump_spares_belt</t>
+          <t>emp_ui_bank_deposit</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>手に持っている物とツールベルトの中身は、ホットバーと同じように、まとめて入れても残ります。オフ：元のゲームと同じ。</t>
+          <t>{0}が銀行に{1}を預けました</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Dump spares keeps what you hold and what is in your tool belt, like the hotbar. Unticked, it works as in the base game.</t>
+          <t>{0} put {1} in the bank</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>emp_ui_travel_no_date</t>
+          <t>emp_ui_bank_withdraw</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>仲間は別の場所にいます。あなたの旅では日付は進みません。</t>
+          <t>{0}が銀行から{1}を引き出しました</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Your friends are elsewhere. Your trip doesn't move the date.</t>
+          <t>{0} took {1} out of the bank</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>emp_ui_bill_paid</t>
+          <t>emp_ui_sv_cfg_world_copy</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>{0}が請求書を支払いました：{1}（{2}）</t>
+          <t>ほかのプレイヤーも世界のコピーを持つ</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>{0} paid a bill: {1} ({2})</t>
+          <t>Other players keep a copy of the world</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>emp_ui_bill_already_paid</t>
+          <t>emp_ui_sv_desc_world_copy</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>この請求書はもう払われています。お金は引かれていません。</t>
+          <t>自動セーブのたびに、全員のPCが自分のセーブとは別に世界のコピーを保管します。オフ：世界はホストのPCにしかありません。</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>This bill is already paid. Nothing was taken from you.</t>
+          <t>After each automatic save, every player's PC keeps a copy of the world, apart from their own saves. Unticked, only the host's PC has it.</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>emp_ui_sleep_alone</t>
+          <t>emp_ui_sv_cfg_shared_tax</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>あなたは眠りました。世界は進みません：{0} がまだ起きています。</t>
+          <t>税金は最も有名なプレイヤーで計算</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>You slept. The world did not move on, as {0} is still awake.</t>
+          <t>Tax follows the most famous player</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>emp_ui_sleep_count</t>
+          <t>emp_ui_sv_desc_shared_tax</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>{0} は眠っている（{1}/{2}）</t>
+          <t>毎月の税金は、接続中のプレイヤーでいちばん高い名声で計算します。オフ：ホストの名声で計算（元のゲームと同じ）。</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>{0} is asleep ({1} of {2})</t>
+          <t>Monthly tax uses the highest fame among the players. Unticked, it uses the host's fame, as in the base game.</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>emp_ui_sleep_all</t>
+          <t>emp_ui_sv_cfg_soft_recall</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>全員が眠りました。夜が明けます。</t>
+          <t>合流のとき世界を読み込み直さない</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Everyone is asleep. The night passes.</t>
+          <t>Rejoin without reloading the world</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>emp_ui_resync</t>
+          <t>emp_ui_sv_desc_soft_recall</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>マップを整えています…</t>
+          <t>ホストとプレイヤーが同じマップになるとき、世界全体は読み込み直さず、そのまま、またはそのマップだけを読み込みます。合わないときは従来どおり読み込み直します。オフ：毎回読み込み直します。</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Fixing the map…</t>
+          <t>When the host and a player meet on one map, the whole world does not reload. Only that map loads, or nothing. If something doesn't match, the world reloads as before. Unticked, it always reloads.</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_auto_resync</t>
+          <t>emp_ui_sv_cfg_publish_mods</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>マップを自動で直す</t>
+          <t>ゲームのMOD一覧をプレイヤーに見せる</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Fix the map automatically</t>
+          <t>Show the game's mods to players</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_auto_resync</t>
+          <t>emp_ui_sv_desc_publish_mods</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>マップがホストと食い違う（物やキャラが足りない）と、自動で読み込み直します。30秒に1回まで。オフ：違いはログに書くだけ。</t>
+          <t>参加前（ゲーム一覧）と参加時にMOD一覧が分かり、断られたときは違うMODが名前で表示されます。デポから取った世界では、デポの一覧（modlist.txt）を使います。オフ：何も伝えません。</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>If a player's map differs from the host's, with an item or character missing, it loads again by itself, at most every 30 seconds. Unticked, the difference is only logged.</t>
+          <t>Players see the mod list before joining and when joining. If refused, they are told which mods differ. For a world from a depot, the depot's list (modlist.txt) is used. Unticked, nothing is shown.</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>emp_ui_bank_deposit</t>
+          <t>emp_ui_cl_fetch_mods</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>{0}が銀行に{1}を預けました</t>
+          <t>ゲームのMODをダウンロードする</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>{0} put {1} in the bank</t>
+          <t>Download the game's mods</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>emp_ui_bank_withdraw</t>
+          <t>emp_ui_cl_desc_fetch_mods</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>{0}が銀行から{1}を引き出しました</t>
+          <t>参加するゲームのMODで足りない Workshop のものを、購読せずにダウンロードします。Elin は一度再起動し、自動でゲームに戻ります。MOD一覧は次の起動で元に戻ります。オフ：違うMODを知らせるだけ。</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>{0} took {1} out of the bank</t>
+          <t>Missing Workshop mods of the game you join are downloaded without subscribing. Elin restarts once with those mods and comes back by itself. Your own list returns at the next start. Unticked, you are only told which mods differ.</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_world_copy</t>
+          <t>emp_ui_mods_lobby</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ほかのプレイヤーも世界のコピーを持つ</t>
+          <t>Mod {0} 個</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Other players keep a copy of the world</t>
+          <t>{0} mods</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_world_copy</t>
+          <t>emp_ui_mods_lobby_missing</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>自動セーブのたびに、全員のPCが自分のセーブとは別に世界のコピーを保管します。オフ：世界はホストのPCにしかありません。</t>
+          <t>{0} 個のMOD（{1} 個が足りません）</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>After each automatic save, every player's PC keeps a copy of the world, apart from their own saves. Unticked, only the host's PC has it.</t>
+          <t>{0} mods, {1} missing</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_shared_tax</t>
+          <t>emp_ui_mods_world</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>税金は最も有名なプレイヤーで計算</t>
+          <t>この世界のMODのうち {0} 個が読み込まれていません：{1}。一覧はログにあります。</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Tax follows the most famous player</t>
+          <t>{0} mods of this world are not loaded: {1}. The full list is in the log.</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_shared_tax</t>
+          <t>emp_ui_mods_missing</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>毎月の税金は、接続中のプレイヤーでいちばん高い名声で計算します。オフ：ホストの名声で計算（元のゲームと同じ）。</t>
+          <t>ホストのMODで足りないもの（{0}）：{1}</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Monthly tax uses the highest fame among the players. Unticked, it uses the host's fame, as in the base game.</t>
+          <t>Host mods you don't have ({0}): {1}</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_soft_recall</t>
+          <t>emp_ui_mods_hand</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>合流のとき世界を読み込み直さない</t>
+          <t>手動で入れるMOD（{0}）：{1}</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Rejoin without reloading the world</t>
+          <t>Mods to install yourself ({0}): {1}</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_soft_recall</t>
+          <t>emp_ui_mods_extra</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>ホストとプレイヤーが同じマップになるとき、世界全体は読み込み直さず、そのまま、またはそのマップだけを読み込みます。合わないときは従来どおり読み込み直します。オフ：毎回読み込み直します。</t>
+          <t>ホストにないMOD（{0}）：{1}</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>When the host and a player meet on one map, the whole world does not reload. Only that map loads, or nothing. If something doesn't match, the world reloads as before. Unticked, it always reloads.</t>
+          <t>Mods the host doesn't have ({0}): {1}</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_publish_mods</t>
+          <t>emp_ui_mods_fetching</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>ゲームのMOD一覧をプレイヤーに見せる</t>
+          <t>ゲームのMODをダウンロード中 {0}/{1}：{2} {3}%（Escで中止）</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Show the game's mods to players</t>
+          <t>Downloading the game's mods {0}/{1}: {2} {3}% (Esc to cancel)</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_publish_mods</t>
+          <t>emp_ui_mods_fetch_failed</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>参加前（ゲーム一覧）と参加時にMOD一覧が分かり、断られたときは違うMODが名前で表示されます。デポから取った世界では、デポの一覧（modlist.txt）を使います。オフ：何も伝えません。</t>
+          <t>ゲームのMODをダウンロードできませんでした。何も変更していません。</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Players see the mod list before joining and when joining. If refused, they are told which mods differ. For a world from a depot, the depot's list (modlist.txt) is used. Unticked, nothing is shown.</t>
+          <t>Could not download the mods. Nothing was changed.</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>emp_ui_cl_fetch_mods</t>
+          <t>emp_ui_mods_restart</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>ゲームのMODをダウンロードする</t>
+          <t>Elin はゲームのMODで再起動し、自動でゲームに戻ります。起動しないときは、Elin をもう一度起動してください。</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Download the game's mods</t>
+          <t>Elin restarts with the game's mods and comes back by itself. If it doesn't start, start Elin again.</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>emp_ui_cl_desc_fetch_mods</t>
+          <t>emp_ui_mods_restart_manual</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>参加するゲームのMODで足りない Workshop のものを、購読せずにダウンロードします。Elin は一度再起動し、自動でゲームに戻ります。MOD一覧は次の起動で元に戻ります。オフ：違うMODを知らせるだけ。</t>
+          <t>Elin を閉じます。もう一度起動すると、ゲームのMODで自動でゲームに戻ります。</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Missing Workshop mods of the game you join are downloaded without subscribing. Elin restarts once with those mods and comes back by itself. Your own list returns at the next start. Unticked, you are only told which mods differ.</t>
+          <t>Elin closes. Start it again and it comes back to the game by itself, with its mods.</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>emp_ui_mods_lobby</t>
+          <t>emp_ui_mods_session</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Mod {0} 個</t>
+          <t>今回の Elin は、マルチプレイのMODで動いています。MOD一覧は次の起動で元に戻ります。次回の再起動を省くには、クライアント設定の「ゲームのMODを残す」にチェックしてください。</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>{0} mods</t>
+          <t>This time Elin runs with the game's mods. Your own list returns at the next start. To skip this restart next time, tick "Keep the game's mods" in Client Settings.</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>emp_ui_mods_lobby_missing</t>
+          <t>emp_ui_mods_session_locked</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>{0} 個のMOD（{1} 個が足りません）</t>
+          <t>今回はMOD一覧を保存しません。次の起動で元の一覧に戻ります。</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>{0} mods, {1} missing</t>
+          <t>The mod list is not saved this time. Yours returns at the next start of Elin.</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>emp_ui_mods_world</t>
+          <t>emp_ui_cl_keep_mods</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>この世界のMODのうち {0} 個が読み込まれていません：{1}。一覧はログにあります。</t>
+          <t>ゲームのMODを残す（Workshop で購読）</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>{0} mods of this world are not loaded: {1}. The full list is in the log.</t>
+          <t>Keep the game's mods (subscribe on the Workshop)</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>emp_ui_mods_missing</t>
+          <t>emp_ui_cl_desc_keep_mods</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>ホストのMODで足りないもの（{0}）：{1}</t>
+          <t>参加するゲームのMODを Steam アカウントで購読し、自分のMOD一覧に残します。最初の一度だけ再起動し、以降は Elin を閉じても再起動なしで同じゲームに入れます。取り消すには Workshop で購読を解除します。オフ：購読せず取得し、起動後の最初の参加で毎回再起動します。</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Host mods you don't have ({0}): {1}</t>
+          <t>Your Steam account subscribes to the mods of the game you join and keeps them on. Elin restarts once, the first time. After that you rejoin the same game with no restart. To undo, unsubscribe on the Workshop. Unticked, Elin restarts at the first join of every start.</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>emp_ui_mods_hand</t>
+          <t>emp_ui_sv_cfg_takeover</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>手動で入れるMOD（{0}）：{1}</t>
+          <t>ホストが抜けたら別のプレイヤーが引き継ぐ</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Mods to install yourself ({0}): {1}</t>
+          <t>Another player takes over when the host leaves</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>emp_ui_mods_extra</t>
+          <t>emp_ui_sv_desc_takeover</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>ホストにないMOD（{0}）：{1}</t>
+          <t>ホストが抜けると、プレイヤーのひとりが自分のコピーから世界を開き、そこでゲームが続きます（「世界のコピー」が必要）。オフ：ホストが抜けるとゲームは終わります。</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Mods the host doesn't have ({0}): {1}</t>
+          <t>When the host leaves, a player opens the world from their copy and the game goes on. Needs the world copy option. Unticked, the game ends with the host.</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>emp_ui_mods_fetching</t>
+          <t>emp_takeover_begin</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>ゲームのMODをダウンロード中 {0}/{1}：{2} {3}%（Escで中止）</t>
+          <t>ホストが抜けました。あなたが世界を引き継ぎます。まもなくここでゲームが続きます。</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Downloading the game's mods {0}/{1}: {2} {3}% (Esc to cancel)</t>
+          <t>The host left. You take over the world. The game goes on here in a moment.</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>emp_ui_mods_fetch_failed</t>
+          <t>emp_takeover_leaving</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>ゲームのMODをダウンロードできませんでした。何も変更していません。</t>
+          <t>退出中：ほかのプレイヤーに最後のセーブを渡しています…</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Could not download the mods. Nothing was changed.</t>
+          <t>Leaving. Giving the last save to the others…</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>emp_ui_mods_restart</t>
+          <t>emp_ui_limited_bought</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Elin はゲームのMODで再起動し、自動でゲームに戻ります。起動しないときは、Elin をもう一度起動してください。</t>
+          <t>それはもう買いました。</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Elin restarts with the game's mods and comes back by itself. If it doesn't start, start Elin again.</t>
+          <t>You already bought this one.</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>emp_ui_mods_restart_manual</t>
+          <t>emp_story_share</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Elin を閉じます。もう一度起動すると、ゲームのMODで自動でゲームに戻ります。</t>
+          <t>{0}の分け前</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Elin closes. Start it again and it comes back to the game by itself, with its mods.</t>
+          <t>{0}'s share</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>emp_ui_mods_session</t>
+          <t>emp_ui_sv_cfg_once_per_player</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>今回の Elin は、マルチプレイのMODで動いています。MOD一覧は次の起動で元に戻ります。次回の再起動を省くには、クライアント設定の「ゲームのMODを残す」にチェックしてください。</t>
+          <t>一度きりの報酬をプレイヤーごとに</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>This time Elin runs with the game's mods. Your own list returns at the next start. To skip this restart next time, tick "Keep the game's mods" in Client Settings.</t>
+          <t>One-time rewards for every player</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>emp_ui_mods_session_locked</t>
+          <t>emp_ui_sv_desc_once_per_player</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>今回はMOD一覧を保存しません。次の起動で元の一覧に戻ります。</t>
+          <t>店の限定品と、ストーリーでもらえる物（依頼の報酬、会話の贈り物）が、プレイヤーごとに1回ずつ手に入ります。オフ：最初のひとりだけ（元のゲームと同じ）。</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>The mod list is not saved this time. Yours returns at the next start of Elin.</t>
+          <t>One-time shop goods and story gifts, like quest rewards, go once to each player. Unticked, only the first player gets them, as in the base game.</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>emp_ui_cl_keep_mods</t>
+          <t>emp_takeover_rejoin</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>ゲームのMODを残す（Workshop で購読）</t>
+          <t>別のプレイヤーがこの世界を引き継ぎました。そのゲームに参加します…</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Keep the game's mods (subscribe on the Workshop)</t>
+          <t>Another player took over this world. Joining them…</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>emp_ui_cl_desc_keep_mods</t>
+          <t>emp_story_share_got</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>参加するゲームのMODを Steam アカウントで購読し、自分のMOD一覧に残します。最初の一度だけ再起動し、以降は Elin を閉じても再起動なしで同じゲームに入れます。取り消すには Workshop で購読を解除します。オフ：購読せず取得し、起動後の最初の参加で毎回再起動します。</t>
+          <t>ストーリーでもらえた物のうち、あなたの分を受け取りました：{0}。</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Your Steam account subscribes to the mods of the game you join and keeps them on. Elin restarts once, the first time. After that you rejoin the same game with no restart. To undo, unsubscribe on the Workshop. Unticked, Elin restarts at the first join of every start.</t>
+          <t>You get your share of what the story gave: {0}.</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_takeover</t>
+          <t>emp_story_share_mail</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>ホストが抜けたら別のプレイヤーが引き継ぐ</t>
+          <t>ストーリーでもらえた物のうち、あなたの分（{0}）を拠点の郵便に送りました。</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Another player takes over when the host leaves</t>
+          <t>Your share of what the story gave ({0}) was sent to the base's mail.</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_takeover</t>
+          <t>emp_ui_report</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>ホストが抜けると、プレイヤーのひとりが自分のコピーから世界を開き、そこでゲームが続きます（「世界のコピー」が必要）。オフ：ホストが抜けるとゲームは終わります。</t>
+          <t>不具合レポートを作成</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>When the host leaves, a player opens the world from their copy and the game goes on. Needs the world copy option. Unticked, the game ends with the host.</t>
+          <t>Prepare a bug report</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>emp_takeover_begin</t>
+          <t>emp_ui_report_desc</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>ホストが抜けました。あなたが世界を引き継ぎます。まもなくここでゲームが続きます。</t>
+          <t>ゲームとMODのログをまとめた zip をデスクトップに作ります。セーブと設定ファイルは含みません。不具合を報告するときに送ってください。</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>The host left. You take over the world. The game goes on here in a moment.</t>
+          <t>Writes a zip with the game and mod logs on your desktop. No save, no settings. Send it when you report a problem.</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>emp_takeover_leaving</t>
+          <t>emp_ui_report_done</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>退出中：ほかのプレイヤーに最後のセーブを渡しています…</t>
+          <t>レポートを作成しました：{0}</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Leaving. Giving the last save to the others…</t>
+          <t>Bug report written: {0}</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>emp_ui_limited_bought</t>
+          <t>emp_ui_report_failed</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>それはもう買いました。</t>
+          <t>レポートを作成できませんでした。</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>You already bought this one.</t>
+          <t>The bug report could not be written.</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>emp_story_share</t>
+          <t>emp_ui_sv_bills</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>{0}の分け前</t>
+          <t>未払いの税金請求書：カウント {0}、実在 {1}（修復する）</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>{0}'s share</t>
+          <t>Unpaid tax bills: counted {0}, existing {1} (repair)</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_once_per_player</t>
+          <t>emp_ui_sv_bills_desc</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>一度きりの報酬をプレイヤーごとに</t>
+          <t>カウントが実際の請求書より多いとき（古い不具合）、実際の数に合わせます。増やすことはありません。</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>One-time rewards for every player</t>
+          <t>If the count is above the bills that exist (an old bug), it is set to the real number. It is never raised.</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_once_per_player</t>
+          <t>emp_ui_sv_bills_done</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>店の限定品と、ストーリーでもらえる物（依頼の報酬、会話の贈り物）が、プレイヤーごとに1回ずつ手に入ります。オフ：最初のひとりだけ（元のゲームと同じ）。</t>
+          <t>支払えない請求書 {0} 件をカウントから外しました。</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>One-time shop goods and story gifts, like quest rewards, go once to each player. Unticked, only the first player gets them, as in the base game.</t>
+          <t>{0} bill(s) that nothing could pay were taken off the count.</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>emp_takeover_rejoin</t>
+          <t>emp_ui_sv_bills_none</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>別のプレイヤーがこの世界を引き継ぎました。そのゲームに参加します…</t>
+          <t>カウントは実在する請求書と一致しています。</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Another player took over this world. Joining them…</t>
+          <t>The count matches the bills that exist.</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>emp_story_share_got</t>
+          <t>emp_ui_chara_delete</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>ストーリーでもらえた物のうち、あなたの分を受け取りました：{0}。</t>
+          <t>キャラクターを削除する</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>You get your share of what the story gave: {0}.</t>
+          <t>Delete a character</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>emp_story_share_mail</t>
+          <t>emp_ui_chara_delete_confirm</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>ストーリーでもらえた物のうち、あなたの分（{0}）を拠点の郵便に送りました。</t>
+          <t>#1 を削除しますか？持ち物も一緒に消えます。仲間はこの世界に残ります。</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Your share of what the story gave ({0}) was sent to the base's mail.</t>
+          <t>Delete #1? Its belongings go with it. Its companions stay in this world.</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>emp_ui_report</t>
+          <t>emp_ui_chara_deleted</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>不具合レポートを作成</t>
+          <t>キャラクターを削除しました。</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Prepare a bug report</t>
+          <t>The character was deleted.</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>emp_ui_report_desc</t>
+          <t>emp_ui_sv_cfg_delete_chara</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>ゲームとMODのログをまとめた zip をデスクトップに作ります。セーブと設定ファイルは含みません。不具合を報告するときに送ってください。</t>
+          <t>プレイヤーが自分のキャラを削除できる</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Writes a zip with the game and mod logs on your desktop. No save, no settings. Send it when you report a problem.</t>
+          <t>Players can delete their characters</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>emp_ui_report_done</t>
+          <t>emp_ui_sv_desc_delete_chara</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>レポートを作成しました：{0}</t>
+          <t>キャラの一覧から削除します（確認は2回）。持ち物も消え、仲間は世界に残ります。</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Bug report written: {0}</t>
+          <t>Done from the character list, with two confirmations. Belongings go too. Companions stay in the world.</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>emp_ui_report_failed</t>
+          <t>emp_world_setting_host</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>レポートを作成できませんでした。</t>
+          <t>世界の設定はホストのものです。変更は保存されませんでした。</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>The bug report could not be written.</t>
+          <t>World settings belong to the host. Your changes were not kept.</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>emp_ui_sv_bills</t>
+          <t>emp_ui_sv_cfg_auto_combat_per_player</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>未払いの税金請求書：カウント {0}、実在 {1}（修復する）</t>
+          <t>自動戦闘はそれぞれ自分の仲間を守る</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Unpaid tax bills: counted {0}, existing {1} (repair)</t>
+          <t>Each player's auto combat protects their own</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>emp_ui_sv_bills_desc</t>
+          <t>emp_ui_sv_desc_auto_combat_per_player</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>カウントが実際の請求書より多いとき（古い不具合）、実際の数に合わせます。増やすことはありません。</t>
+          <t>自動戦闘を使うプレイヤーと仲間を、そのプレイヤー自身の戦術とスタミナで致命傷から守ります。オフ：ホストの自動戦闘が全員を守り、ゲストのは誰も守りません。</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>If the count is above the bills that exist (an old bug), it is set to the real number. It is never raised.</t>
+          <t>Auto combat saves the player using it, and their companions, from a deadly hit, with their own tactics and stamina. Unticked, the host's auto combat protects everyone and a guest's protects no one.</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>emp_ui_sv_bills_done</t>
+          <t>emp_duel_win</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>支払えない請求書 {0} 件をカウントから外しました。</t>
+          <t>{0}との決闘に勝った！</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>{0} bill(s) that nothing could pay were taken off the count.</t>
+          <t>You win the duel against {0}!</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>emp_ui_sv_bills_none</t>
+          <t>emp_duel_lose</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>カウントは実在する請求書と一致しています。</t>
+          <t>{0}との決闘に負けた。</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>The count matches the bills that exist.</t>
+          <t>You lose the duel against {0}.</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>emp_ui_chara_delete</t>
+          <t>emp_duel_wait</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>キャラクターを削除する</t>
+          <t>まだ {0} に決闘を申し込めません。</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Delete a character</t>
+          <t>You can't challenge {0} again so soon.</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>emp_ui_chara_delete_confirm</t>
+          <t>emp_trade_gold_button</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>#1 を削除しますか？持ち物も一緒に消えます。仲間はこの世界に残ります。</t>
+          <t>お金</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Delete #1? Its belongings go with it. Its companions stay in this world.</t>
+          <t>Gold</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>emp_ui_chara_deleted</t>
+          <t>emp_trade_locked</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>キャラクターを削除しました。</t>
+          <t>変更があったばかりだ。少し待ってから確定しよう。</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>The character was deleted.</t>
+          <t>The offer just changed. Wait a moment before validating.</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_delete_chara</t>
+          <t>emp_trade_log_add</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>プレイヤーが自分のキャラを削除できる</t>
+          <t>{0}が{1}を差し出した。</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Players can delete their characters</t>
+          <t>{0} offers {1}.</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_delete_chara</t>
+          <t>emp_trade_log_remove</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>キャラの一覧から削除します（確認は2回）。持ち物も消え、仲間は世界に残ります。</t>
+          <t>{0}が{1}を引っ込めた。</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Done from the character list, with two confirmations. Belongings go too. Companions stay in the world.</t>
+          <t>{0} takes back {1}.</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>emp_world_setting_host</t>
+          <t>emp_trade_log_gold</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>世界の設定はホストのものです。変更は保存されませんでした。</t>
+          <t>{0}の提示額は{1}オレンになった。</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>World settings belong to the host. Your changes were not kept.</t>
+          <t>{0} now offers {1} gold.</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>emp_ui_sv_cfg_auto_combat_per_player</t>
+          <t>emp_trade_cant_offer</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>自動戦闘はそれぞれ自分の仲間を守る</t>
+          <t>{0}は差し出せない。</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Each player's auto combat protects their own</t>
+          <t>You can't offer {0}.</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>emp_ui_sv_desc_auto_combat_per_player</t>
+          <t>emp_trade_status</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>自動戦闘を使うプレイヤーと仲間を、そのプレイヤー自身の戦術とスタミナで致命傷から守ります。オフ：ホストの自動戦闘が全員を守り、ゲストのは誰も守りません。</t>
+          <t>{0}: {1}オレン、{2}</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
-        <is>
-          <t>Auto combat saves the player using it, and their companions, from a deadly hit, with their own tactics and stamina. Unticked, the host's auto combat protects everyone and a guest's protects no one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="inlineStr">
-        <is>
-          <t>emp_duel_win</t>
-        </is>
-      </c>
-      <c r="C315" t="inlineStr">
-        <is>
-          <t>{0}との決闘に勝った！</t>
-        </is>
-      </c>
-      <c r="D315" t="inlineStr">
-        <is>
-          <t>You win the duel against {0}!</t>
-        </is>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="inlineStr">
-        <is>
-          <t>emp_duel_lose</t>
-        </is>
-      </c>
-      <c r="C316" t="inlineStr">
-        <is>
-          <t>{0}との決闘に負けた。</t>
-        </is>
-      </c>
-      <c r="D316" t="inlineStr">
-        <is>
-          <t>You lose the duel against {0}.</t>
-        </is>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="inlineStr">
-        <is>
-          <t>emp_duel_wait</t>
-        </is>
-      </c>
-      <c r="C317" t="inlineStr">
-        <is>
-          <t>まだ {0} に決闘を申し込めません。</t>
-        </is>
-      </c>
-      <c r="D317" t="inlineStr">
-        <is>
-          <t>You can't challenge {0} again so soon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="inlineStr">
-        <is>
-          <t>emp_trade_gold_button</t>
-        </is>
-      </c>
-      <c r="C318" t="inlineStr">
-        <is>
-          <t>お金</t>
-        </is>
-      </c>
-      <c r="D318" t="inlineStr">
-        <is>
-          <t>Gold</t>
-        </is>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="inlineStr">
-        <is>
-          <t>emp_trade_locked</t>
-        </is>
-      </c>
-      <c r="C319" t="inlineStr">
-        <is>
-          <t>変更があったばかりだ。少し待ってから確定しよう。</t>
-        </is>
-      </c>
-      <c r="D319" t="inlineStr">
-        <is>
-          <t>The offer just changed. Wait a moment before validating.</t>
-        </is>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="inlineStr">
-        <is>
-          <t>emp_trade_log_add</t>
-        </is>
-      </c>
-      <c r="C320" t="inlineStr">
-        <is>
-          <t>{0}が{1}を差し出した。</t>
-        </is>
-      </c>
-      <c r="D320" t="inlineStr">
-        <is>
-          <t>{0} offers {1}.</t>
-        </is>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="inlineStr">
-        <is>
-          <t>emp_trade_log_remove</t>
-        </is>
-      </c>
-      <c r="C321" t="inlineStr">
-        <is>
-          <t>{0}が{1}を引っ込めた。</t>
-        </is>
-      </c>
-      <c r="D321" t="inlineStr">
-        <is>
-          <t>{0} takes back {1}.</t>
-        </is>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="inlineStr">
-        <is>
-          <t>emp_trade_log_gold</t>
-        </is>
-      </c>
-      <c r="C322" t="inlineStr">
-        <is>
-          <t>{0}の提示額は{1}オレンになった。</t>
-        </is>
-      </c>
-      <c r="D322" t="inlineStr">
-        <is>
-          <t>{0} now offers {1} gold.</t>
-        </is>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="inlineStr">
-        <is>
-          <t>emp_trade_cant_offer</t>
-        </is>
-      </c>
-      <c r="C323" t="inlineStr">
-        <is>
-          <t>{0}は差し出せない。</t>
-        </is>
-      </c>
-      <c r="D323" t="inlineStr">
-        <is>
-          <t>You can't offer {0}.</t>
-        </is>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="inlineStr">
-        <is>
-          <t>emp_trade_status</t>
-        </is>
-      </c>
-      <c r="C324" t="inlineStr">
-        <is>
-          <t>{0}: {1}オレン、{2}</t>
-        </is>
-      </c>
-      <c r="D324" t="inlineStr">
         <is>
           <t>{0}: {1} gold, {2}</t>
         </is>

</xml_diff>

<commit_message>
Town life around every player: townspeople's idle life near every player, rumours and stones by that player's karma
Council 2026-10-23, point 4. In the host's game AI_Idle chatted, greeted, gossiped and threw stones only near the
host's screen (isSynced, IsInMutterDistance) and always about the host's character and karma. A transpiler on
AI_Idle.Run widens the three idle-talk / greeting reads to "seen by the host or near another player" and makes the
greeting / rumour / stone branch use the nearest player and its own karma (ElinNetHost.KarmaOf). The NPC's talk
passes the game's isSynced gate for that step only, its bubble goes to the guests and the host's renderer draws
nothing. Host checkbox "Town life around every player", default on. With no other player near, the game's own.

Compiled only, not run in game. Bench step y14 (oct10_suite) written, not run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D314"/>
+  <dimension ref="A1:D316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5787,6 +5787,40 @@
         </is>
       </c>
     </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_town_life</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>全プレイヤーの周りで町の人が暮らす</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Town life around every player</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_town_life</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>町の人は、ホストの画面の近くだけでなく、すべてのプレイヤーの近くで雑談し、あいさつし、噂し、石を投げます。噂と石は、その相手のプレイヤー自身のカルマで決まります。オフにすると、ホストの近くだけで、ホストのカルマで決まります（バニラと同じ）。</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Townspeople chat, greet, gossip and throw stones near every player, not only near the host's screen. Gossip and stones go by the karma of the player they are about. Unticked: only near the host, by the host's karma (as in vanilla).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Town boards: the fame gate reads the highest fame on the map, the danger follows the players present (host box 'Town boards from every player present', on)
Only when the game regenerates the board (Zone.UpdateQuests) with at least two players on the map; the host alone and the box off are the game's own. Supply rewards need no change: the turn-in already runs under PlayerStandIn. Compiled, never run; suite boards_suite.py written, not run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D314"/>
+  <dimension ref="A1:D316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5787,6 +5787,40 @@
         </is>
       </c>
     </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_town_boards</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>町の掲示板を全員の分で作る</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Town boards from every player present</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_town_boards</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>ゲームが町の掲示板の依頼を引き直すとき、マップにいる全員の中で最も高い名声が名声が必要な依頼を開き、難易度は在場のプレイヤーの平均になります。オフの場合はホストのキャラだけで決まります（原作どおり）。</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>When the game draws a town board's offers again, the highest fame among the players on the map opens the offers that need fame, and the difficulty follows the players present. Unticked, the board is drawn for the host's character alone (as in the base game).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Map spawns read the feats of the player nearest to the spawn
Zone.SpawnMob and TryGenerateEvolved/BigDaddy/Shrine read the feats (1270/1271/1216) of EClass.pc: on the host always the host's character. A transpiler now asks the player nearest to the spawn point (host rule Spawns from the nearest player, default on). Alone, rule off, a guest's own action (stand-in) or no point: the game's player, unchanged. Not run in game: bench spawns_suite.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D314"/>
+  <dimension ref="A1:D316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5787,6 +5787,40 @@
         </is>
       </c>
     </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_nearest_spawns</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>スポーンはいちばん近いプレイヤーから</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Spawns from the nearest player</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_nearest_spawns</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>マップのスポーン（伝説の個体の確率、サンタなどの敵味方、進化個体、ビッグダディ、祠）は、ホストではなくスポーン地点にいちばん近いプレイヤーの特性で決まります。オフならホストの特性（元のゲームと同じ）。</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>What a map spawns (legendary chance, friend or foe of Santa and the like, evolved, big daddy, shrines) reads the feats of the player nearest to the spawn, not always the host's. Unticked: the host's, as in the game.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Shops: the stock bonus is the best player's on the map, special shelves follow the player who opens the shop
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D314"/>
+  <dimension ref="A1:D316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5787,6 +5787,40 @@
         </is>
       </c>
     </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_shops_from_every_player</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>全員の進行に合わせた店</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Shops from every player present</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_shops_from_every_player</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>店の仕入れ量は地図上で最も強いプレイヤーの特性で決まり、特別な棚（結婚とカセットの店、ロイテルのマート、異国の商人）は店を開いたプレイヤーの進行に従います。オフの場合は常にホストの進行（原作と同じ）。</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>A shop restocks with the stock bonus of the best player on the map, and its special shelves (marriage and tape shop, Loytel's mart, exotic merchant) follow the player who opens it. Off: always the host's progress, as the game does.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Review fixes for the council features
- Shops: the mages guild's trial letter follows the opener (ShopGates Key 3, postfix on Guild.IsMember during a restock); Loytel's level from a guest clamped to 0..2.
- Gifts: things that do not stack are no longer cut to 1 (a dialog gives several spellbooks or deeds), cap 1000 like stacks; an element unknown to the host is left as it came instead of throwing.
- Town boards: the option text says it needs personal quests.
Compiles; not yet run in game (shops_suite MAGE step added).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -5846,12 +5846,12 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>ゲームが町の掲示板の依頼を引き直すとき、マップにいる全員の中で最も高い名声が名声が必要な依頼を開き、難易度は在場のプレイヤーの平均になります。オフの場合はホストのキャラだけで決まります（原作どおり）。</t>
+          <t>ゲームが町の掲示板の依頼を引き直すとき、マップにいる全員の中で最も高い名声が名声が必要な依頼を開き、難易度は在場のプレイヤーの平均になります。オフの場合はホストのキャラだけで決まります（原作どおり）。（個人クエストが有効な場合のみ。）</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>When the game draws a town board's offers again, the highest fame among the players on the map opens the offers that need fame, and the difficulty follows the players present. Unticked, the board is drawn for the host's character alone (as in the base game).</t>
+          <t>When the game draws a town board's offers again, the highest fame among the players on the map opens the offers that need fame, and the difficulty follows the players present. Unticked, the board is drawn for the host's character alone (as in the base game). Needs personal quests.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mod config page drawn from the settings table (council 2026-10-23, step 5)
The game's own mod config page renders the same table as the World rules
tab: the preset line with what differs, Reset to recommended, Undo, the
visible rows (choices as dropdowns, boxes greyed by what they need, the
description under each), "Show advanced options" for all the boxes (a
host on the title screen has no World rules tab: every box stays
reachable here), "More options in the Elin Together window", then the
two client mod toggles. The joining check boxes and the tax bills stay in
the mod window. A dropdown gets its value before it listens: drawing the
page writes nothing. The cycling world map time button and the old
Sections() list are gone (the table replaces them).

Not tested in game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D391"/>
+  <dimension ref="A1:D392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7096,6 +7096,23 @@
         </is>
       </c>
     </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_more</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>その他の設定は Elin Together のウィンドウ（「ワールドのルール」タブ）にあります。</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>More options in the Elin Together window (World rules tab).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Client tab in cards: Controls, Workshop mods, Shared save folder, Help (council 2026-10-23, step 6)
The player's own options, one card each: Controls (ping key, with a line
saying what it does), Workshop mods (download, keep: greyed without
download), Shared save folder (optional) (the depot address and key, a
line saying it is not needed to play together, the GitHub help), Help
(bug report). Same keys, same dialogs; texts in EN/JA/ZH.

Not tested in game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D392"/>
+  <dimension ref="A1:D398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7113,6 +7113,108 @@
         </is>
       </c>
     </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_sec_controls</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>操作</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_sec_mods</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>ワークショップのMOD</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Workshop mods</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_sec_depot</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>共有のセーブフォルダ（任意）</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Shared save folder (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_sec_help</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>ヘルプ</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_desc_ping</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>このキーを押すと、マップ上の場所を他のプレイヤーに知らせます。</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Press this key to show a spot on the map to the other players.</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_desc_depot</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>ワールドを置いておく場所で、誰でもホストになれます。一緒に遊ぶだけなら必要ありません。</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Where the world is kept so that any of you can host it. Not needed to play together.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Session tab: "This world's rules" for friends, read only, with a line when the host changes one (council 2026-10-23, step 7)
A player in someone else's game sees, in the Session tab, the visible
rows of the host's World rules with their value, as the host last sent
them: the rules a guest already receives (NetSessionRules), no new
message and no delta. Rows a guest is not told (the joining rows, the
fallbacks not in the rules message) are left out; "every player gets
their own" is read from the six of twelve it is told. Not editable.
The first rules of a session are the snapshot of the join; after that a
changed row is told in one line ("The host changed X: A -> B"), kept on
the card, and the page is drawn again.

Not tested in game (needs two instances: card content, the notice, that
nothing is editable). Release build not checked here (NuGet audit error
NU1902 on MessagePack, unrelated).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D398"/>
+  <dimension ref="A1:D405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7215,6 +7215,125 @@
         </is>
       </c>
     </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_title</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>このワールドのルール</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>This world's rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_note</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>ホストが決めたルールです。変更は全員に同時に適用されます。</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Set by the host. A change applies to everyone at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_line</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>{0}：{1}</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>{0}: {1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_changed</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>ホストが「{0}」を変更しました：{1} → {2}</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>The host changed "{0}": {1} -&gt; {2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_yes</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>はい</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_no</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>いいえ</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_custom</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>カスタム</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Custom</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Global chat: player chat reaches every player wherever they are, behind a host box (default on)
Player chat lines (OnEnterChat) now carry Chat + ChatId; the host relays them to every connected peer, away
or not, and a host line goes to all peers instead of the players of its map. A guest holding its own map
forwards zone chat up to the host. A chat id is shown once. GlobalChat off: map-local as before.
NPC and game lines are untouched. Texts EN/JA/CN. Compiled (DebugNightly), not run in game.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D414"/>
+  <dimension ref="A1:D416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7487,6 +7487,40 @@
         </is>
       </c>
     </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_global_chat</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>全員にチャットを届ける</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Chat is read by every player</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_global_chat</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>プレイヤーが入力したチャットは、別のマップ、ワールドマップ、単独行動中など、どこにいる全員にも届きます。オフ：同じマップのプレイヤーにだけ届きます。住民やゲームのセリフは常にそのマップだけです</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>What a player types in the chat is read by every player, wherever they are: on another map, on the world map, away on their own. Off: only the players on the same map as the speaker read it. Lines of townspeople and the game stay on their map either way</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Follow: walk after another player's character on the same map
New menu entry "Follow" on another player's character (host option
Server.Follow, default on, NetSessionRules key 96). The local character
walks after it with the game's own click-to-move (AI_Goto), on the same
map only, nothing new on the wire. Any key or click, a blow, a hostile
in sight, an open window, the leader leaving the map, dead, out of
sight or unreachable stop it, with a line in the log.

Tested (follow_suite, host + 1 guest, both directions): menu offers it,
the follower closes in after an 8-step walk and both games agree on its
tile, a blow stops it, the leader moving to Vernis stops it and the
follower stays home, box unticked hides the entry. 21/21, 0 exceptions.
Not tested: a real key press stopping it (minimized windows).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D416"/>
+  <dimension ref="A1:D424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7521,6 +7521,142 @@
         </is>
       </c>
     </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>emp_act_follow</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>ついていく</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Follow</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>emp_follow_start</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>#1についていく。何かキーを押すと止まる。</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>You follow #1. Press any key to stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>emp_follow_stop</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>#1についていくのをやめた。</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>You stop following #1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>emp_follow_left</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>#1はこのマップを離れた。ついていくのをやめた。</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>#1 left the map. You stop following.</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>emp_follow_lost</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>#1を見失った。</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>You lost sight of #1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>emp_follow_danger</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>危険だ。ついていくのをやめた。</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Danger! You stop following.</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_follow</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>ほかのプレイヤーについていける</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Players can follow each other</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_follow</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>ほかのプレイヤーをクリックして「ついていく」を選ぶと、同じマップの中で自動で後を歩きます。キー、攻撃、敵、相手のマップ移動で止まります。</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Click another player and choose Follow: your character walks after it on the same map. A key, a blow, a monster in sight or the other player leaving the map stops it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>